<commit_message>
chore: actualiza dashboard 2026-05-19T11:43Z
</commit_message>
<xml_diff>
--- a/INFORME EXCESOS DE VELOCIDAD.xlsx
+++ b/INFORME EXCESOS DE VELOCIDAD.xlsx
@@ -5929,6 +5929,30 @@
   </x:si>
   <x:si>
     <x:t>-33.699782,-70.802484</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026/05/18 20:35:29</x:t>
+  </x:si>
+  <x:si>
+    <x:t>-33.699632,-70.802315</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026/05/18 20:35:37</x:t>
+  </x:si>
+  <x:si>
+    <x:t>-33.699382,-70.801901</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026/05/18 20:39:19</x:t>
+  </x:si>
+  <x:si>
+    <x:t>-33.699588,-70.802288</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026/05/18 20:39:25</x:t>
+  </x:si>
+  <x:si>
+    <x:t>-33.699859,-70.802454</x:t>
   </x:si>
   <x:si>
     <x:t>Fecha</x:t>
@@ -6114,8 +6138,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="SpeedingByUnitsFleetsDetailTable_1" displayName="SpeedingByUnitsFleetsDetailTable_1" ref="A5:O489" totalsRowShown="0">
-  <x:autoFilter ref="A5:O489"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="SpeedingByUnitsFleetsDetailTable_1" displayName="SpeedingByUnitsFleetsDetailTable_1" ref="A5:O491" totalsRowShown="0">
+  <x:autoFilter ref="A5:O491"/>
   <x:tableColumns count="15">
     <x:tableColumn id="1" name="Alias"/>
     <x:tableColumn id="2" name="Conductor"/>
@@ -6138,8 +6162,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SpeedingByUnitsFleetsDataTable_1" displayName="SpeedingByUnitsFleetsDataTable_1" ref="A5:H975" totalsRowShown="0">
-  <x:autoFilter ref="A5:H975"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SpeedingByUnitsFleetsDataTable_1" displayName="SpeedingByUnitsFleetsDataTable_1" ref="A5:H979" totalsRowShown="0">
+  <x:autoFilter ref="A5:H979"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="Alias"/>
     <x:tableColumn id="2" name="Secuencial" dataDxfId="0"/>
@@ -6580,22 +6604,22 @@
         <x:v>14</x:v>
       </x:c>
       <x:c r="B8" s="4">
-        <x:v>259</x:v>
+        <x:v>261</x:v>
       </x:c>
       <x:c r="C8" s="5">
-        <x:v>0.0247569444444444</x:v>
+        <x:v>0.0249189814814815</x:v>
       </x:c>
       <x:c r="D8" s="5">
-        <x:v>9.55866585648148E-05</x:v>
+        <x:v>9.54750243055556E-05</x:v>
       </x:c>
       <x:c r="E8" s="4">
-        <x:v>17.9</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="F8" s="4">
         <x:v>47.4</x:v>
       </x:c>
       <x:c r="G8" s="4">
-        <x:v>25.5</x:v>
+        <x:v>25.4</x:v>
       </x:c>
       <x:c r="H8" s="4">
         <x:v>0</x:v>
@@ -6625,7 +6649,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:O489"/>
+  <x:dimension ref="A1:O491"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="30.710625" style="0" customWidth="1"/>
@@ -29486,6 +29510,100 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="O489" s="4">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="490" spans="1:15">
+      <x:c r="A490" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="B490" s="0" t="s">
+        <x:v>1934</x:v>
+      </x:c>
+      <x:c r="C490" s="4">
+        <x:v>495</x:v>
+      </x:c>
+      <x:c r="D490" s="4" t="s">
+        <x:v>1971</x:v>
+      </x:c>
+      <x:c r="E490" s="6" t="s">
+        <x:v>1972</x:v>
+      </x:c>
+      <x:c r="F490" s="4" t="s">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="G490" s="4" t="s">
+        <x:v>1973</x:v>
+      </x:c>
+      <x:c r="H490" s="6" t="s">
+        <x:v>1974</x:v>
+      </x:c>
+      <x:c r="I490" s="4" t="s">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="J490" s="5">
+        <x:v>9.25925925925926E-05</x:v>
+      </x:c>
+      <x:c r="K490" s="4" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="L490" s="4">
+        <x:v>23.1</x:v>
+      </x:c>
+      <x:c r="M490" s="4">
+        <x:v>20.1</x:v>
+      </x:c>
+      <x:c r="N490" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O490" s="4">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="491" spans="1:15">
+      <x:c r="A491" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="B491" s="0" t="s">
+        <x:v>1934</x:v>
+      </x:c>
+      <x:c r="C491" s="4">
+        <x:v>498</x:v>
+      </x:c>
+      <x:c r="D491" s="4" t="s">
+        <x:v>1975</x:v>
+      </x:c>
+      <x:c r="E491" s="6" t="s">
+        <x:v>1976</x:v>
+      </x:c>
+      <x:c r="F491" s="4" t="s">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="G491" s="4" t="s">
+        <x:v>1977</x:v>
+      </x:c>
+      <x:c r="H491" s="6" t="s">
+        <x:v>1978</x:v>
+      </x:c>
+      <x:c r="I491" s="4" t="s">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="J491" s="5">
+        <x:v>6.94444444444444E-05</x:v>
+      </x:c>
+      <x:c r="K491" s="4">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="L491" s="4">
+        <x:v>24.4</x:v>
+      </x:c>
+      <x:c r="M491" s="4">
+        <x:v>21.9</x:v>
+      </x:c>
+      <x:c r="N491" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O491" s="4">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -30464,6 +30582,10 @@
     <x:hyperlink ref="H488" r:id="rId974"/>
     <x:hyperlink ref="E489" r:id="rId975"/>
     <x:hyperlink ref="H489" r:id="rId976"/>
+    <x:hyperlink ref="E490" r:id="rId977"/>
+    <x:hyperlink ref="H490" r:id="rId978"/>
+    <x:hyperlink ref="E491" r:id="rId979"/>
+    <x:hyperlink ref="H491" r:id="rId980"/>
   </x:hyperlinks>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
@@ -30480,7 +30602,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:H975"/>
+  <x:dimension ref="A1:H979"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="30.710625" style="0" customWidth="1"/>
@@ -30533,22 +30655,22 @@
         <x:v>16</x:v>
       </x:c>
       <x:c r="C5" s="3" t="s">
-        <x:v>1971</x:v>
+        <x:v>1979</x:v>
       </x:c>
       <x:c r="D5" s="3" t="s">
-        <x:v>1972</x:v>
+        <x:v>1980</x:v>
       </x:c>
       <x:c r="E5" s="3" t="s">
-        <x:v>1973</x:v>
+        <x:v>1981</x:v>
       </x:c>
       <x:c r="F5" s="3" t="s">
-        <x:v>1974</x:v>
+        <x:v>1982</x:v>
       </x:c>
       <x:c r="G5" s="3" t="s">
-        <x:v>1975</x:v>
+        <x:v>1983</x:v>
       </x:c>
       <x:c r="H5" s="3" t="s">
-        <x:v>1976</x:v>
+        <x:v>1984</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:8">
@@ -43071,7 +43193,7 @@
         <x:v>997</x:v>
       </x:c>
       <x:c r="E487" s="4" t="s">
-        <x:v>1977</x:v>
+        <x:v>1985</x:v>
       </x:c>
       <x:c r="F487" s="4">
         <x:v>25.8</x:v>
@@ -54531,10 +54653,10 @@
         <x:v>459</x:v>
       </x:c>
       <x:c r="C928" s="4" t="s">
-        <x:v>1978</x:v>
+        <x:v>1986</x:v>
       </x:c>
       <x:c r="D928" s="6" t="s">
-        <x:v>1979</x:v>
+        <x:v>1987</x:v>
       </x:c>
       <x:c r="E928" s="4" t="s">
         <x:v>36</x:v>
@@ -55769,6 +55891,110 @@
       </x:c>
       <x:c r="H975" s="4">
         <x:v>546.7</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="976" spans="1:8">
+      <x:c r="A976" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="B976" s="4">
+        <x:v>495</x:v>
+      </x:c>
+      <x:c r="C976" s="4" t="s">
+        <x:v>1971</x:v>
+      </x:c>
+      <x:c r="D976" s="6" t="s">
+        <x:v>1972</x:v>
+      </x:c>
+      <x:c r="E976" s="4" t="s">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="F976" s="4">
+        <x:v>23.1</x:v>
+      </x:c>
+      <x:c r="G976" s="4">
+        <x:v>4626.3</x:v>
+      </x:c>
+      <x:c r="H976" s="4">
+        <x:v>543.8</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="977" spans="1:8">
+      <x:c r="A977" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="B977" s="4">
+        <x:v>495</x:v>
+      </x:c>
+      <x:c r="C977" s="4" t="s">
+        <x:v>1973</x:v>
+      </x:c>
+      <x:c r="D977" s="6" t="s">
+        <x:v>1974</x:v>
+      </x:c>
+      <x:c r="E977" s="4" t="s">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="F977" s="4">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="G977" s="4">
+        <x:v>4626.3</x:v>
+      </x:c>
+      <x:c r="H977" s="4">
+        <x:v>541.7</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="978" spans="1:8">
+      <x:c r="A978" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="B978" s="4">
+        <x:v>498</x:v>
+      </x:c>
+      <x:c r="C978" s="4" t="s">
+        <x:v>1975</x:v>
+      </x:c>
+      <x:c r="D978" s="6" t="s">
+        <x:v>1976</x:v>
+      </x:c>
+      <x:c r="E978" s="4" t="s">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="F978" s="4">
+        <x:v>24.4</x:v>
+      </x:c>
+      <x:c r="G978" s="4">
+        <x:v>4626.8</x:v>
+      </x:c>
+      <x:c r="H978" s="4">
+        <x:v>544.4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="979" spans="1:8">
+      <x:c r="A979" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="B979" s="4">
+        <x:v>498</x:v>
+      </x:c>
+      <x:c r="C979" s="4" t="s">
+        <x:v>1977</x:v>
+      </x:c>
+      <x:c r="D979" s="6" t="s">
+        <x:v>1978</x:v>
+      </x:c>
+      <x:c r="E979" s="4" t="s">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="F979" s="4">
+        <x:v>19.4</x:v>
+      </x:c>
+      <x:c r="G979" s="4">
+        <x:v>4626.9</x:v>
+      </x:c>
+      <x:c r="H979" s="4">
+        <x:v>546.8</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -55778,983 +56004,987 @@
     <x:mergeCell ref="A3:H3"/>
   </x:mergeCells>
   <x:hyperlinks>
-    <x:hyperlink ref="D6" r:id="rId978"/>
-    <x:hyperlink ref="D7" r:id="rId979"/>
-    <x:hyperlink ref="D8" r:id="rId980"/>
-    <x:hyperlink ref="D9" r:id="rId981"/>
-    <x:hyperlink ref="D10" r:id="rId982"/>
-    <x:hyperlink ref="D11" r:id="rId983"/>
-    <x:hyperlink ref="D12" r:id="rId984"/>
-    <x:hyperlink ref="D13" r:id="rId985"/>
-    <x:hyperlink ref="D14" r:id="rId986"/>
-    <x:hyperlink ref="D15" r:id="rId987"/>
-    <x:hyperlink ref="D16" r:id="rId988"/>
-    <x:hyperlink ref="D17" r:id="rId989"/>
-    <x:hyperlink ref="D18" r:id="rId990"/>
-    <x:hyperlink ref="D19" r:id="rId991"/>
-    <x:hyperlink ref="D20" r:id="rId992"/>
-    <x:hyperlink ref="D21" r:id="rId993"/>
-    <x:hyperlink ref="D22" r:id="rId994"/>
-    <x:hyperlink ref="D23" r:id="rId995"/>
-    <x:hyperlink ref="D24" r:id="rId996"/>
-    <x:hyperlink ref="D25" r:id="rId997"/>
-    <x:hyperlink ref="D26" r:id="rId998"/>
-    <x:hyperlink ref="D27" r:id="rId999"/>
-    <x:hyperlink ref="D28" r:id="rId1000"/>
-    <x:hyperlink ref="D29" r:id="rId1001"/>
-    <x:hyperlink ref="D30" r:id="rId1002"/>
-    <x:hyperlink ref="D31" r:id="rId1003"/>
-    <x:hyperlink ref="D32" r:id="rId1004"/>
-    <x:hyperlink ref="D33" r:id="rId1005"/>
-    <x:hyperlink ref="D34" r:id="rId1006"/>
-    <x:hyperlink ref="D35" r:id="rId1007"/>
-    <x:hyperlink ref="D36" r:id="rId1008"/>
-    <x:hyperlink ref="D37" r:id="rId1009"/>
-    <x:hyperlink ref="D38" r:id="rId1010"/>
-    <x:hyperlink ref="D39" r:id="rId1011"/>
-    <x:hyperlink ref="D40" r:id="rId1012"/>
-    <x:hyperlink ref="D41" r:id="rId1013"/>
-    <x:hyperlink ref="D42" r:id="rId1014"/>
-    <x:hyperlink ref="D43" r:id="rId1015"/>
-    <x:hyperlink ref="D44" r:id="rId1016"/>
-    <x:hyperlink ref="D45" r:id="rId1017"/>
-    <x:hyperlink ref="D46" r:id="rId1018"/>
-    <x:hyperlink ref="D47" r:id="rId1019"/>
-    <x:hyperlink ref="D48" r:id="rId1020"/>
-    <x:hyperlink ref="D49" r:id="rId1021"/>
-    <x:hyperlink ref="D50" r:id="rId1022"/>
-    <x:hyperlink ref="D51" r:id="rId1023"/>
-    <x:hyperlink ref="D52" r:id="rId1024"/>
-    <x:hyperlink ref="D53" r:id="rId1025"/>
-    <x:hyperlink ref="D54" r:id="rId1026"/>
-    <x:hyperlink ref="D55" r:id="rId1027"/>
-    <x:hyperlink ref="D56" r:id="rId1028"/>
-    <x:hyperlink ref="D57" r:id="rId1029"/>
-    <x:hyperlink ref="D58" r:id="rId1030"/>
-    <x:hyperlink ref="D59" r:id="rId1031"/>
-    <x:hyperlink ref="D60" r:id="rId1032"/>
-    <x:hyperlink ref="D61" r:id="rId1033"/>
-    <x:hyperlink ref="D62" r:id="rId1034"/>
-    <x:hyperlink ref="D63" r:id="rId1035"/>
-    <x:hyperlink ref="D64" r:id="rId1036"/>
-    <x:hyperlink ref="D65" r:id="rId1037"/>
-    <x:hyperlink ref="D66" r:id="rId1038"/>
-    <x:hyperlink ref="D67" r:id="rId1039"/>
-    <x:hyperlink ref="D68" r:id="rId1040"/>
-    <x:hyperlink ref="D69" r:id="rId1041"/>
-    <x:hyperlink ref="D70" r:id="rId1042"/>
-    <x:hyperlink ref="D71" r:id="rId1043"/>
-    <x:hyperlink ref="D72" r:id="rId1044"/>
-    <x:hyperlink ref="D73" r:id="rId1045"/>
-    <x:hyperlink ref="D74" r:id="rId1046"/>
-    <x:hyperlink ref="D75" r:id="rId1047"/>
-    <x:hyperlink ref="D76" r:id="rId1048"/>
-    <x:hyperlink ref="D77" r:id="rId1049"/>
-    <x:hyperlink ref="D78" r:id="rId1050"/>
-    <x:hyperlink ref="D79" r:id="rId1051"/>
-    <x:hyperlink ref="D80" r:id="rId1052"/>
-    <x:hyperlink ref="D81" r:id="rId1053"/>
-    <x:hyperlink ref="D82" r:id="rId1054"/>
-    <x:hyperlink ref="D83" r:id="rId1055"/>
-    <x:hyperlink ref="D84" r:id="rId1056"/>
-    <x:hyperlink ref="D85" r:id="rId1057"/>
-    <x:hyperlink ref="D86" r:id="rId1058"/>
-    <x:hyperlink ref="D87" r:id="rId1059"/>
-    <x:hyperlink ref="D88" r:id="rId1060"/>
-    <x:hyperlink ref="D89" r:id="rId1061"/>
-    <x:hyperlink ref="D90" r:id="rId1062"/>
-    <x:hyperlink ref="D91" r:id="rId1063"/>
-    <x:hyperlink ref="D92" r:id="rId1064"/>
-    <x:hyperlink ref="D93" r:id="rId1065"/>
-    <x:hyperlink ref="D94" r:id="rId1066"/>
-    <x:hyperlink ref="D95" r:id="rId1067"/>
-    <x:hyperlink ref="D96" r:id="rId1068"/>
-    <x:hyperlink ref="D97" r:id="rId1069"/>
-    <x:hyperlink ref="D98" r:id="rId1070"/>
-    <x:hyperlink ref="D99" r:id="rId1071"/>
-    <x:hyperlink ref="D100" r:id="rId1072"/>
-    <x:hyperlink ref="D101" r:id="rId1073"/>
-    <x:hyperlink ref="D102" r:id="rId1074"/>
-    <x:hyperlink ref="D103" r:id="rId1075"/>
-    <x:hyperlink ref="D104" r:id="rId1076"/>
-    <x:hyperlink ref="D105" r:id="rId1077"/>
-    <x:hyperlink ref="D106" r:id="rId1078"/>
-    <x:hyperlink ref="D107" r:id="rId1079"/>
-    <x:hyperlink ref="D108" r:id="rId1080"/>
-    <x:hyperlink ref="D109" r:id="rId1081"/>
-    <x:hyperlink ref="D110" r:id="rId1082"/>
-    <x:hyperlink ref="D111" r:id="rId1083"/>
-    <x:hyperlink ref="D112" r:id="rId1084"/>
-    <x:hyperlink ref="D113" r:id="rId1085"/>
-    <x:hyperlink ref="D114" r:id="rId1086"/>
-    <x:hyperlink ref="D115" r:id="rId1087"/>
-    <x:hyperlink ref="D116" r:id="rId1088"/>
-    <x:hyperlink ref="D117" r:id="rId1089"/>
-    <x:hyperlink ref="D118" r:id="rId1090"/>
-    <x:hyperlink ref="D119" r:id="rId1091"/>
-    <x:hyperlink ref="D120" r:id="rId1092"/>
-    <x:hyperlink ref="D121" r:id="rId1093"/>
-    <x:hyperlink ref="D122" r:id="rId1094"/>
-    <x:hyperlink ref="D123" r:id="rId1095"/>
-    <x:hyperlink ref="D124" r:id="rId1096"/>
-    <x:hyperlink ref="D125" r:id="rId1097"/>
-    <x:hyperlink ref="D126" r:id="rId1098"/>
-    <x:hyperlink ref="D127" r:id="rId1099"/>
-    <x:hyperlink ref="D128" r:id="rId1100"/>
-    <x:hyperlink ref="D129" r:id="rId1101"/>
-    <x:hyperlink ref="D130" r:id="rId1102"/>
-    <x:hyperlink ref="D131" r:id="rId1103"/>
-    <x:hyperlink ref="D132" r:id="rId1104"/>
-    <x:hyperlink ref="D133" r:id="rId1105"/>
-    <x:hyperlink ref="D134" r:id="rId1106"/>
-    <x:hyperlink ref="D135" r:id="rId1107"/>
-    <x:hyperlink ref="D136" r:id="rId1108"/>
-    <x:hyperlink ref="D137" r:id="rId1109"/>
-    <x:hyperlink ref="D138" r:id="rId1110"/>
-    <x:hyperlink ref="D139" r:id="rId1111"/>
-    <x:hyperlink ref="D140" r:id="rId1112"/>
-    <x:hyperlink ref="D141" r:id="rId1113"/>
-    <x:hyperlink ref="D142" r:id="rId1114"/>
-    <x:hyperlink ref="D143" r:id="rId1115"/>
-    <x:hyperlink ref="D144" r:id="rId1116"/>
-    <x:hyperlink ref="D145" r:id="rId1117"/>
-    <x:hyperlink ref="D146" r:id="rId1118"/>
-    <x:hyperlink ref="D147" r:id="rId1119"/>
-    <x:hyperlink ref="D148" r:id="rId1120"/>
-    <x:hyperlink ref="D149" r:id="rId1121"/>
-    <x:hyperlink ref="D150" r:id="rId1122"/>
-    <x:hyperlink ref="D151" r:id="rId1123"/>
-    <x:hyperlink ref="D152" r:id="rId1124"/>
-    <x:hyperlink ref="D153" r:id="rId1125"/>
-    <x:hyperlink ref="D154" r:id="rId1126"/>
-    <x:hyperlink ref="D155" r:id="rId1127"/>
-    <x:hyperlink ref="D156" r:id="rId1128"/>
-    <x:hyperlink ref="D157" r:id="rId1129"/>
-    <x:hyperlink ref="D158" r:id="rId1130"/>
-    <x:hyperlink ref="D159" r:id="rId1131"/>
-    <x:hyperlink ref="D160" r:id="rId1132"/>
-    <x:hyperlink ref="D161" r:id="rId1133"/>
-    <x:hyperlink ref="D162" r:id="rId1134"/>
-    <x:hyperlink ref="D163" r:id="rId1135"/>
-    <x:hyperlink ref="D164" r:id="rId1136"/>
-    <x:hyperlink ref="D165" r:id="rId1137"/>
-    <x:hyperlink ref="D166" r:id="rId1138"/>
-    <x:hyperlink ref="D167" r:id="rId1139"/>
-    <x:hyperlink ref="D168" r:id="rId1140"/>
-    <x:hyperlink ref="D169" r:id="rId1141"/>
-    <x:hyperlink ref="D170" r:id="rId1142"/>
-    <x:hyperlink ref="D171" r:id="rId1143"/>
-    <x:hyperlink ref="D172" r:id="rId1144"/>
-    <x:hyperlink ref="D173" r:id="rId1145"/>
-    <x:hyperlink ref="D174" r:id="rId1146"/>
-    <x:hyperlink ref="D175" r:id="rId1147"/>
-    <x:hyperlink ref="D176" r:id="rId1148"/>
-    <x:hyperlink ref="D177" r:id="rId1149"/>
-    <x:hyperlink ref="D178" r:id="rId1150"/>
-    <x:hyperlink ref="D179" r:id="rId1151"/>
-    <x:hyperlink ref="D180" r:id="rId1152"/>
-    <x:hyperlink ref="D181" r:id="rId1153"/>
-    <x:hyperlink ref="D182" r:id="rId1154"/>
-    <x:hyperlink ref="D183" r:id="rId1155"/>
-    <x:hyperlink ref="D184" r:id="rId1156"/>
-    <x:hyperlink ref="D185" r:id="rId1157"/>
-    <x:hyperlink ref="D186" r:id="rId1158"/>
-    <x:hyperlink ref="D187" r:id="rId1159"/>
-    <x:hyperlink ref="D188" r:id="rId1160"/>
-    <x:hyperlink ref="D189" r:id="rId1161"/>
-    <x:hyperlink ref="D190" r:id="rId1162"/>
-    <x:hyperlink ref="D191" r:id="rId1163"/>
-    <x:hyperlink ref="D192" r:id="rId1164"/>
-    <x:hyperlink ref="D193" r:id="rId1165"/>
-    <x:hyperlink ref="D194" r:id="rId1166"/>
-    <x:hyperlink ref="D195" r:id="rId1167"/>
-    <x:hyperlink ref="D196" r:id="rId1168"/>
-    <x:hyperlink ref="D197" r:id="rId1169"/>
-    <x:hyperlink ref="D198" r:id="rId1170"/>
-    <x:hyperlink ref="D199" r:id="rId1171"/>
-    <x:hyperlink ref="D200" r:id="rId1172"/>
-    <x:hyperlink ref="D201" r:id="rId1173"/>
-    <x:hyperlink ref="D202" r:id="rId1174"/>
-    <x:hyperlink ref="D203" r:id="rId1175"/>
-    <x:hyperlink ref="D204" r:id="rId1176"/>
-    <x:hyperlink ref="D205" r:id="rId1177"/>
-    <x:hyperlink ref="D206" r:id="rId1178"/>
-    <x:hyperlink ref="D207" r:id="rId1179"/>
-    <x:hyperlink ref="D208" r:id="rId1180"/>
-    <x:hyperlink ref="D209" r:id="rId1181"/>
-    <x:hyperlink ref="D210" r:id="rId1182"/>
-    <x:hyperlink ref="D211" r:id="rId1183"/>
-    <x:hyperlink ref="D212" r:id="rId1184"/>
-    <x:hyperlink ref="D213" r:id="rId1185"/>
-    <x:hyperlink ref="D214" r:id="rId1186"/>
-    <x:hyperlink ref="D215" r:id="rId1187"/>
-    <x:hyperlink ref="D216" r:id="rId1188"/>
-    <x:hyperlink ref="D217" r:id="rId1189"/>
-    <x:hyperlink ref="D218" r:id="rId1190"/>
-    <x:hyperlink ref="D219" r:id="rId1191"/>
-    <x:hyperlink ref="D220" r:id="rId1192"/>
-    <x:hyperlink ref="D221" r:id="rId1193"/>
-    <x:hyperlink ref="D222" r:id="rId1194"/>
-    <x:hyperlink ref="D223" r:id="rId1195"/>
-    <x:hyperlink ref="D224" r:id="rId1196"/>
-    <x:hyperlink ref="D225" r:id="rId1197"/>
-    <x:hyperlink ref="D226" r:id="rId1198"/>
-    <x:hyperlink ref="D227" r:id="rId1199"/>
-    <x:hyperlink ref="D228" r:id="rId1200"/>
-    <x:hyperlink ref="D229" r:id="rId1201"/>
-    <x:hyperlink ref="D230" r:id="rId1202"/>
-    <x:hyperlink ref="D231" r:id="rId1203"/>
-    <x:hyperlink ref="D232" r:id="rId1204"/>
-    <x:hyperlink ref="D233" r:id="rId1205"/>
-    <x:hyperlink ref="D234" r:id="rId1206"/>
-    <x:hyperlink ref="D235" r:id="rId1207"/>
-    <x:hyperlink ref="D236" r:id="rId1208"/>
-    <x:hyperlink ref="D237" r:id="rId1209"/>
-    <x:hyperlink ref="D238" r:id="rId1210"/>
-    <x:hyperlink ref="D239" r:id="rId1211"/>
-    <x:hyperlink ref="D240" r:id="rId1212"/>
-    <x:hyperlink ref="D241" r:id="rId1213"/>
-    <x:hyperlink ref="D242" r:id="rId1214"/>
-    <x:hyperlink ref="D243" r:id="rId1215"/>
-    <x:hyperlink ref="D244" r:id="rId1216"/>
-    <x:hyperlink ref="D245" r:id="rId1217"/>
-    <x:hyperlink ref="D246" r:id="rId1218"/>
-    <x:hyperlink ref="D247" r:id="rId1219"/>
-    <x:hyperlink ref="D248" r:id="rId1220"/>
-    <x:hyperlink ref="D249" r:id="rId1221"/>
-    <x:hyperlink ref="D250" r:id="rId1222"/>
-    <x:hyperlink ref="D251" r:id="rId1223"/>
-    <x:hyperlink ref="D252" r:id="rId1224"/>
-    <x:hyperlink ref="D253" r:id="rId1225"/>
-    <x:hyperlink ref="D254" r:id="rId1226"/>
-    <x:hyperlink ref="D255" r:id="rId1227"/>
-    <x:hyperlink ref="D256" r:id="rId1228"/>
-    <x:hyperlink ref="D257" r:id="rId1229"/>
-    <x:hyperlink ref="D258" r:id="rId1230"/>
-    <x:hyperlink ref="D259" r:id="rId1231"/>
-    <x:hyperlink ref="D260" r:id="rId1232"/>
-    <x:hyperlink ref="D261" r:id="rId1233"/>
-    <x:hyperlink ref="D262" r:id="rId1234"/>
-    <x:hyperlink ref="D263" r:id="rId1235"/>
-    <x:hyperlink ref="D264" r:id="rId1236"/>
-    <x:hyperlink ref="D265" r:id="rId1237"/>
-    <x:hyperlink ref="D266" r:id="rId1238"/>
-    <x:hyperlink ref="D267" r:id="rId1239"/>
-    <x:hyperlink ref="D268" r:id="rId1240"/>
-    <x:hyperlink ref="D269" r:id="rId1241"/>
-    <x:hyperlink ref="D270" r:id="rId1242"/>
-    <x:hyperlink ref="D271" r:id="rId1243"/>
-    <x:hyperlink ref="D272" r:id="rId1244"/>
-    <x:hyperlink ref="D273" r:id="rId1245"/>
-    <x:hyperlink ref="D274" r:id="rId1246"/>
-    <x:hyperlink ref="D275" r:id="rId1247"/>
-    <x:hyperlink ref="D276" r:id="rId1248"/>
-    <x:hyperlink ref="D277" r:id="rId1249"/>
-    <x:hyperlink ref="D278" r:id="rId1250"/>
-    <x:hyperlink ref="D279" r:id="rId1251"/>
-    <x:hyperlink ref="D280" r:id="rId1252"/>
-    <x:hyperlink ref="D281" r:id="rId1253"/>
-    <x:hyperlink ref="D282" r:id="rId1254"/>
-    <x:hyperlink ref="D283" r:id="rId1255"/>
-    <x:hyperlink ref="D284" r:id="rId1256"/>
-    <x:hyperlink ref="D285" r:id="rId1257"/>
-    <x:hyperlink ref="D286" r:id="rId1258"/>
-    <x:hyperlink ref="D287" r:id="rId1259"/>
-    <x:hyperlink ref="D288" r:id="rId1260"/>
-    <x:hyperlink ref="D289" r:id="rId1261"/>
-    <x:hyperlink ref="D290" r:id="rId1262"/>
-    <x:hyperlink ref="D291" r:id="rId1263"/>
-    <x:hyperlink ref="D292" r:id="rId1264"/>
-    <x:hyperlink ref="D293" r:id="rId1265"/>
-    <x:hyperlink ref="D294" r:id="rId1266"/>
-    <x:hyperlink ref="D295" r:id="rId1267"/>
-    <x:hyperlink ref="D296" r:id="rId1268"/>
-    <x:hyperlink ref="D297" r:id="rId1269"/>
-    <x:hyperlink ref="D298" r:id="rId1270"/>
-    <x:hyperlink ref="D299" r:id="rId1271"/>
-    <x:hyperlink ref="D300" r:id="rId1272"/>
-    <x:hyperlink ref="D301" r:id="rId1273"/>
-    <x:hyperlink ref="D302" r:id="rId1274"/>
-    <x:hyperlink ref="D303" r:id="rId1275"/>
-    <x:hyperlink ref="D304" r:id="rId1276"/>
-    <x:hyperlink ref="D305" r:id="rId1277"/>
-    <x:hyperlink ref="D306" r:id="rId1278"/>
-    <x:hyperlink ref="D307" r:id="rId1279"/>
-    <x:hyperlink ref="D308" r:id="rId1280"/>
-    <x:hyperlink ref="D309" r:id="rId1281"/>
-    <x:hyperlink ref="D310" r:id="rId1282"/>
-    <x:hyperlink ref="D311" r:id="rId1283"/>
-    <x:hyperlink ref="D312" r:id="rId1284"/>
-    <x:hyperlink ref="D313" r:id="rId1285"/>
-    <x:hyperlink ref="D314" r:id="rId1286"/>
-    <x:hyperlink ref="D315" r:id="rId1287"/>
-    <x:hyperlink ref="D316" r:id="rId1288"/>
-    <x:hyperlink ref="D317" r:id="rId1289"/>
-    <x:hyperlink ref="D318" r:id="rId1290"/>
-    <x:hyperlink ref="D319" r:id="rId1291"/>
-    <x:hyperlink ref="D320" r:id="rId1292"/>
-    <x:hyperlink ref="D321" r:id="rId1293"/>
-    <x:hyperlink ref="D322" r:id="rId1294"/>
-    <x:hyperlink ref="D323" r:id="rId1295"/>
-    <x:hyperlink ref="D324" r:id="rId1296"/>
-    <x:hyperlink ref="D325" r:id="rId1297"/>
-    <x:hyperlink ref="D326" r:id="rId1298"/>
-    <x:hyperlink ref="D327" r:id="rId1299"/>
-    <x:hyperlink ref="D328" r:id="rId1300"/>
-    <x:hyperlink ref="D329" r:id="rId1301"/>
-    <x:hyperlink ref="D330" r:id="rId1302"/>
-    <x:hyperlink ref="D331" r:id="rId1303"/>
-    <x:hyperlink ref="D332" r:id="rId1304"/>
-    <x:hyperlink ref="D333" r:id="rId1305"/>
-    <x:hyperlink ref="D334" r:id="rId1306"/>
-    <x:hyperlink ref="D335" r:id="rId1307"/>
-    <x:hyperlink ref="D336" r:id="rId1308"/>
-    <x:hyperlink ref="D337" r:id="rId1309"/>
-    <x:hyperlink ref="D338" r:id="rId1310"/>
-    <x:hyperlink ref="D339" r:id="rId1311"/>
-    <x:hyperlink ref="D340" r:id="rId1312"/>
-    <x:hyperlink ref="D341" r:id="rId1313"/>
-    <x:hyperlink ref="D342" r:id="rId1314"/>
-    <x:hyperlink ref="D343" r:id="rId1315"/>
-    <x:hyperlink ref="D344" r:id="rId1316"/>
-    <x:hyperlink ref="D345" r:id="rId1317"/>
-    <x:hyperlink ref="D346" r:id="rId1318"/>
-    <x:hyperlink ref="D347" r:id="rId1319"/>
-    <x:hyperlink ref="D348" r:id="rId1320"/>
-    <x:hyperlink ref="D349" r:id="rId1321"/>
-    <x:hyperlink ref="D350" r:id="rId1322"/>
-    <x:hyperlink ref="D351" r:id="rId1323"/>
-    <x:hyperlink ref="D352" r:id="rId1324"/>
-    <x:hyperlink ref="D353" r:id="rId1325"/>
-    <x:hyperlink ref="D354" r:id="rId1326"/>
-    <x:hyperlink ref="D355" r:id="rId1327"/>
-    <x:hyperlink ref="D356" r:id="rId1328"/>
-    <x:hyperlink ref="D357" r:id="rId1329"/>
-    <x:hyperlink ref="D358" r:id="rId1330"/>
-    <x:hyperlink ref="D359" r:id="rId1331"/>
-    <x:hyperlink ref="D360" r:id="rId1332"/>
-    <x:hyperlink ref="D361" r:id="rId1333"/>
-    <x:hyperlink ref="D362" r:id="rId1334"/>
-    <x:hyperlink ref="D363" r:id="rId1335"/>
-    <x:hyperlink ref="D364" r:id="rId1336"/>
-    <x:hyperlink ref="D365" r:id="rId1337"/>
-    <x:hyperlink ref="D366" r:id="rId1338"/>
-    <x:hyperlink ref="D367" r:id="rId1339"/>
-    <x:hyperlink ref="D368" r:id="rId1340"/>
-    <x:hyperlink ref="D369" r:id="rId1341"/>
-    <x:hyperlink ref="D370" r:id="rId1342"/>
-    <x:hyperlink ref="D371" r:id="rId1343"/>
-    <x:hyperlink ref="D372" r:id="rId1344"/>
-    <x:hyperlink ref="D373" r:id="rId1345"/>
-    <x:hyperlink ref="D374" r:id="rId1346"/>
-    <x:hyperlink ref="D375" r:id="rId1347"/>
-    <x:hyperlink ref="D376" r:id="rId1348"/>
-    <x:hyperlink ref="D377" r:id="rId1349"/>
-    <x:hyperlink ref="D378" r:id="rId1350"/>
-    <x:hyperlink ref="D379" r:id="rId1351"/>
-    <x:hyperlink ref="D380" r:id="rId1352"/>
-    <x:hyperlink ref="D381" r:id="rId1353"/>
-    <x:hyperlink ref="D382" r:id="rId1354"/>
-    <x:hyperlink ref="D383" r:id="rId1355"/>
-    <x:hyperlink ref="D384" r:id="rId1356"/>
-    <x:hyperlink ref="D385" r:id="rId1357"/>
-    <x:hyperlink ref="D386" r:id="rId1358"/>
-    <x:hyperlink ref="D387" r:id="rId1359"/>
-    <x:hyperlink ref="D388" r:id="rId1360"/>
-    <x:hyperlink ref="D389" r:id="rId1361"/>
-    <x:hyperlink ref="D390" r:id="rId1362"/>
-    <x:hyperlink ref="D391" r:id="rId1363"/>
-    <x:hyperlink ref="D392" r:id="rId1364"/>
-    <x:hyperlink ref="D393" r:id="rId1365"/>
-    <x:hyperlink ref="D394" r:id="rId1366"/>
-    <x:hyperlink ref="D395" r:id="rId1367"/>
-    <x:hyperlink ref="D396" r:id="rId1368"/>
-    <x:hyperlink ref="D397" r:id="rId1369"/>
-    <x:hyperlink ref="D398" r:id="rId1370"/>
-    <x:hyperlink ref="D399" r:id="rId1371"/>
-    <x:hyperlink ref="D400" r:id="rId1372"/>
-    <x:hyperlink ref="D401" r:id="rId1373"/>
-    <x:hyperlink ref="D402" r:id="rId1374"/>
-    <x:hyperlink ref="D403" r:id="rId1375"/>
-    <x:hyperlink ref="D404" r:id="rId1376"/>
-    <x:hyperlink ref="D405" r:id="rId1377"/>
-    <x:hyperlink ref="D406" r:id="rId1378"/>
-    <x:hyperlink ref="D407" r:id="rId1379"/>
-    <x:hyperlink ref="D408" r:id="rId1380"/>
-    <x:hyperlink ref="D409" r:id="rId1381"/>
-    <x:hyperlink ref="D410" r:id="rId1382"/>
-    <x:hyperlink ref="D411" r:id="rId1383"/>
-    <x:hyperlink ref="D412" r:id="rId1384"/>
-    <x:hyperlink ref="D413" r:id="rId1385"/>
-    <x:hyperlink ref="D414" r:id="rId1386"/>
-    <x:hyperlink ref="D415" r:id="rId1387"/>
-    <x:hyperlink ref="D416" r:id="rId1388"/>
-    <x:hyperlink ref="D417" r:id="rId1389"/>
-    <x:hyperlink ref="D418" r:id="rId1390"/>
-    <x:hyperlink ref="D419" r:id="rId1391"/>
-    <x:hyperlink ref="D420" r:id="rId1392"/>
-    <x:hyperlink ref="D421" r:id="rId1393"/>
-    <x:hyperlink ref="D422" r:id="rId1394"/>
-    <x:hyperlink ref="D423" r:id="rId1395"/>
-    <x:hyperlink ref="D424" r:id="rId1396"/>
-    <x:hyperlink ref="D425" r:id="rId1397"/>
-    <x:hyperlink ref="D426" r:id="rId1398"/>
-    <x:hyperlink ref="D427" r:id="rId1399"/>
-    <x:hyperlink ref="D428" r:id="rId1400"/>
-    <x:hyperlink ref="D429" r:id="rId1401"/>
-    <x:hyperlink ref="D430" r:id="rId1402"/>
-    <x:hyperlink ref="D431" r:id="rId1403"/>
-    <x:hyperlink ref="D432" r:id="rId1404"/>
-    <x:hyperlink ref="D433" r:id="rId1405"/>
-    <x:hyperlink ref="D434" r:id="rId1406"/>
-    <x:hyperlink ref="D435" r:id="rId1407"/>
-    <x:hyperlink ref="D436" r:id="rId1408"/>
-    <x:hyperlink ref="D437" r:id="rId1409"/>
-    <x:hyperlink ref="D438" r:id="rId1410"/>
-    <x:hyperlink ref="D439" r:id="rId1411"/>
-    <x:hyperlink ref="D440" r:id="rId1412"/>
-    <x:hyperlink ref="D441" r:id="rId1413"/>
-    <x:hyperlink ref="D442" r:id="rId1414"/>
-    <x:hyperlink ref="D443" r:id="rId1415"/>
-    <x:hyperlink ref="D444" r:id="rId1416"/>
-    <x:hyperlink ref="D445" r:id="rId1417"/>
-    <x:hyperlink ref="D446" r:id="rId1418"/>
-    <x:hyperlink ref="D447" r:id="rId1419"/>
-    <x:hyperlink ref="D448" r:id="rId1420"/>
-    <x:hyperlink ref="D449" r:id="rId1421"/>
-    <x:hyperlink ref="D450" r:id="rId1422"/>
-    <x:hyperlink ref="D451" r:id="rId1423"/>
-    <x:hyperlink ref="D452" r:id="rId1424"/>
-    <x:hyperlink ref="D453" r:id="rId1425"/>
-    <x:hyperlink ref="D454" r:id="rId1426"/>
-    <x:hyperlink ref="D455" r:id="rId1427"/>
-    <x:hyperlink ref="D456" r:id="rId1428"/>
-    <x:hyperlink ref="D457" r:id="rId1429"/>
-    <x:hyperlink ref="D458" r:id="rId1430"/>
-    <x:hyperlink ref="D459" r:id="rId1431"/>
-    <x:hyperlink ref="D460" r:id="rId1432"/>
-    <x:hyperlink ref="D461" r:id="rId1433"/>
-    <x:hyperlink ref="D462" r:id="rId1434"/>
-    <x:hyperlink ref="D463" r:id="rId1435"/>
-    <x:hyperlink ref="D464" r:id="rId1436"/>
-    <x:hyperlink ref="D465" r:id="rId1437"/>
-    <x:hyperlink ref="D466" r:id="rId1438"/>
-    <x:hyperlink ref="D467" r:id="rId1439"/>
-    <x:hyperlink ref="D468" r:id="rId1440"/>
-    <x:hyperlink ref="D469" r:id="rId1441"/>
-    <x:hyperlink ref="D470" r:id="rId1442"/>
-    <x:hyperlink ref="D471" r:id="rId1443"/>
-    <x:hyperlink ref="D472" r:id="rId1444"/>
-    <x:hyperlink ref="D473" r:id="rId1445"/>
-    <x:hyperlink ref="D474" r:id="rId1446"/>
-    <x:hyperlink ref="D475" r:id="rId1447"/>
-    <x:hyperlink ref="D476" r:id="rId1448"/>
-    <x:hyperlink ref="D477" r:id="rId1449"/>
-    <x:hyperlink ref="D478" r:id="rId1450"/>
-    <x:hyperlink ref="D479" r:id="rId1451"/>
-    <x:hyperlink ref="D480" r:id="rId1452"/>
-    <x:hyperlink ref="D481" r:id="rId1453"/>
-    <x:hyperlink ref="D482" r:id="rId1454"/>
-    <x:hyperlink ref="D483" r:id="rId1455"/>
-    <x:hyperlink ref="D484" r:id="rId1456"/>
-    <x:hyperlink ref="D485" r:id="rId1457"/>
-    <x:hyperlink ref="D486" r:id="rId1458"/>
-    <x:hyperlink ref="D487" r:id="rId1459"/>
-    <x:hyperlink ref="D488" r:id="rId1460"/>
-    <x:hyperlink ref="D489" r:id="rId1461"/>
-    <x:hyperlink ref="D490" r:id="rId1462"/>
-    <x:hyperlink ref="D491" r:id="rId1463"/>
-    <x:hyperlink ref="D492" r:id="rId1464"/>
-    <x:hyperlink ref="D493" r:id="rId1465"/>
-    <x:hyperlink ref="D494" r:id="rId1466"/>
-    <x:hyperlink ref="D495" r:id="rId1467"/>
-    <x:hyperlink ref="D496" r:id="rId1468"/>
-    <x:hyperlink ref="D497" r:id="rId1469"/>
-    <x:hyperlink ref="D498" r:id="rId1470"/>
-    <x:hyperlink ref="D499" r:id="rId1471"/>
-    <x:hyperlink ref="D500" r:id="rId1472"/>
-    <x:hyperlink ref="D501" r:id="rId1473"/>
-    <x:hyperlink ref="D502" r:id="rId1474"/>
-    <x:hyperlink ref="D503" r:id="rId1475"/>
-    <x:hyperlink ref="D504" r:id="rId1476"/>
-    <x:hyperlink ref="D505" r:id="rId1477"/>
-    <x:hyperlink ref="D506" r:id="rId1478"/>
-    <x:hyperlink ref="D507" r:id="rId1479"/>
-    <x:hyperlink ref="D508" r:id="rId1480"/>
-    <x:hyperlink ref="D509" r:id="rId1481"/>
-    <x:hyperlink ref="D510" r:id="rId1482"/>
-    <x:hyperlink ref="D511" r:id="rId1483"/>
-    <x:hyperlink ref="D512" r:id="rId1484"/>
-    <x:hyperlink ref="D513" r:id="rId1485"/>
-    <x:hyperlink ref="D514" r:id="rId1486"/>
-    <x:hyperlink ref="D515" r:id="rId1487"/>
-    <x:hyperlink ref="D516" r:id="rId1488"/>
-    <x:hyperlink ref="D517" r:id="rId1489"/>
-    <x:hyperlink ref="D518" r:id="rId1490"/>
-    <x:hyperlink ref="D519" r:id="rId1491"/>
-    <x:hyperlink ref="D520" r:id="rId1492"/>
-    <x:hyperlink ref="D521" r:id="rId1493"/>
-    <x:hyperlink ref="D522" r:id="rId1494"/>
-    <x:hyperlink ref="D523" r:id="rId1495"/>
-    <x:hyperlink ref="D524" r:id="rId1496"/>
-    <x:hyperlink ref="D525" r:id="rId1497"/>
-    <x:hyperlink ref="D526" r:id="rId1498"/>
-    <x:hyperlink ref="D527" r:id="rId1499"/>
-    <x:hyperlink ref="D528" r:id="rId1500"/>
-    <x:hyperlink ref="D529" r:id="rId1501"/>
-    <x:hyperlink ref="D530" r:id="rId1502"/>
-    <x:hyperlink ref="D531" r:id="rId1503"/>
-    <x:hyperlink ref="D532" r:id="rId1504"/>
-    <x:hyperlink ref="D533" r:id="rId1505"/>
-    <x:hyperlink ref="D534" r:id="rId1506"/>
-    <x:hyperlink ref="D535" r:id="rId1507"/>
-    <x:hyperlink ref="D536" r:id="rId1508"/>
-    <x:hyperlink ref="D537" r:id="rId1509"/>
-    <x:hyperlink ref="D538" r:id="rId1510"/>
-    <x:hyperlink ref="D539" r:id="rId1511"/>
-    <x:hyperlink ref="D540" r:id="rId1512"/>
-    <x:hyperlink ref="D541" r:id="rId1513"/>
-    <x:hyperlink ref="D542" r:id="rId1514"/>
-    <x:hyperlink ref="D543" r:id="rId1515"/>
-    <x:hyperlink ref="D544" r:id="rId1516"/>
-    <x:hyperlink ref="D545" r:id="rId1517"/>
-    <x:hyperlink ref="D546" r:id="rId1518"/>
-    <x:hyperlink ref="D547" r:id="rId1519"/>
-    <x:hyperlink ref="D548" r:id="rId1520"/>
-    <x:hyperlink ref="D549" r:id="rId1521"/>
-    <x:hyperlink ref="D550" r:id="rId1522"/>
-    <x:hyperlink ref="D551" r:id="rId1523"/>
-    <x:hyperlink ref="D552" r:id="rId1524"/>
-    <x:hyperlink ref="D553" r:id="rId1525"/>
-    <x:hyperlink ref="D554" r:id="rId1526"/>
-    <x:hyperlink ref="D555" r:id="rId1527"/>
-    <x:hyperlink ref="D556" r:id="rId1528"/>
-    <x:hyperlink ref="D557" r:id="rId1529"/>
-    <x:hyperlink ref="D558" r:id="rId1530"/>
-    <x:hyperlink ref="D559" r:id="rId1531"/>
-    <x:hyperlink ref="D560" r:id="rId1532"/>
-    <x:hyperlink ref="D561" r:id="rId1533"/>
-    <x:hyperlink ref="D562" r:id="rId1534"/>
-    <x:hyperlink ref="D563" r:id="rId1535"/>
-    <x:hyperlink ref="D564" r:id="rId1536"/>
-    <x:hyperlink ref="D565" r:id="rId1537"/>
-    <x:hyperlink ref="D566" r:id="rId1538"/>
-    <x:hyperlink ref="D567" r:id="rId1539"/>
-    <x:hyperlink ref="D568" r:id="rId1540"/>
-    <x:hyperlink ref="D569" r:id="rId1541"/>
-    <x:hyperlink ref="D570" r:id="rId1542"/>
-    <x:hyperlink ref="D571" r:id="rId1543"/>
-    <x:hyperlink ref="D572" r:id="rId1544"/>
-    <x:hyperlink ref="D573" r:id="rId1545"/>
-    <x:hyperlink ref="D574" r:id="rId1546"/>
-    <x:hyperlink ref="D575" r:id="rId1547"/>
-    <x:hyperlink ref="D576" r:id="rId1548"/>
-    <x:hyperlink ref="D577" r:id="rId1549"/>
-    <x:hyperlink ref="D578" r:id="rId1550"/>
-    <x:hyperlink ref="D579" r:id="rId1551"/>
-    <x:hyperlink ref="D580" r:id="rId1552"/>
-    <x:hyperlink ref="D581" r:id="rId1553"/>
-    <x:hyperlink ref="D582" r:id="rId1554"/>
-    <x:hyperlink ref="D583" r:id="rId1555"/>
-    <x:hyperlink ref="D584" r:id="rId1556"/>
-    <x:hyperlink ref="D585" r:id="rId1557"/>
-    <x:hyperlink ref="D586" r:id="rId1558"/>
-    <x:hyperlink ref="D587" r:id="rId1559"/>
-    <x:hyperlink ref="D588" r:id="rId1560"/>
-    <x:hyperlink ref="D589" r:id="rId1561"/>
-    <x:hyperlink ref="D590" r:id="rId1562"/>
-    <x:hyperlink ref="D591" r:id="rId1563"/>
-    <x:hyperlink ref="D592" r:id="rId1564"/>
-    <x:hyperlink ref="D593" r:id="rId1565"/>
-    <x:hyperlink ref="D594" r:id="rId1566"/>
-    <x:hyperlink ref="D595" r:id="rId1567"/>
-    <x:hyperlink ref="D596" r:id="rId1568"/>
-    <x:hyperlink ref="D597" r:id="rId1569"/>
-    <x:hyperlink ref="D598" r:id="rId1570"/>
-    <x:hyperlink ref="D599" r:id="rId1571"/>
-    <x:hyperlink ref="D600" r:id="rId1572"/>
-    <x:hyperlink ref="D601" r:id="rId1573"/>
-    <x:hyperlink ref="D602" r:id="rId1574"/>
-    <x:hyperlink ref="D603" r:id="rId1575"/>
-    <x:hyperlink ref="D604" r:id="rId1576"/>
-    <x:hyperlink ref="D605" r:id="rId1577"/>
-    <x:hyperlink ref="D606" r:id="rId1578"/>
-    <x:hyperlink ref="D607" r:id="rId1579"/>
-    <x:hyperlink ref="D608" r:id="rId1580"/>
-    <x:hyperlink ref="D609" r:id="rId1581"/>
-    <x:hyperlink ref="D610" r:id="rId1582"/>
-    <x:hyperlink ref="D611" r:id="rId1583"/>
-    <x:hyperlink ref="D612" r:id="rId1584"/>
-    <x:hyperlink ref="D613" r:id="rId1585"/>
-    <x:hyperlink ref="D614" r:id="rId1586"/>
-    <x:hyperlink ref="D615" r:id="rId1587"/>
-    <x:hyperlink ref="D616" r:id="rId1588"/>
-    <x:hyperlink ref="D617" r:id="rId1589"/>
-    <x:hyperlink ref="D618" r:id="rId1590"/>
-    <x:hyperlink ref="D619" r:id="rId1591"/>
-    <x:hyperlink ref="D620" r:id="rId1592"/>
-    <x:hyperlink ref="D621" r:id="rId1593"/>
-    <x:hyperlink ref="D622" r:id="rId1594"/>
-    <x:hyperlink ref="D623" r:id="rId1595"/>
-    <x:hyperlink ref="D624" r:id="rId1596"/>
-    <x:hyperlink ref="D625" r:id="rId1597"/>
-    <x:hyperlink ref="D626" r:id="rId1598"/>
-    <x:hyperlink ref="D627" r:id="rId1599"/>
-    <x:hyperlink ref="D628" r:id="rId1600"/>
-    <x:hyperlink ref="D629" r:id="rId1601"/>
-    <x:hyperlink ref="D630" r:id="rId1602"/>
-    <x:hyperlink ref="D631" r:id="rId1603"/>
-    <x:hyperlink ref="D632" r:id="rId1604"/>
-    <x:hyperlink ref="D633" r:id="rId1605"/>
-    <x:hyperlink ref="D634" r:id="rId1606"/>
-    <x:hyperlink ref="D635" r:id="rId1607"/>
-    <x:hyperlink ref="D636" r:id="rId1608"/>
-    <x:hyperlink ref="D637" r:id="rId1609"/>
-    <x:hyperlink ref="D638" r:id="rId1610"/>
-    <x:hyperlink ref="D639" r:id="rId1611"/>
-    <x:hyperlink ref="D640" r:id="rId1612"/>
-    <x:hyperlink ref="D641" r:id="rId1613"/>
-    <x:hyperlink ref="D642" r:id="rId1614"/>
-    <x:hyperlink ref="D643" r:id="rId1615"/>
-    <x:hyperlink ref="D644" r:id="rId1616"/>
-    <x:hyperlink ref="D645" r:id="rId1617"/>
-    <x:hyperlink ref="D646" r:id="rId1618"/>
-    <x:hyperlink ref="D647" r:id="rId1619"/>
-    <x:hyperlink ref="D648" r:id="rId1620"/>
-    <x:hyperlink ref="D649" r:id="rId1621"/>
-    <x:hyperlink ref="D650" r:id="rId1622"/>
-    <x:hyperlink ref="D651" r:id="rId1623"/>
-    <x:hyperlink ref="D652" r:id="rId1624"/>
-    <x:hyperlink ref="D653" r:id="rId1625"/>
-    <x:hyperlink ref="D654" r:id="rId1626"/>
-    <x:hyperlink ref="D655" r:id="rId1627"/>
-    <x:hyperlink ref="D656" r:id="rId1628"/>
-    <x:hyperlink ref="D657" r:id="rId1629"/>
-    <x:hyperlink ref="D658" r:id="rId1630"/>
-    <x:hyperlink ref="D659" r:id="rId1631"/>
-    <x:hyperlink ref="D660" r:id="rId1632"/>
-    <x:hyperlink ref="D661" r:id="rId1633"/>
-    <x:hyperlink ref="D662" r:id="rId1634"/>
-    <x:hyperlink ref="D663" r:id="rId1635"/>
-    <x:hyperlink ref="D664" r:id="rId1636"/>
-    <x:hyperlink ref="D665" r:id="rId1637"/>
-    <x:hyperlink ref="D666" r:id="rId1638"/>
-    <x:hyperlink ref="D667" r:id="rId1639"/>
-    <x:hyperlink ref="D668" r:id="rId1640"/>
-    <x:hyperlink ref="D669" r:id="rId1641"/>
-    <x:hyperlink ref="D670" r:id="rId1642"/>
-    <x:hyperlink ref="D671" r:id="rId1643"/>
-    <x:hyperlink ref="D672" r:id="rId1644"/>
-    <x:hyperlink ref="D673" r:id="rId1645"/>
-    <x:hyperlink ref="D674" r:id="rId1646"/>
-    <x:hyperlink ref="D675" r:id="rId1647"/>
-    <x:hyperlink ref="D676" r:id="rId1648"/>
-    <x:hyperlink ref="D677" r:id="rId1649"/>
-    <x:hyperlink ref="D678" r:id="rId1650"/>
-    <x:hyperlink ref="D679" r:id="rId1651"/>
-    <x:hyperlink ref="D680" r:id="rId1652"/>
-    <x:hyperlink ref="D681" r:id="rId1653"/>
-    <x:hyperlink ref="D682" r:id="rId1654"/>
-    <x:hyperlink ref="D683" r:id="rId1655"/>
-    <x:hyperlink ref="D684" r:id="rId1656"/>
-    <x:hyperlink ref="D685" r:id="rId1657"/>
-    <x:hyperlink ref="D686" r:id="rId1658"/>
-    <x:hyperlink ref="D687" r:id="rId1659"/>
-    <x:hyperlink ref="D688" r:id="rId1660"/>
-    <x:hyperlink ref="D689" r:id="rId1661"/>
-    <x:hyperlink ref="D690" r:id="rId1662"/>
-    <x:hyperlink ref="D691" r:id="rId1663"/>
-    <x:hyperlink ref="D692" r:id="rId1664"/>
-    <x:hyperlink ref="D693" r:id="rId1665"/>
-    <x:hyperlink ref="D694" r:id="rId1666"/>
-    <x:hyperlink ref="D695" r:id="rId1667"/>
-    <x:hyperlink ref="D696" r:id="rId1668"/>
-    <x:hyperlink ref="D697" r:id="rId1669"/>
-    <x:hyperlink ref="D698" r:id="rId1670"/>
-    <x:hyperlink ref="D699" r:id="rId1671"/>
-    <x:hyperlink ref="D700" r:id="rId1672"/>
-    <x:hyperlink ref="D701" r:id="rId1673"/>
-    <x:hyperlink ref="D702" r:id="rId1674"/>
-    <x:hyperlink ref="D703" r:id="rId1675"/>
-    <x:hyperlink ref="D704" r:id="rId1676"/>
-    <x:hyperlink ref="D705" r:id="rId1677"/>
-    <x:hyperlink ref="D706" r:id="rId1678"/>
-    <x:hyperlink ref="D707" r:id="rId1679"/>
-    <x:hyperlink ref="D708" r:id="rId1680"/>
-    <x:hyperlink ref="D709" r:id="rId1681"/>
-    <x:hyperlink ref="D710" r:id="rId1682"/>
-    <x:hyperlink ref="D711" r:id="rId1683"/>
-    <x:hyperlink ref="D712" r:id="rId1684"/>
-    <x:hyperlink ref="D713" r:id="rId1685"/>
-    <x:hyperlink ref="D714" r:id="rId1686"/>
-    <x:hyperlink ref="D715" r:id="rId1687"/>
-    <x:hyperlink ref="D716" r:id="rId1688"/>
-    <x:hyperlink ref="D717" r:id="rId1689"/>
-    <x:hyperlink ref="D718" r:id="rId1690"/>
-    <x:hyperlink ref="D719" r:id="rId1691"/>
-    <x:hyperlink ref="D720" r:id="rId1692"/>
-    <x:hyperlink ref="D721" r:id="rId1693"/>
-    <x:hyperlink ref="D722" r:id="rId1694"/>
-    <x:hyperlink ref="D723" r:id="rId1695"/>
-    <x:hyperlink ref="D724" r:id="rId1696"/>
-    <x:hyperlink ref="D725" r:id="rId1697"/>
-    <x:hyperlink ref="D726" r:id="rId1698"/>
-    <x:hyperlink ref="D727" r:id="rId1699"/>
-    <x:hyperlink ref="D728" r:id="rId1700"/>
-    <x:hyperlink ref="D729" r:id="rId1701"/>
-    <x:hyperlink ref="D730" r:id="rId1702"/>
-    <x:hyperlink ref="D731" r:id="rId1703"/>
-    <x:hyperlink ref="D732" r:id="rId1704"/>
-    <x:hyperlink ref="D733" r:id="rId1705"/>
-    <x:hyperlink ref="D734" r:id="rId1706"/>
-    <x:hyperlink ref="D735" r:id="rId1707"/>
-    <x:hyperlink ref="D736" r:id="rId1708"/>
-    <x:hyperlink ref="D737" r:id="rId1709"/>
-    <x:hyperlink ref="D738" r:id="rId1710"/>
-    <x:hyperlink ref="D739" r:id="rId1711"/>
-    <x:hyperlink ref="D740" r:id="rId1712"/>
-    <x:hyperlink ref="D741" r:id="rId1713"/>
-    <x:hyperlink ref="D742" r:id="rId1714"/>
-    <x:hyperlink ref="D743" r:id="rId1715"/>
-    <x:hyperlink ref="D744" r:id="rId1716"/>
-    <x:hyperlink ref="D745" r:id="rId1717"/>
-    <x:hyperlink ref="D746" r:id="rId1718"/>
-    <x:hyperlink ref="D747" r:id="rId1719"/>
-    <x:hyperlink ref="D748" r:id="rId1720"/>
-    <x:hyperlink ref="D749" r:id="rId1721"/>
-    <x:hyperlink ref="D750" r:id="rId1722"/>
-    <x:hyperlink ref="D751" r:id="rId1723"/>
-    <x:hyperlink ref="D752" r:id="rId1724"/>
-    <x:hyperlink ref="D753" r:id="rId1725"/>
-    <x:hyperlink ref="D754" r:id="rId1726"/>
-    <x:hyperlink ref="D755" r:id="rId1727"/>
-    <x:hyperlink ref="D756" r:id="rId1728"/>
-    <x:hyperlink ref="D757" r:id="rId1729"/>
-    <x:hyperlink ref="D758" r:id="rId1730"/>
-    <x:hyperlink ref="D759" r:id="rId1731"/>
-    <x:hyperlink ref="D760" r:id="rId1732"/>
-    <x:hyperlink ref="D761" r:id="rId1733"/>
-    <x:hyperlink ref="D762" r:id="rId1734"/>
-    <x:hyperlink ref="D763" r:id="rId1735"/>
-    <x:hyperlink ref="D764" r:id="rId1736"/>
-    <x:hyperlink ref="D765" r:id="rId1737"/>
-    <x:hyperlink ref="D766" r:id="rId1738"/>
-    <x:hyperlink ref="D767" r:id="rId1739"/>
-    <x:hyperlink ref="D768" r:id="rId1740"/>
-    <x:hyperlink ref="D769" r:id="rId1741"/>
-    <x:hyperlink ref="D770" r:id="rId1742"/>
-    <x:hyperlink ref="D771" r:id="rId1743"/>
-    <x:hyperlink ref="D772" r:id="rId1744"/>
-    <x:hyperlink ref="D773" r:id="rId1745"/>
-    <x:hyperlink ref="D774" r:id="rId1746"/>
-    <x:hyperlink ref="D775" r:id="rId1747"/>
-    <x:hyperlink ref="D776" r:id="rId1748"/>
-    <x:hyperlink ref="D777" r:id="rId1749"/>
-    <x:hyperlink ref="D778" r:id="rId1750"/>
-    <x:hyperlink ref="D779" r:id="rId1751"/>
-    <x:hyperlink ref="D780" r:id="rId1752"/>
-    <x:hyperlink ref="D781" r:id="rId1753"/>
-    <x:hyperlink ref="D782" r:id="rId1754"/>
-    <x:hyperlink ref="D783" r:id="rId1755"/>
-    <x:hyperlink ref="D784" r:id="rId1756"/>
-    <x:hyperlink ref="D785" r:id="rId1757"/>
-    <x:hyperlink ref="D786" r:id="rId1758"/>
-    <x:hyperlink ref="D787" r:id="rId1759"/>
-    <x:hyperlink ref="D788" r:id="rId1760"/>
-    <x:hyperlink ref="D789" r:id="rId1761"/>
-    <x:hyperlink ref="D790" r:id="rId1762"/>
-    <x:hyperlink ref="D791" r:id="rId1763"/>
-    <x:hyperlink ref="D792" r:id="rId1764"/>
-    <x:hyperlink ref="D793" r:id="rId1765"/>
-    <x:hyperlink ref="D794" r:id="rId1766"/>
-    <x:hyperlink ref="D795" r:id="rId1767"/>
-    <x:hyperlink ref="D796" r:id="rId1768"/>
-    <x:hyperlink ref="D797" r:id="rId1769"/>
-    <x:hyperlink ref="D798" r:id="rId1770"/>
-    <x:hyperlink ref="D799" r:id="rId1771"/>
-    <x:hyperlink ref="D800" r:id="rId1772"/>
-    <x:hyperlink ref="D801" r:id="rId1773"/>
-    <x:hyperlink ref="D802" r:id="rId1774"/>
-    <x:hyperlink ref="D803" r:id="rId1775"/>
-    <x:hyperlink ref="D804" r:id="rId1776"/>
-    <x:hyperlink ref="D805" r:id="rId1777"/>
-    <x:hyperlink ref="D806" r:id="rId1778"/>
-    <x:hyperlink ref="D807" r:id="rId1779"/>
-    <x:hyperlink ref="D808" r:id="rId1780"/>
-    <x:hyperlink ref="D809" r:id="rId1781"/>
-    <x:hyperlink ref="D810" r:id="rId1782"/>
-    <x:hyperlink ref="D811" r:id="rId1783"/>
-    <x:hyperlink ref="D812" r:id="rId1784"/>
-    <x:hyperlink ref="D813" r:id="rId1785"/>
-    <x:hyperlink ref="D814" r:id="rId1786"/>
-    <x:hyperlink ref="D815" r:id="rId1787"/>
-    <x:hyperlink ref="D816" r:id="rId1788"/>
-    <x:hyperlink ref="D817" r:id="rId1789"/>
-    <x:hyperlink ref="D818" r:id="rId1790"/>
-    <x:hyperlink ref="D819" r:id="rId1791"/>
-    <x:hyperlink ref="D820" r:id="rId1792"/>
-    <x:hyperlink ref="D821" r:id="rId1793"/>
-    <x:hyperlink ref="D822" r:id="rId1794"/>
-    <x:hyperlink ref="D823" r:id="rId1795"/>
-    <x:hyperlink ref="D824" r:id="rId1796"/>
-    <x:hyperlink ref="D825" r:id="rId1797"/>
-    <x:hyperlink ref="D826" r:id="rId1798"/>
-    <x:hyperlink ref="D827" r:id="rId1799"/>
-    <x:hyperlink ref="D828" r:id="rId1800"/>
-    <x:hyperlink ref="D829" r:id="rId1801"/>
-    <x:hyperlink ref="D830" r:id="rId1802"/>
-    <x:hyperlink ref="D831" r:id="rId1803"/>
-    <x:hyperlink ref="D832" r:id="rId1804"/>
-    <x:hyperlink ref="D833" r:id="rId1805"/>
-    <x:hyperlink ref="D834" r:id="rId1806"/>
-    <x:hyperlink ref="D835" r:id="rId1807"/>
-    <x:hyperlink ref="D836" r:id="rId1808"/>
-    <x:hyperlink ref="D837" r:id="rId1809"/>
-    <x:hyperlink ref="D838" r:id="rId1810"/>
-    <x:hyperlink ref="D839" r:id="rId1811"/>
-    <x:hyperlink ref="D840" r:id="rId1812"/>
-    <x:hyperlink ref="D841" r:id="rId1813"/>
-    <x:hyperlink ref="D842" r:id="rId1814"/>
-    <x:hyperlink ref="D843" r:id="rId1815"/>
-    <x:hyperlink ref="D844" r:id="rId1816"/>
-    <x:hyperlink ref="D845" r:id="rId1817"/>
-    <x:hyperlink ref="D846" r:id="rId1818"/>
-    <x:hyperlink ref="D847" r:id="rId1819"/>
-    <x:hyperlink ref="D848" r:id="rId1820"/>
-    <x:hyperlink ref="D849" r:id="rId1821"/>
-    <x:hyperlink ref="D850" r:id="rId1822"/>
-    <x:hyperlink ref="D851" r:id="rId1823"/>
-    <x:hyperlink ref="D852" r:id="rId1824"/>
-    <x:hyperlink ref="D853" r:id="rId1825"/>
-    <x:hyperlink ref="D854" r:id="rId1826"/>
-    <x:hyperlink ref="D855" r:id="rId1827"/>
-    <x:hyperlink ref="D856" r:id="rId1828"/>
-    <x:hyperlink ref="D857" r:id="rId1829"/>
-    <x:hyperlink ref="D858" r:id="rId1830"/>
-    <x:hyperlink ref="D859" r:id="rId1831"/>
-    <x:hyperlink ref="D860" r:id="rId1832"/>
-    <x:hyperlink ref="D861" r:id="rId1833"/>
-    <x:hyperlink ref="D862" r:id="rId1834"/>
-    <x:hyperlink ref="D863" r:id="rId1835"/>
-    <x:hyperlink ref="D864" r:id="rId1836"/>
-    <x:hyperlink ref="D865" r:id="rId1837"/>
-    <x:hyperlink ref="D866" r:id="rId1838"/>
-    <x:hyperlink ref="D867" r:id="rId1839"/>
-    <x:hyperlink ref="D868" r:id="rId1840"/>
-    <x:hyperlink ref="D869" r:id="rId1841"/>
-    <x:hyperlink ref="D870" r:id="rId1842"/>
-    <x:hyperlink ref="D871" r:id="rId1843"/>
-    <x:hyperlink ref="D872" r:id="rId1844"/>
-    <x:hyperlink ref="D873" r:id="rId1845"/>
-    <x:hyperlink ref="D874" r:id="rId1846"/>
-    <x:hyperlink ref="D875" r:id="rId1847"/>
-    <x:hyperlink ref="D876" r:id="rId1848"/>
-    <x:hyperlink ref="D877" r:id="rId1849"/>
-    <x:hyperlink ref="D878" r:id="rId1850"/>
-    <x:hyperlink ref="D879" r:id="rId1851"/>
-    <x:hyperlink ref="D880" r:id="rId1852"/>
-    <x:hyperlink ref="D881" r:id="rId1853"/>
-    <x:hyperlink ref="D882" r:id="rId1854"/>
-    <x:hyperlink ref="D883" r:id="rId1855"/>
-    <x:hyperlink ref="D884" r:id="rId1856"/>
-    <x:hyperlink ref="D885" r:id="rId1857"/>
-    <x:hyperlink ref="D886" r:id="rId1858"/>
-    <x:hyperlink ref="D887" r:id="rId1859"/>
-    <x:hyperlink ref="D888" r:id="rId1860"/>
-    <x:hyperlink ref="D889" r:id="rId1861"/>
-    <x:hyperlink ref="D890" r:id="rId1862"/>
-    <x:hyperlink ref="D891" r:id="rId1863"/>
-    <x:hyperlink ref="D892" r:id="rId1864"/>
-    <x:hyperlink ref="D893" r:id="rId1865"/>
-    <x:hyperlink ref="D894" r:id="rId1866"/>
-    <x:hyperlink ref="D895" r:id="rId1867"/>
-    <x:hyperlink ref="D896" r:id="rId1868"/>
-    <x:hyperlink ref="D897" r:id="rId1869"/>
-    <x:hyperlink ref="D898" r:id="rId1870"/>
-    <x:hyperlink ref="D899" r:id="rId1871"/>
-    <x:hyperlink ref="D900" r:id="rId1872"/>
-    <x:hyperlink ref="D901" r:id="rId1873"/>
-    <x:hyperlink ref="D902" r:id="rId1874"/>
-    <x:hyperlink ref="D903" r:id="rId1875"/>
-    <x:hyperlink ref="D904" r:id="rId1876"/>
-    <x:hyperlink ref="D905" r:id="rId1877"/>
-    <x:hyperlink ref="D906" r:id="rId1878"/>
-    <x:hyperlink ref="D907" r:id="rId1879"/>
-    <x:hyperlink ref="D908" r:id="rId1880"/>
-    <x:hyperlink ref="D909" r:id="rId1881"/>
-    <x:hyperlink ref="D910" r:id="rId1882"/>
-    <x:hyperlink ref="D911" r:id="rId1883"/>
-    <x:hyperlink ref="D912" r:id="rId1884"/>
-    <x:hyperlink ref="D913" r:id="rId1885"/>
-    <x:hyperlink ref="D914" r:id="rId1886"/>
-    <x:hyperlink ref="D915" r:id="rId1887"/>
-    <x:hyperlink ref="D916" r:id="rId1888"/>
-    <x:hyperlink ref="D917" r:id="rId1889"/>
-    <x:hyperlink ref="D918" r:id="rId1890"/>
-    <x:hyperlink ref="D919" r:id="rId1891"/>
-    <x:hyperlink ref="D920" r:id="rId1892"/>
-    <x:hyperlink ref="D921" r:id="rId1893"/>
-    <x:hyperlink ref="D922" r:id="rId1894"/>
-    <x:hyperlink ref="D923" r:id="rId1895"/>
-    <x:hyperlink ref="D924" r:id="rId1896"/>
-    <x:hyperlink ref="D925" r:id="rId1897"/>
-    <x:hyperlink ref="D926" r:id="rId1898"/>
-    <x:hyperlink ref="D927" r:id="rId1899"/>
-    <x:hyperlink ref="D928" r:id="rId1900"/>
-    <x:hyperlink ref="D929" r:id="rId1901"/>
-    <x:hyperlink ref="D930" r:id="rId1902"/>
-    <x:hyperlink ref="D931" r:id="rId1903"/>
-    <x:hyperlink ref="D932" r:id="rId1904"/>
-    <x:hyperlink ref="D933" r:id="rId1905"/>
-    <x:hyperlink ref="D934" r:id="rId1906"/>
-    <x:hyperlink ref="D935" r:id="rId1907"/>
-    <x:hyperlink ref="D936" r:id="rId1908"/>
-    <x:hyperlink ref="D937" r:id="rId1909"/>
-    <x:hyperlink ref="D938" r:id="rId1910"/>
-    <x:hyperlink ref="D939" r:id="rId1911"/>
-    <x:hyperlink ref="D940" r:id="rId1912"/>
-    <x:hyperlink ref="D941" r:id="rId1913"/>
-    <x:hyperlink ref="D942" r:id="rId1914"/>
-    <x:hyperlink ref="D943" r:id="rId1915"/>
-    <x:hyperlink ref="D944" r:id="rId1916"/>
-    <x:hyperlink ref="D945" r:id="rId1917"/>
-    <x:hyperlink ref="D946" r:id="rId1918"/>
-    <x:hyperlink ref="D947" r:id="rId1919"/>
-    <x:hyperlink ref="D948" r:id="rId1920"/>
-    <x:hyperlink ref="D949" r:id="rId1921"/>
-    <x:hyperlink ref="D950" r:id="rId1922"/>
-    <x:hyperlink ref="D951" r:id="rId1923"/>
-    <x:hyperlink ref="D952" r:id="rId1924"/>
-    <x:hyperlink ref="D953" r:id="rId1925"/>
-    <x:hyperlink ref="D954" r:id="rId1926"/>
-    <x:hyperlink ref="D955" r:id="rId1927"/>
-    <x:hyperlink ref="D956" r:id="rId1928"/>
-    <x:hyperlink ref="D957" r:id="rId1929"/>
-    <x:hyperlink ref="D958" r:id="rId1930"/>
-    <x:hyperlink ref="D959" r:id="rId1931"/>
-    <x:hyperlink ref="D960" r:id="rId1932"/>
-    <x:hyperlink ref="D961" r:id="rId1933"/>
-    <x:hyperlink ref="D962" r:id="rId1934"/>
-    <x:hyperlink ref="D963" r:id="rId1935"/>
-    <x:hyperlink ref="D964" r:id="rId1936"/>
-    <x:hyperlink ref="D965" r:id="rId1937"/>
-    <x:hyperlink ref="D966" r:id="rId1938"/>
-    <x:hyperlink ref="D967" r:id="rId1939"/>
-    <x:hyperlink ref="D968" r:id="rId1940"/>
-    <x:hyperlink ref="D969" r:id="rId1941"/>
-    <x:hyperlink ref="D970" r:id="rId1942"/>
-    <x:hyperlink ref="D971" r:id="rId1943"/>
-    <x:hyperlink ref="D972" r:id="rId1944"/>
-    <x:hyperlink ref="D973" r:id="rId1945"/>
-    <x:hyperlink ref="D974" r:id="rId1946"/>
-    <x:hyperlink ref="D975" r:id="rId1947"/>
+    <x:hyperlink ref="D6" r:id="rId982"/>
+    <x:hyperlink ref="D7" r:id="rId983"/>
+    <x:hyperlink ref="D8" r:id="rId984"/>
+    <x:hyperlink ref="D9" r:id="rId985"/>
+    <x:hyperlink ref="D10" r:id="rId986"/>
+    <x:hyperlink ref="D11" r:id="rId987"/>
+    <x:hyperlink ref="D12" r:id="rId988"/>
+    <x:hyperlink ref="D13" r:id="rId989"/>
+    <x:hyperlink ref="D14" r:id="rId990"/>
+    <x:hyperlink ref="D15" r:id="rId991"/>
+    <x:hyperlink ref="D16" r:id="rId992"/>
+    <x:hyperlink ref="D17" r:id="rId993"/>
+    <x:hyperlink ref="D18" r:id="rId994"/>
+    <x:hyperlink ref="D19" r:id="rId995"/>
+    <x:hyperlink ref="D20" r:id="rId996"/>
+    <x:hyperlink ref="D21" r:id="rId997"/>
+    <x:hyperlink ref="D22" r:id="rId998"/>
+    <x:hyperlink ref="D23" r:id="rId999"/>
+    <x:hyperlink ref="D24" r:id="rId1000"/>
+    <x:hyperlink ref="D25" r:id="rId1001"/>
+    <x:hyperlink ref="D26" r:id="rId1002"/>
+    <x:hyperlink ref="D27" r:id="rId1003"/>
+    <x:hyperlink ref="D28" r:id="rId1004"/>
+    <x:hyperlink ref="D29" r:id="rId1005"/>
+    <x:hyperlink ref="D30" r:id="rId1006"/>
+    <x:hyperlink ref="D31" r:id="rId1007"/>
+    <x:hyperlink ref="D32" r:id="rId1008"/>
+    <x:hyperlink ref="D33" r:id="rId1009"/>
+    <x:hyperlink ref="D34" r:id="rId1010"/>
+    <x:hyperlink ref="D35" r:id="rId1011"/>
+    <x:hyperlink ref="D36" r:id="rId1012"/>
+    <x:hyperlink ref="D37" r:id="rId1013"/>
+    <x:hyperlink ref="D38" r:id="rId1014"/>
+    <x:hyperlink ref="D39" r:id="rId1015"/>
+    <x:hyperlink ref="D40" r:id="rId1016"/>
+    <x:hyperlink ref="D41" r:id="rId1017"/>
+    <x:hyperlink ref="D42" r:id="rId1018"/>
+    <x:hyperlink ref="D43" r:id="rId1019"/>
+    <x:hyperlink ref="D44" r:id="rId1020"/>
+    <x:hyperlink ref="D45" r:id="rId1021"/>
+    <x:hyperlink ref="D46" r:id="rId1022"/>
+    <x:hyperlink ref="D47" r:id="rId1023"/>
+    <x:hyperlink ref="D48" r:id="rId1024"/>
+    <x:hyperlink ref="D49" r:id="rId1025"/>
+    <x:hyperlink ref="D50" r:id="rId1026"/>
+    <x:hyperlink ref="D51" r:id="rId1027"/>
+    <x:hyperlink ref="D52" r:id="rId1028"/>
+    <x:hyperlink ref="D53" r:id="rId1029"/>
+    <x:hyperlink ref="D54" r:id="rId1030"/>
+    <x:hyperlink ref="D55" r:id="rId1031"/>
+    <x:hyperlink ref="D56" r:id="rId1032"/>
+    <x:hyperlink ref="D57" r:id="rId1033"/>
+    <x:hyperlink ref="D58" r:id="rId1034"/>
+    <x:hyperlink ref="D59" r:id="rId1035"/>
+    <x:hyperlink ref="D60" r:id="rId1036"/>
+    <x:hyperlink ref="D61" r:id="rId1037"/>
+    <x:hyperlink ref="D62" r:id="rId1038"/>
+    <x:hyperlink ref="D63" r:id="rId1039"/>
+    <x:hyperlink ref="D64" r:id="rId1040"/>
+    <x:hyperlink ref="D65" r:id="rId1041"/>
+    <x:hyperlink ref="D66" r:id="rId1042"/>
+    <x:hyperlink ref="D67" r:id="rId1043"/>
+    <x:hyperlink ref="D68" r:id="rId1044"/>
+    <x:hyperlink ref="D69" r:id="rId1045"/>
+    <x:hyperlink ref="D70" r:id="rId1046"/>
+    <x:hyperlink ref="D71" r:id="rId1047"/>
+    <x:hyperlink ref="D72" r:id="rId1048"/>
+    <x:hyperlink ref="D73" r:id="rId1049"/>
+    <x:hyperlink ref="D74" r:id="rId1050"/>
+    <x:hyperlink ref="D75" r:id="rId1051"/>
+    <x:hyperlink ref="D76" r:id="rId1052"/>
+    <x:hyperlink ref="D77" r:id="rId1053"/>
+    <x:hyperlink ref="D78" r:id="rId1054"/>
+    <x:hyperlink ref="D79" r:id="rId1055"/>
+    <x:hyperlink ref="D80" r:id="rId1056"/>
+    <x:hyperlink ref="D81" r:id="rId1057"/>
+    <x:hyperlink ref="D82" r:id="rId1058"/>
+    <x:hyperlink ref="D83" r:id="rId1059"/>
+    <x:hyperlink ref="D84" r:id="rId1060"/>
+    <x:hyperlink ref="D85" r:id="rId1061"/>
+    <x:hyperlink ref="D86" r:id="rId1062"/>
+    <x:hyperlink ref="D87" r:id="rId1063"/>
+    <x:hyperlink ref="D88" r:id="rId1064"/>
+    <x:hyperlink ref="D89" r:id="rId1065"/>
+    <x:hyperlink ref="D90" r:id="rId1066"/>
+    <x:hyperlink ref="D91" r:id="rId1067"/>
+    <x:hyperlink ref="D92" r:id="rId1068"/>
+    <x:hyperlink ref="D93" r:id="rId1069"/>
+    <x:hyperlink ref="D94" r:id="rId1070"/>
+    <x:hyperlink ref="D95" r:id="rId1071"/>
+    <x:hyperlink ref="D96" r:id="rId1072"/>
+    <x:hyperlink ref="D97" r:id="rId1073"/>
+    <x:hyperlink ref="D98" r:id="rId1074"/>
+    <x:hyperlink ref="D99" r:id="rId1075"/>
+    <x:hyperlink ref="D100" r:id="rId1076"/>
+    <x:hyperlink ref="D101" r:id="rId1077"/>
+    <x:hyperlink ref="D102" r:id="rId1078"/>
+    <x:hyperlink ref="D103" r:id="rId1079"/>
+    <x:hyperlink ref="D104" r:id="rId1080"/>
+    <x:hyperlink ref="D105" r:id="rId1081"/>
+    <x:hyperlink ref="D106" r:id="rId1082"/>
+    <x:hyperlink ref="D107" r:id="rId1083"/>
+    <x:hyperlink ref="D108" r:id="rId1084"/>
+    <x:hyperlink ref="D109" r:id="rId1085"/>
+    <x:hyperlink ref="D110" r:id="rId1086"/>
+    <x:hyperlink ref="D111" r:id="rId1087"/>
+    <x:hyperlink ref="D112" r:id="rId1088"/>
+    <x:hyperlink ref="D113" r:id="rId1089"/>
+    <x:hyperlink ref="D114" r:id="rId1090"/>
+    <x:hyperlink ref="D115" r:id="rId1091"/>
+    <x:hyperlink ref="D116" r:id="rId1092"/>
+    <x:hyperlink ref="D117" r:id="rId1093"/>
+    <x:hyperlink ref="D118" r:id="rId1094"/>
+    <x:hyperlink ref="D119" r:id="rId1095"/>
+    <x:hyperlink ref="D120" r:id="rId1096"/>
+    <x:hyperlink ref="D121" r:id="rId1097"/>
+    <x:hyperlink ref="D122" r:id="rId1098"/>
+    <x:hyperlink ref="D123" r:id="rId1099"/>
+    <x:hyperlink ref="D124" r:id="rId1100"/>
+    <x:hyperlink ref="D125" r:id="rId1101"/>
+    <x:hyperlink ref="D126" r:id="rId1102"/>
+    <x:hyperlink ref="D127" r:id="rId1103"/>
+    <x:hyperlink ref="D128" r:id="rId1104"/>
+    <x:hyperlink ref="D129" r:id="rId1105"/>
+    <x:hyperlink ref="D130" r:id="rId1106"/>
+    <x:hyperlink ref="D131" r:id="rId1107"/>
+    <x:hyperlink ref="D132" r:id="rId1108"/>
+    <x:hyperlink ref="D133" r:id="rId1109"/>
+    <x:hyperlink ref="D134" r:id="rId1110"/>
+    <x:hyperlink ref="D135" r:id="rId1111"/>
+    <x:hyperlink ref="D136" r:id="rId1112"/>
+    <x:hyperlink ref="D137" r:id="rId1113"/>
+    <x:hyperlink ref="D138" r:id="rId1114"/>
+    <x:hyperlink ref="D139" r:id="rId1115"/>
+    <x:hyperlink ref="D140" r:id="rId1116"/>
+    <x:hyperlink ref="D141" r:id="rId1117"/>
+    <x:hyperlink ref="D142" r:id="rId1118"/>
+    <x:hyperlink ref="D143" r:id="rId1119"/>
+    <x:hyperlink ref="D144" r:id="rId1120"/>
+    <x:hyperlink ref="D145" r:id="rId1121"/>
+    <x:hyperlink ref="D146" r:id="rId1122"/>
+    <x:hyperlink ref="D147" r:id="rId1123"/>
+    <x:hyperlink ref="D148" r:id="rId1124"/>
+    <x:hyperlink ref="D149" r:id="rId1125"/>
+    <x:hyperlink ref="D150" r:id="rId1126"/>
+    <x:hyperlink ref="D151" r:id="rId1127"/>
+    <x:hyperlink ref="D152" r:id="rId1128"/>
+    <x:hyperlink ref="D153" r:id="rId1129"/>
+    <x:hyperlink ref="D154" r:id="rId1130"/>
+    <x:hyperlink ref="D155" r:id="rId1131"/>
+    <x:hyperlink ref="D156" r:id="rId1132"/>
+    <x:hyperlink ref="D157" r:id="rId1133"/>
+    <x:hyperlink ref="D158" r:id="rId1134"/>
+    <x:hyperlink ref="D159" r:id="rId1135"/>
+    <x:hyperlink ref="D160" r:id="rId1136"/>
+    <x:hyperlink ref="D161" r:id="rId1137"/>
+    <x:hyperlink ref="D162" r:id="rId1138"/>
+    <x:hyperlink ref="D163" r:id="rId1139"/>
+    <x:hyperlink ref="D164" r:id="rId1140"/>
+    <x:hyperlink ref="D165" r:id="rId1141"/>
+    <x:hyperlink ref="D166" r:id="rId1142"/>
+    <x:hyperlink ref="D167" r:id="rId1143"/>
+    <x:hyperlink ref="D168" r:id="rId1144"/>
+    <x:hyperlink ref="D169" r:id="rId1145"/>
+    <x:hyperlink ref="D170" r:id="rId1146"/>
+    <x:hyperlink ref="D171" r:id="rId1147"/>
+    <x:hyperlink ref="D172" r:id="rId1148"/>
+    <x:hyperlink ref="D173" r:id="rId1149"/>
+    <x:hyperlink ref="D174" r:id="rId1150"/>
+    <x:hyperlink ref="D175" r:id="rId1151"/>
+    <x:hyperlink ref="D176" r:id="rId1152"/>
+    <x:hyperlink ref="D177" r:id="rId1153"/>
+    <x:hyperlink ref="D178" r:id="rId1154"/>
+    <x:hyperlink ref="D179" r:id="rId1155"/>
+    <x:hyperlink ref="D180" r:id="rId1156"/>
+    <x:hyperlink ref="D181" r:id="rId1157"/>
+    <x:hyperlink ref="D182" r:id="rId1158"/>
+    <x:hyperlink ref="D183" r:id="rId1159"/>
+    <x:hyperlink ref="D184" r:id="rId1160"/>
+    <x:hyperlink ref="D185" r:id="rId1161"/>
+    <x:hyperlink ref="D186" r:id="rId1162"/>
+    <x:hyperlink ref="D187" r:id="rId1163"/>
+    <x:hyperlink ref="D188" r:id="rId1164"/>
+    <x:hyperlink ref="D189" r:id="rId1165"/>
+    <x:hyperlink ref="D190" r:id="rId1166"/>
+    <x:hyperlink ref="D191" r:id="rId1167"/>
+    <x:hyperlink ref="D192" r:id="rId1168"/>
+    <x:hyperlink ref="D193" r:id="rId1169"/>
+    <x:hyperlink ref="D194" r:id="rId1170"/>
+    <x:hyperlink ref="D195" r:id="rId1171"/>
+    <x:hyperlink ref="D196" r:id="rId1172"/>
+    <x:hyperlink ref="D197" r:id="rId1173"/>
+    <x:hyperlink ref="D198" r:id="rId1174"/>
+    <x:hyperlink ref="D199" r:id="rId1175"/>
+    <x:hyperlink ref="D200" r:id="rId1176"/>
+    <x:hyperlink ref="D201" r:id="rId1177"/>
+    <x:hyperlink ref="D202" r:id="rId1178"/>
+    <x:hyperlink ref="D203" r:id="rId1179"/>
+    <x:hyperlink ref="D204" r:id="rId1180"/>
+    <x:hyperlink ref="D205" r:id="rId1181"/>
+    <x:hyperlink ref="D206" r:id="rId1182"/>
+    <x:hyperlink ref="D207" r:id="rId1183"/>
+    <x:hyperlink ref="D208" r:id="rId1184"/>
+    <x:hyperlink ref="D209" r:id="rId1185"/>
+    <x:hyperlink ref="D210" r:id="rId1186"/>
+    <x:hyperlink ref="D211" r:id="rId1187"/>
+    <x:hyperlink ref="D212" r:id="rId1188"/>
+    <x:hyperlink ref="D213" r:id="rId1189"/>
+    <x:hyperlink ref="D214" r:id="rId1190"/>
+    <x:hyperlink ref="D215" r:id="rId1191"/>
+    <x:hyperlink ref="D216" r:id="rId1192"/>
+    <x:hyperlink ref="D217" r:id="rId1193"/>
+    <x:hyperlink ref="D218" r:id="rId1194"/>
+    <x:hyperlink ref="D219" r:id="rId1195"/>
+    <x:hyperlink ref="D220" r:id="rId1196"/>
+    <x:hyperlink ref="D221" r:id="rId1197"/>
+    <x:hyperlink ref="D222" r:id="rId1198"/>
+    <x:hyperlink ref="D223" r:id="rId1199"/>
+    <x:hyperlink ref="D224" r:id="rId1200"/>
+    <x:hyperlink ref="D225" r:id="rId1201"/>
+    <x:hyperlink ref="D226" r:id="rId1202"/>
+    <x:hyperlink ref="D227" r:id="rId1203"/>
+    <x:hyperlink ref="D228" r:id="rId1204"/>
+    <x:hyperlink ref="D229" r:id="rId1205"/>
+    <x:hyperlink ref="D230" r:id="rId1206"/>
+    <x:hyperlink ref="D231" r:id="rId1207"/>
+    <x:hyperlink ref="D232" r:id="rId1208"/>
+    <x:hyperlink ref="D233" r:id="rId1209"/>
+    <x:hyperlink ref="D234" r:id="rId1210"/>
+    <x:hyperlink ref="D235" r:id="rId1211"/>
+    <x:hyperlink ref="D236" r:id="rId1212"/>
+    <x:hyperlink ref="D237" r:id="rId1213"/>
+    <x:hyperlink ref="D238" r:id="rId1214"/>
+    <x:hyperlink ref="D239" r:id="rId1215"/>
+    <x:hyperlink ref="D240" r:id="rId1216"/>
+    <x:hyperlink ref="D241" r:id="rId1217"/>
+    <x:hyperlink ref="D242" r:id="rId1218"/>
+    <x:hyperlink ref="D243" r:id="rId1219"/>
+    <x:hyperlink ref="D244" r:id="rId1220"/>
+    <x:hyperlink ref="D245" r:id="rId1221"/>
+    <x:hyperlink ref="D246" r:id="rId1222"/>
+    <x:hyperlink ref="D247" r:id="rId1223"/>
+    <x:hyperlink ref="D248" r:id="rId1224"/>
+    <x:hyperlink ref="D249" r:id="rId1225"/>
+    <x:hyperlink ref="D250" r:id="rId1226"/>
+    <x:hyperlink ref="D251" r:id="rId1227"/>
+    <x:hyperlink ref="D252" r:id="rId1228"/>
+    <x:hyperlink ref="D253" r:id="rId1229"/>
+    <x:hyperlink ref="D254" r:id="rId1230"/>
+    <x:hyperlink ref="D255" r:id="rId1231"/>
+    <x:hyperlink ref="D256" r:id="rId1232"/>
+    <x:hyperlink ref="D257" r:id="rId1233"/>
+    <x:hyperlink ref="D258" r:id="rId1234"/>
+    <x:hyperlink ref="D259" r:id="rId1235"/>
+    <x:hyperlink ref="D260" r:id="rId1236"/>
+    <x:hyperlink ref="D261" r:id="rId1237"/>
+    <x:hyperlink ref="D262" r:id="rId1238"/>
+    <x:hyperlink ref="D263" r:id="rId1239"/>
+    <x:hyperlink ref="D264" r:id="rId1240"/>
+    <x:hyperlink ref="D265" r:id="rId1241"/>
+    <x:hyperlink ref="D266" r:id="rId1242"/>
+    <x:hyperlink ref="D267" r:id="rId1243"/>
+    <x:hyperlink ref="D268" r:id="rId1244"/>
+    <x:hyperlink ref="D269" r:id="rId1245"/>
+    <x:hyperlink ref="D270" r:id="rId1246"/>
+    <x:hyperlink ref="D271" r:id="rId1247"/>
+    <x:hyperlink ref="D272" r:id="rId1248"/>
+    <x:hyperlink ref="D273" r:id="rId1249"/>
+    <x:hyperlink ref="D274" r:id="rId1250"/>
+    <x:hyperlink ref="D275" r:id="rId1251"/>
+    <x:hyperlink ref="D276" r:id="rId1252"/>
+    <x:hyperlink ref="D277" r:id="rId1253"/>
+    <x:hyperlink ref="D278" r:id="rId1254"/>
+    <x:hyperlink ref="D279" r:id="rId1255"/>
+    <x:hyperlink ref="D280" r:id="rId1256"/>
+    <x:hyperlink ref="D281" r:id="rId1257"/>
+    <x:hyperlink ref="D282" r:id="rId1258"/>
+    <x:hyperlink ref="D283" r:id="rId1259"/>
+    <x:hyperlink ref="D284" r:id="rId1260"/>
+    <x:hyperlink ref="D285" r:id="rId1261"/>
+    <x:hyperlink ref="D286" r:id="rId1262"/>
+    <x:hyperlink ref="D287" r:id="rId1263"/>
+    <x:hyperlink ref="D288" r:id="rId1264"/>
+    <x:hyperlink ref="D289" r:id="rId1265"/>
+    <x:hyperlink ref="D290" r:id="rId1266"/>
+    <x:hyperlink ref="D291" r:id="rId1267"/>
+    <x:hyperlink ref="D292" r:id="rId1268"/>
+    <x:hyperlink ref="D293" r:id="rId1269"/>
+    <x:hyperlink ref="D294" r:id="rId1270"/>
+    <x:hyperlink ref="D295" r:id="rId1271"/>
+    <x:hyperlink ref="D296" r:id="rId1272"/>
+    <x:hyperlink ref="D297" r:id="rId1273"/>
+    <x:hyperlink ref="D298" r:id="rId1274"/>
+    <x:hyperlink ref="D299" r:id="rId1275"/>
+    <x:hyperlink ref="D300" r:id="rId1276"/>
+    <x:hyperlink ref="D301" r:id="rId1277"/>
+    <x:hyperlink ref="D302" r:id="rId1278"/>
+    <x:hyperlink ref="D303" r:id="rId1279"/>
+    <x:hyperlink ref="D304" r:id="rId1280"/>
+    <x:hyperlink ref="D305" r:id="rId1281"/>
+    <x:hyperlink ref="D306" r:id="rId1282"/>
+    <x:hyperlink ref="D307" r:id="rId1283"/>
+    <x:hyperlink ref="D308" r:id="rId1284"/>
+    <x:hyperlink ref="D309" r:id="rId1285"/>
+    <x:hyperlink ref="D310" r:id="rId1286"/>
+    <x:hyperlink ref="D311" r:id="rId1287"/>
+    <x:hyperlink ref="D312" r:id="rId1288"/>
+    <x:hyperlink ref="D313" r:id="rId1289"/>
+    <x:hyperlink ref="D314" r:id="rId1290"/>
+    <x:hyperlink ref="D315" r:id="rId1291"/>
+    <x:hyperlink ref="D316" r:id="rId1292"/>
+    <x:hyperlink ref="D317" r:id="rId1293"/>
+    <x:hyperlink ref="D318" r:id="rId1294"/>
+    <x:hyperlink ref="D319" r:id="rId1295"/>
+    <x:hyperlink ref="D320" r:id="rId1296"/>
+    <x:hyperlink ref="D321" r:id="rId1297"/>
+    <x:hyperlink ref="D322" r:id="rId1298"/>
+    <x:hyperlink ref="D323" r:id="rId1299"/>
+    <x:hyperlink ref="D324" r:id="rId1300"/>
+    <x:hyperlink ref="D325" r:id="rId1301"/>
+    <x:hyperlink ref="D326" r:id="rId1302"/>
+    <x:hyperlink ref="D327" r:id="rId1303"/>
+    <x:hyperlink ref="D328" r:id="rId1304"/>
+    <x:hyperlink ref="D329" r:id="rId1305"/>
+    <x:hyperlink ref="D330" r:id="rId1306"/>
+    <x:hyperlink ref="D331" r:id="rId1307"/>
+    <x:hyperlink ref="D332" r:id="rId1308"/>
+    <x:hyperlink ref="D333" r:id="rId1309"/>
+    <x:hyperlink ref="D334" r:id="rId1310"/>
+    <x:hyperlink ref="D335" r:id="rId1311"/>
+    <x:hyperlink ref="D336" r:id="rId1312"/>
+    <x:hyperlink ref="D337" r:id="rId1313"/>
+    <x:hyperlink ref="D338" r:id="rId1314"/>
+    <x:hyperlink ref="D339" r:id="rId1315"/>
+    <x:hyperlink ref="D340" r:id="rId1316"/>
+    <x:hyperlink ref="D341" r:id="rId1317"/>
+    <x:hyperlink ref="D342" r:id="rId1318"/>
+    <x:hyperlink ref="D343" r:id="rId1319"/>
+    <x:hyperlink ref="D344" r:id="rId1320"/>
+    <x:hyperlink ref="D345" r:id="rId1321"/>
+    <x:hyperlink ref="D346" r:id="rId1322"/>
+    <x:hyperlink ref="D347" r:id="rId1323"/>
+    <x:hyperlink ref="D348" r:id="rId1324"/>
+    <x:hyperlink ref="D349" r:id="rId1325"/>
+    <x:hyperlink ref="D350" r:id="rId1326"/>
+    <x:hyperlink ref="D351" r:id="rId1327"/>
+    <x:hyperlink ref="D352" r:id="rId1328"/>
+    <x:hyperlink ref="D353" r:id="rId1329"/>
+    <x:hyperlink ref="D354" r:id="rId1330"/>
+    <x:hyperlink ref="D355" r:id="rId1331"/>
+    <x:hyperlink ref="D356" r:id="rId1332"/>
+    <x:hyperlink ref="D357" r:id="rId1333"/>
+    <x:hyperlink ref="D358" r:id="rId1334"/>
+    <x:hyperlink ref="D359" r:id="rId1335"/>
+    <x:hyperlink ref="D360" r:id="rId1336"/>
+    <x:hyperlink ref="D361" r:id="rId1337"/>
+    <x:hyperlink ref="D362" r:id="rId1338"/>
+    <x:hyperlink ref="D363" r:id="rId1339"/>
+    <x:hyperlink ref="D364" r:id="rId1340"/>
+    <x:hyperlink ref="D365" r:id="rId1341"/>
+    <x:hyperlink ref="D366" r:id="rId1342"/>
+    <x:hyperlink ref="D367" r:id="rId1343"/>
+    <x:hyperlink ref="D368" r:id="rId1344"/>
+    <x:hyperlink ref="D369" r:id="rId1345"/>
+    <x:hyperlink ref="D370" r:id="rId1346"/>
+    <x:hyperlink ref="D371" r:id="rId1347"/>
+    <x:hyperlink ref="D372" r:id="rId1348"/>
+    <x:hyperlink ref="D373" r:id="rId1349"/>
+    <x:hyperlink ref="D374" r:id="rId1350"/>
+    <x:hyperlink ref="D375" r:id="rId1351"/>
+    <x:hyperlink ref="D376" r:id="rId1352"/>
+    <x:hyperlink ref="D377" r:id="rId1353"/>
+    <x:hyperlink ref="D378" r:id="rId1354"/>
+    <x:hyperlink ref="D379" r:id="rId1355"/>
+    <x:hyperlink ref="D380" r:id="rId1356"/>
+    <x:hyperlink ref="D381" r:id="rId1357"/>
+    <x:hyperlink ref="D382" r:id="rId1358"/>
+    <x:hyperlink ref="D383" r:id="rId1359"/>
+    <x:hyperlink ref="D384" r:id="rId1360"/>
+    <x:hyperlink ref="D385" r:id="rId1361"/>
+    <x:hyperlink ref="D386" r:id="rId1362"/>
+    <x:hyperlink ref="D387" r:id="rId1363"/>
+    <x:hyperlink ref="D388" r:id="rId1364"/>
+    <x:hyperlink ref="D389" r:id="rId1365"/>
+    <x:hyperlink ref="D390" r:id="rId1366"/>
+    <x:hyperlink ref="D391" r:id="rId1367"/>
+    <x:hyperlink ref="D392" r:id="rId1368"/>
+    <x:hyperlink ref="D393" r:id="rId1369"/>
+    <x:hyperlink ref="D394" r:id="rId1370"/>
+    <x:hyperlink ref="D395" r:id="rId1371"/>
+    <x:hyperlink ref="D396" r:id="rId1372"/>
+    <x:hyperlink ref="D397" r:id="rId1373"/>
+    <x:hyperlink ref="D398" r:id="rId1374"/>
+    <x:hyperlink ref="D399" r:id="rId1375"/>
+    <x:hyperlink ref="D400" r:id="rId1376"/>
+    <x:hyperlink ref="D401" r:id="rId1377"/>
+    <x:hyperlink ref="D402" r:id="rId1378"/>
+    <x:hyperlink ref="D403" r:id="rId1379"/>
+    <x:hyperlink ref="D404" r:id="rId1380"/>
+    <x:hyperlink ref="D405" r:id="rId1381"/>
+    <x:hyperlink ref="D406" r:id="rId1382"/>
+    <x:hyperlink ref="D407" r:id="rId1383"/>
+    <x:hyperlink ref="D408" r:id="rId1384"/>
+    <x:hyperlink ref="D409" r:id="rId1385"/>
+    <x:hyperlink ref="D410" r:id="rId1386"/>
+    <x:hyperlink ref="D411" r:id="rId1387"/>
+    <x:hyperlink ref="D412" r:id="rId1388"/>
+    <x:hyperlink ref="D413" r:id="rId1389"/>
+    <x:hyperlink ref="D414" r:id="rId1390"/>
+    <x:hyperlink ref="D415" r:id="rId1391"/>
+    <x:hyperlink ref="D416" r:id="rId1392"/>
+    <x:hyperlink ref="D417" r:id="rId1393"/>
+    <x:hyperlink ref="D418" r:id="rId1394"/>
+    <x:hyperlink ref="D419" r:id="rId1395"/>
+    <x:hyperlink ref="D420" r:id="rId1396"/>
+    <x:hyperlink ref="D421" r:id="rId1397"/>
+    <x:hyperlink ref="D422" r:id="rId1398"/>
+    <x:hyperlink ref="D423" r:id="rId1399"/>
+    <x:hyperlink ref="D424" r:id="rId1400"/>
+    <x:hyperlink ref="D425" r:id="rId1401"/>
+    <x:hyperlink ref="D426" r:id="rId1402"/>
+    <x:hyperlink ref="D427" r:id="rId1403"/>
+    <x:hyperlink ref="D428" r:id="rId1404"/>
+    <x:hyperlink ref="D429" r:id="rId1405"/>
+    <x:hyperlink ref="D430" r:id="rId1406"/>
+    <x:hyperlink ref="D431" r:id="rId1407"/>
+    <x:hyperlink ref="D432" r:id="rId1408"/>
+    <x:hyperlink ref="D433" r:id="rId1409"/>
+    <x:hyperlink ref="D434" r:id="rId1410"/>
+    <x:hyperlink ref="D435" r:id="rId1411"/>
+    <x:hyperlink ref="D436" r:id="rId1412"/>
+    <x:hyperlink ref="D437" r:id="rId1413"/>
+    <x:hyperlink ref="D438" r:id="rId1414"/>
+    <x:hyperlink ref="D439" r:id="rId1415"/>
+    <x:hyperlink ref="D440" r:id="rId1416"/>
+    <x:hyperlink ref="D441" r:id="rId1417"/>
+    <x:hyperlink ref="D442" r:id="rId1418"/>
+    <x:hyperlink ref="D443" r:id="rId1419"/>
+    <x:hyperlink ref="D444" r:id="rId1420"/>
+    <x:hyperlink ref="D445" r:id="rId1421"/>
+    <x:hyperlink ref="D446" r:id="rId1422"/>
+    <x:hyperlink ref="D447" r:id="rId1423"/>
+    <x:hyperlink ref="D448" r:id="rId1424"/>
+    <x:hyperlink ref="D449" r:id="rId1425"/>
+    <x:hyperlink ref="D450" r:id="rId1426"/>
+    <x:hyperlink ref="D451" r:id="rId1427"/>
+    <x:hyperlink ref="D452" r:id="rId1428"/>
+    <x:hyperlink ref="D453" r:id="rId1429"/>
+    <x:hyperlink ref="D454" r:id="rId1430"/>
+    <x:hyperlink ref="D455" r:id="rId1431"/>
+    <x:hyperlink ref="D456" r:id="rId1432"/>
+    <x:hyperlink ref="D457" r:id="rId1433"/>
+    <x:hyperlink ref="D458" r:id="rId1434"/>
+    <x:hyperlink ref="D459" r:id="rId1435"/>
+    <x:hyperlink ref="D460" r:id="rId1436"/>
+    <x:hyperlink ref="D461" r:id="rId1437"/>
+    <x:hyperlink ref="D462" r:id="rId1438"/>
+    <x:hyperlink ref="D463" r:id="rId1439"/>
+    <x:hyperlink ref="D464" r:id="rId1440"/>
+    <x:hyperlink ref="D465" r:id="rId1441"/>
+    <x:hyperlink ref="D466" r:id="rId1442"/>
+    <x:hyperlink ref="D467" r:id="rId1443"/>
+    <x:hyperlink ref="D468" r:id="rId1444"/>
+    <x:hyperlink ref="D469" r:id="rId1445"/>
+    <x:hyperlink ref="D470" r:id="rId1446"/>
+    <x:hyperlink ref="D471" r:id="rId1447"/>
+    <x:hyperlink ref="D472" r:id="rId1448"/>
+    <x:hyperlink ref="D473" r:id="rId1449"/>
+    <x:hyperlink ref="D474" r:id="rId1450"/>
+    <x:hyperlink ref="D475" r:id="rId1451"/>
+    <x:hyperlink ref="D476" r:id="rId1452"/>
+    <x:hyperlink ref="D477" r:id="rId1453"/>
+    <x:hyperlink ref="D478" r:id="rId1454"/>
+    <x:hyperlink ref="D479" r:id="rId1455"/>
+    <x:hyperlink ref="D480" r:id="rId1456"/>
+    <x:hyperlink ref="D481" r:id="rId1457"/>
+    <x:hyperlink ref="D482" r:id="rId1458"/>
+    <x:hyperlink ref="D483" r:id="rId1459"/>
+    <x:hyperlink ref="D484" r:id="rId1460"/>
+    <x:hyperlink ref="D485" r:id="rId1461"/>
+    <x:hyperlink ref="D486" r:id="rId1462"/>
+    <x:hyperlink ref="D487" r:id="rId1463"/>
+    <x:hyperlink ref="D488" r:id="rId1464"/>
+    <x:hyperlink ref="D489" r:id="rId1465"/>
+    <x:hyperlink ref="D490" r:id="rId1466"/>
+    <x:hyperlink ref="D491" r:id="rId1467"/>
+    <x:hyperlink ref="D492" r:id="rId1468"/>
+    <x:hyperlink ref="D493" r:id="rId1469"/>
+    <x:hyperlink ref="D494" r:id="rId1470"/>
+    <x:hyperlink ref="D495" r:id="rId1471"/>
+    <x:hyperlink ref="D496" r:id="rId1472"/>
+    <x:hyperlink ref="D497" r:id="rId1473"/>
+    <x:hyperlink ref="D498" r:id="rId1474"/>
+    <x:hyperlink ref="D499" r:id="rId1475"/>
+    <x:hyperlink ref="D500" r:id="rId1476"/>
+    <x:hyperlink ref="D501" r:id="rId1477"/>
+    <x:hyperlink ref="D502" r:id="rId1478"/>
+    <x:hyperlink ref="D503" r:id="rId1479"/>
+    <x:hyperlink ref="D504" r:id="rId1480"/>
+    <x:hyperlink ref="D505" r:id="rId1481"/>
+    <x:hyperlink ref="D506" r:id="rId1482"/>
+    <x:hyperlink ref="D507" r:id="rId1483"/>
+    <x:hyperlink ref="D508" r:id="rId1484"/>
+    <x:hyperlink ref="D509" r:id="rId1485"/>
+    <x:hyperlink ref="D510" r:id="rId1486"/>
+    <x:hyperlink ref="D511" r:id="rId1487"/>
+    <x:hyperlink ref="D512" r:id="rId1488"/>
+    <x:hyperlink ref="D513" r:id="rId1489"/>
+    <x:hyperlink ref="D514" r:id="rId1490"/>
+    <x:hyperlink ref="D515" r:id="rId1491"/>
+    <x:hyperlink ref="D516" r:id="rId1492"/>
+    <x:hyperlink ref="D517" r:id="rId1493"/>
+    <x:hyperlink ref="D518" r:id="rId1494"/>
+    <x:hyperlink ref="D519" r:id="rId1495"/>
+    <x:hyperlink ref="D520" r:id="rId1496"/>
+    <x:hyperlink ref="D521" r:id="rId1497"/>
+    <x:hyperlink ref="D522" r:id="rId1498"/>
+    <x:hyperlink ref="D523" r:id="rId1499"/>
+    <x:hyperlink ref="D524" r:id="rId1500"/>
+    <x:hyperlink ref="D525" r:id="rId1501"/>
+    <x:hyperlink ref="D526" r:id="rId1502"/>
+    <x:hyperlink ref="D527" r:id="rId1503"/>
+    <x:hyperlink ref="D528" r:id="rId1504"/>
+    <x:hyperlink ref="D529" r:id="rId1505"/>
+    <x:hyperlink ref="D530" r:id="rId1506"/>
+    <x:hyperlink ref="D531" r:id="rId1507"/>
+    <x:hyperlink ref="D532" r:id="rId1508"/>
+    <x:hyperlink ref="D533" r:id="rId1509"/>
+    <x:hyperlink ref="D534" r:id="rId1510"/>
+    <x:hyperlink ref="D535" r:id="rId1511"/>
+    <x:hyperlink ref="D536" r:id="rId1512"/>
+    <x:hyperlink ref="D537" r:id="rId1513"/>
+    <x:hyperlink ref="D538" r:id="rId1514"/>
+    <x:hyperlink ref="D539" r:id="rId1515"/>
+    <x:hyperlink ref="D540" r:id="rId1516"/>
+    <x:hyperlink ref="D541" r:id="rId1517"/>
+    <x:hyperlink ref="D542" r:id="rId1518"/>
+    <x:hyperlink ref="D543" r:id="rId1519"/>
+    <x:hyperlink ref="D544" r:id="rId1520"/>
+    <x:hyperlink ref="D545" r:id="rId1521"/>
+    <x:hyperlink ref="D546" r:id="rId1522"/>
+    <x:hyperlink ref="D547" r:id="rId1523"/>
+    <x:hyperlink ref="D548" r:id="rId1524"/>
+    <x:hyperlink ref="D549" r:id="rId1525"/>
+    <x:hyperlink ref="D550" r:id="rId1526"/>
+    <x:hyperlink ref="D551" r:id="rId1527"/>
+    <x:hyperlink ref="D552" r:id="rId1528"/>
+    <x:hyperlink ref="D553" r:id="rId1529"/>
+    <x:hyperlink ref="D554" r:id="rId1530"/>
+    <x:hyperlink ref="D555" r:id="rId1531"/>
+    <x:hyperlink ref="D556" r:id="rId1532"/>
+    <x:hyperlink ref="D557" r:id="rId1533"/>
+    <x:hyperlink ref="D558" r:id="rId1534"/>
+    <x:hyperlink ref="D559" r:id="rId1535"/>
+    <x:hyperlink ref="D560" r:id="rId1536"/>
+    <x:hyperlink ref="D561" r:id="rId1537"/>
+    <x:hyperlink ref="D562" r:id="rId1538"/>
+    <x:hyperlink ref="D563" r:id="rId1539"/>
+    <x:hyperlink ref="D564" r:id="rId1540"/>
+    <x:hyperlink ref="D565" r:id="rId1541"/>
+    <x:hyperlink ref="D566" r:id="rId1542"/>
+    <x:hyperlink ref="D567" r:id="rId1543"/>
+    <x:hyperlink ref="D568" r:id="rId1544"/>
+    <x:hyperlink ref="D569" r:id="rId1545"/>
+    <x:hyperlink ref="D570" r:id="rId1546"/>
+    <x:hyperlink ref="D571" r:id="rId1547"/>
+    <x:hyperlink ref="D572" r:id="rId1548"/>
+    <x:hyperlink ref="D573" r:id="rId1549"/>
+    <x:hyperlink ref="D574" r:id="rId1550"/>
+    <x:hyperlink ref="D575" r:id="rId1551"/>
+    <x:hyperlink ref="D576" r:id="rId1552"/>
+    <x:hyperlink ref="D577" r:id="rId1553"/>
+    <x:hyperlink ref="D578" r:id="rId1554"/>
+    <x:hyperlink ref="D579" r:id="rId1555"/>
+    <x:hyperlink ref="D580" r:id="rId1556"/>
+    <x:hyperlink ref="D581" r:id="rId1557"/>
+    <x:hyperlink ref="D582" r:id="rId1558"/>
+    <x:hyperlink ref="D583" r:id="rId1559"/>
+    <x:hyperlink ref="D584" r:id="rId1560"/>
+    <x:hyperlink ref="D585" r:id="rId1561"/>
+    <x:hyperlink ref="D586" r:id="rId1562"/>
+    <x:hyperlink ref="D587" r:id="rId1563"/>
+    <x:hyperlink ref="D588" r:id="rId1564"/>
+    <x:hyperlink ref="D589" r:id="rId1565"/>
+    <x:hyperlink ref="D590" r:id="rId1566"/>
+    <x:hyperlink ref="D591" r:id="rId1567"/>
+    <x:hyperlink ref="D592" r:id="rId1568"/>
+    <x:hyperlink ref="D593" r:id="rId1569"/>
+    <x:hyperlink ref="D594" r:id="rId1570"/>
+    <x:hyperlink ref="D595" r:id="rId1571"/>
+    <x:hyperlink ref="D596" r:id="rId1572"/>
+    <x:hyperlink ref="D597" r:id="rId1573"/>
+    <x:hyperlink ref="D598" r:id="rId1574"/>
+    <x:hyperlink ref="D599" r:id="rId1575"/>
+    <x:hyperlink ref="D600" r:id="rId1576"/>
+    <x:hyperlink ref="D601" r:id="rId1577"/>
+    <x:hyperlink ref="D602" r:id="rId1578"/>
+    <x:hyperlink ref="D603" r:id="rId1579"/>
+    <x:hyperlink ref="D604" r:id="rId1580"/>
+    <x:hyperlink ref="D605" r:id="rId1581"/>
+    <x:hyperlink ref="D606" r:id="rId1582"/>
+    <x:hyperlink ref="D607" r:id="rId1583"/>
+    <x:hyperlink ref="D608" r:id="rId1584"/>
+    <x:hyperlink ref="D609" r:id="rId1585"/>
+    <x:hyperlink ref="D610" r:id="rId1586"/>
+    <x:hyperlink ref="D611" r:id="rId1587"/>
+    <x:hyperlink ref="D612" r:id="rId1588"/>
+    <x:hyperlink ref="D613" r:id="rId1589"/>
+    <x:hyperlink ref="D614" r:id="rId1590"/>
+    <x:hyperlink ref="D615" r:id="rId1591"/>
+    <x:hyperlink ref="D616" r:id="rId1592"/>
+    <x:hyperlink ref="D617" r:id="rId1593"/>
+    <x:hyperlink ref="D618" r:id="rId1594"/>
+    <x:hyperlink ref="D619" r:id="rId1595"/>
+    <x:hyperlink ref="D620" r:id="rId1596"/>
+    <x:hyperlink ref="D621" r:id="rId1597"/>
+    <x:hyperlink ref="D622" r:id="rId1598"/>
+    <x:hyperlink ref="D623" r:id="rId1599"/>
+    <x:hyperlink ref="D624" r:id="rId1600"/>
+    <x:hyperlink ref="D625" r:id="rId1601"/>
+    <x:hyperlink ref="D626" r:id="rId1602"/>
+    <x:hyperlink ref="D627" r:id="rId1603"/>
+    <x:hyperlink ref="D628" r:id="rId1604"/>
+    <x:hyperlink ref="D629" r:id="rId1605"/>
+    <x:hyperlink ref="D630" r:id="rId1606"/>
+    <x:hyperlink ref="D631" r:id="rId1607"/>
+    <x:hyperlink ref="D632" r:id="rId1608"/>
+    <x:hyperlink ref="D633" r:id="rId1609"/>
+    <x:hyperlink ref="D634" r:id="rId1610"/>
+    <x:hyperlink ref="D635" r:id="rId1611"/>
+    <x:hyperlink ref="D636" r:id="rId1612"/>
+    <x:hyperlink ref="D637" r:id="rId1613"/>
+    <x:hyperlink ref="D638" r:id="rId1614"/>
+    <x:hyperlink ref="D639" r:id="rId1615"/>
+    <x:hyperlink ref="D640" r:id="rId1616"/>
+    <x:hyperlink ref="D641" r:id="rId1617"/>
+    <x:hyperlink ref="D642" r:id="rId1618"/>
+    <x:hyperlink ref="D643" r:id="rId1619"/>
+    <x:hyperlink ref="D644" r:id="rId1620"/>
+    <x:hyperlink ref="D645" r:id="rId1621"/>
+    <x:hyperlink ref="D646" r:id="rId1622"/>
+    <x:hyperlink ref="D647" r:id="rId1623"/>
+    <x:hyperlink ref="D648" r:id="rId1624"/>
+    <x:hyperlink ref="D649" r:id="rId1625"/>
+    <x:hyperlink ref="D650" r:id="rId1626"/>
+    <x:hyperlink ref="D651" r:id="rId1627"/>
+    <x:hyperlink ref="D652" r:id="rId1628"/>
+    <x:hyperlink ref="D653" r:id="rId1629"/>
+    <x:hyperlink ref="D654" r:id="rId1630"/>
+    <x:hyperlink ref="D655" r:id="rId1631"/>
+    <x:hyperlink ref="D656" r:id="rId1632"/>
+    <x:hyperlink ref="D657" r:id="rId1633"/>
+    <x:hyperlink ref="D658" r:id="rId1634"/>
+    <x:hyperlink ref="D659" r:id="rId1635"/>
+    <x:hyperlink ref="D660" r:id="rId1636"/>
+    <x:hyperlink ref="D661" r:id="rId1637"/>
+    <x:hyperlink ref="D662" r:id="rId1638"/>
+    <x:hyperlink ref="D663" r:id="rId1639"/>
+    <x:hyperlink ref="D664" r:id="rId1640"/>
+    <x:hyperlink ref="D665" r:id="rId1641"/>
+    <x:hyperlink ref="D666" r:id="rId1642"/>
+    <x:hyperlink ref="D667" r:id="rId1643"/>
+    <x:hyperlink ref="D668" r:id="rId1644"/>
+    <x:hyperlink ref="D669" r:id="rId1645"/>
+    <x:hyperlink ref="D670" r:id="rId1646"/>
+    <x:hyperlink ref="D671" r:id="rId1647"/>
+    <x:hyperlink ref="D672" r:id="rId1648"/>
+    <x:hyperlink ref="D673" r:id="rId1649"/>
+    <x:hyperlink ref="D674" r:id="rId1650"/>
+    <x:hyperlink ref="D675" r:id="rId1651"/>
+    <x:hyperlink ref="D676" r:id="rId1652"/>
+    <x:hyperlink ref="D677" r:id="rId1653"/>
+    <x:hyperlink ref="D678" r:id="rId1654"/>
+    <x:hyperlink ref="D679" r:id="rId1655"/>
+    <x:hyperlink ref="D680" r:id="rId1656"/>
+    <x:hyperlink ref="D681" r:id="rId1657"/>
+    <x:hyperlink ref="D682" r:id="rId1658"/>
+    <x:hyperlink ref="D683" r:id="rId1659"/>
+    <x:hyperlink ref="D684" r:id="rId1660"/>
+    <x:hyperlink ref="D685" r:id="rId1661"/>
+    <x:hyperlink ref="D686" r:id="rId1662"/>
+    <x:hyperlink ref="D687" r:id="rId1663"/>
+    <x:hyperlink ref="D688" r:id="rId1664"/>
+    <x:hyperlink ref="D689" r:id="rId1665"/>
+    <x:hyperlink ref="D690" r:id="rId1666"/>
+    <x:hyperlink ref="D691" r:id="rId1667"/>
+    <x:hyperlink ref="D692" r:id="rId1668"/>
+    <x:hyperlink ref="D693" r:id="rId1669"/>
+    <x:hyperlink ref="D694" r:id="rId1670"/>
+    <x:hyperlink ref="D695" r:id="rId1671"/>
+    <x:hyperlink ref="D696" r:id="rId1672"/>
+    <x:hyperlink ref="D697" r:id="rId1673"/>
+    <x:hyperlink ref="D698" r:id="rId1674"/>
+    <x:hyperlink ref="D699" r:id="rId1675"/>
+    <x:hyperlink ref="D700" r:id="rId1676"/>
+    <x:hyperlink ref="D701" r:id="rId1677"/>
+    <x:hyperlink ref="D702" r:id="rId1678"/>
+    <x:hyperlink ref="D703" r:id="rId1679"/>
+    <x:hyperlink ref="D704" r:id="rId1680"/>
+    <x:hyperlink ref="D705" r:id="rId1681"/>
+    <x:hyperlink ref="D706" r:id="rId1682"/>
+    <x:hyperlink ref="D707" r:id="rId1683"/>
+    <x:hyperlink ref="D708" r:id="rId1684"/>
+    <x:hyperlink ref="D709" r:id="rId1685"/>
+    <x:hyperlink ref="D710" r:id="rId1686"/>
+    <x:hyperlink ref="D711" r:id="rId1687"/>
+    <x:hyperlink ref="D712" r:id="rId1688"/>
+    <x:hyperlink ref="D713" r:id="rId1689"/>
+    <x:hyperlink ref="D714" r:id="rId1690"/>
+    <x:hyperlink ref="D715" r:id="rId1691"/>
+    <x:hyperlink ref="D716" r:id="rId1692"/>
+    <x:hyperlink ref="D717" r:id="rId1693"/>
+    <x:hyperlink ref="D718" r:id="rId1694"/>
+    <x:hyperlink ref="D719" r:id="rId1695"/>
+    <x:hyperlink ref="D720" r:id="rId1696"/>
+    <x:hyperlink ref="D721" r:id="rId1697"/>
+    <x:hyperlink ref="D722" r:id="rId1698"/>
+    <x:hyperlink ref="D723" r:id="rId1699"/>
+    <x:hyperlink ref="D724" r:id="rId1700"/>
+    <x:hyperlink ref="D725" r:id="rId1701"/>
+    <x:hyperlink ref="D726" r:id="rId1702"/>
+    <x:hyperlink ref="D727" r:id="rId1703"/>
+    <x:hyperlink ref="D728" r:id="rId1704"/>
+    <x:hyperlink ref="D729" r:id="rId1705"/>
+    <x:hyperlink ref="D730" r:id="rId1706"/>
+    <x:hyperlink ref="D731" r:id="rId1707"/>
+    <x:hyperlink ref="D732" r:id="rId1708"/>
+    <x:hyperlink ref="D733" r:id="rId1709"/>
+    <x:hyperlink ref="D734" r:id="rId1710"/>
+    <x:hyperlink ref="D735" r:id="rId1711"/>
+    <x:hyperlink ref="D736" r:id="rId1712"/>
+    <x:hyperlink ref="D737" r:id="rId1713"/>
+    <x:hyperlink ref="D738" r:id="rId1714"/>
+    <x:hyperlink ref="D739" r:id="rId1715"/>
+    <x:hyperlink ref="D740" r:id="rId1716"/>
+    <x:hyperlink ref="D741" r:id="rId1717"/>
+    <x:hyperlink ref="D742" r:id="rId1718"/>
+    <x:hyperlink ref="D743" r:id="rId1719"/>
+    <x:hyperlink ref="D744" r:id="rId1720"/>
+    <x:hyperlink ref="D745" r:id="rId1721"/>
+    <x:hyperlink ref="D746" r:id="rId1722"/>
+    <x:hyperlink ref="D747" r:id="rId1723"/>
+    <x:hyperlink ref="D748" r:id="rId1724"/>
+    <x:hyperlink ref="D749" r:id="rId1725"/>
+    <x:hyperlink ref="D750" r:id="rId1726"/>
+    <x:hyperlink ref="D751" r:id="rId1727"/>
+    <x:hyperlink ref="D752" r:id="rId1728"/>
+    <x:hyperlink ref="D753" r:id="rId1729"/>
+    <x:hyperlink ref="D754" r:id="rId1730"/>
+    <x:hyperlink ref="D755" r:id="rId1731"/>
+    <x:hyperlink ref="D756" r:id="rId1732"/>
+    <x:hyperlink ref="D757" r:id="rId1733"/>
+    <x:hyperlink ref="D758" r:id="rId1734"/>
+    <x:hyperlink ref="D759" r:id="rId1735"/>
+    <x:hyperlink ref="D760" r:id="rId1736"/>
+    <x:hyperlink ref="D761" r:id="rId1737"/>
+    <x:hyperlink ref="D762" r:id="rId1738"/>
+    <x:hyperlink ref="D763" r:id="rId1739"/>
+    <x:hyperlink ref="D764" r:id="rId1740"/>
+    <x:hyperlink ref="D765" r:id="rId1741"/>
+    <x:hyperlink ref="D766" r:id="rId1742"/>
+    <x:hyperlink ref="D767" r:id="rId1743"/>
+    <x:hyperlink ref="D768" r:id="rId1744"/>
+    <x:hyperlink ref="D769" r:id="rId1745"/>
+    <x:hyperlink ref="D770" r:id="rId1746"/>
+    <x:hyperlink ref="D771" r:id="rId1747"/>
+    <x:hyperlink ref="D772" r:id="rId1748"/>
+    <x:hyperlink ref="D773" r:id="rId1749"/>
+    <x:hyperlink ref="D774" r:id="rId1750"/>
+    <x:hyperlink ref="D775" r:id="rId1751"/>
+    <x:hyperlink ref="D776" r:id="rId1752"/>
+    <x:hyperlink ref="D777" r:id="rId1753"/>
+    <x:hyperlink ref="D778" r:id="rId1754"/>
+    <x:hyperlink ref="D779" r:id="rId1755"/>
+    <x:hyperlink ref="D780" r:id="rId1756"/>
+    <x:hyperlink ref="D781" r:id="rId1757"/>
+    <x:hyperlink ref="D782" r:id="rId1758"/>
+    <x:hyperlink ref="D783" r:id="rId1759"/>
+    <x:hyperlink ref="D784" r:id="rId1760"/>
+    <x:hyperlink ref="D785" r:id="rId1761"/>
+    <x:hyperlink ref="D786" r:id="rId1762"/>
+    <x:hyperlink ref="D787" r:id="rId1763"/>
+    <x:hyperlink ref="D788" r:id="rId1764"/>
+    <x:hyperlink ref="D789" r:id="rId1765"/>
+    <x:hyperlink ref="D790" r:id="rId1766"/>
+    <x:hyperlink ref="D791" r:id="rId1767"/>
+    <x:hyperlink ref="D792" r:id="rId1768"/>
+    <x:hyperlink ref="D793" r:id="rId1769"/>
+    <x:hyperlink ref="D794" r:id="rId1770"/>
+    <x:hyperlink ref="D795" r:id="rId1771"/>
+    <x:hyperlink ref="D796" r:id="rId1772"/>
+    <x:hyperlink ref="D797" r:id="rId1773"/>
+    <x:hyperlink ref="D798" r:id="rId1774"/>
+    <x:hyperlink ref="D799" r:id="rId1775"/>
+    <x:hyperlink ref="D800" r:id="rId1776"/>
+    <x:hyperlink ref="D801" r:id="rId1777"/>
+    <x:hyperlink ref="D802" r:id="rId1778"/>
+    <x:hyperlink ref="D803" r:id="rId1779"/>
+    <x:hyperlink ref="D804" r:id="rId1780"/>
+    <x:hyperlink ref="D805" r:id="rId1781"/>
+    <x:hyperlink ref="D806" r:id="rId1782"/>
+    <x:hyperlink ref="D807" r:id="rId1783"/>
+    <x:hyperlink ref="D808" r:id="rId1784"/>
+    <x:hyperlink ref="D809" r:id="rId1785"/>
+    <x:hyperlink ref="D810" r:id="rId1786"/>
+    <x:hyperlink ref="D811" r:id="rId1787"/>
+    <x:hyperlink ref="D812" r:id="rId1788"/>
+    <x:hyperlink ref="D813" r:id="rId1789"/>
+    <x:hyperlink ref="D814" r:id="rId1790"/>
+    <x:hyperlink ref="D815" r:id="rId1791"/>
+    <x:hyperlink ref="D816" r:id="rId1792"/>
+    <x:hyperlink ref="D817" r:id="rId1793"/>
+    <x:hyperlink ref="D818" r:id="rId1794"/>
+    <x:hyperlink ref="D819" r:id="rId1795"/>
+    <x:hyperlink ref="D820" r:id="rId1796"/>
+    <x:hyperlink ref="D821" r:id="rId1797"/>
+    <x:hyperlink ref="D822" r:id="rId1798"/>
+    <x:hyperlink ref="D823" r:id="rId1799"/>
+    <x:hyperlink ref="D824" r:id="rId1800"/>
+    <x:hyperlink ref="D825" r:id="rId1801"/>
+    <x:hyperlink ref="D826" r:id="rId1802"/>
+    <x:hyperlink ref="D827" r:id="rId1803"/>
+    <x:hyperlink ref="D828" r:id="rId1804"/>
+    <x:hyperlink ref="D829" r:id="rId1805"/>
+    <x:hyperlink ref="D830" r:id="rId1806"/>
+    <x:hyperlink ref="D831" r:id="rId1807"/>
+    <x:hyperlink ref="D832" r:id="rId1808"/>
+    <x:hyperlink ref="D833" r:id="rId1809"/>
+    <x:hyperlink ref="D834" r:id="rId1810"/>
+    <x:hyperlink ref="D835" r:id="rId1811"/>
+    <x:hyperlink ref="D836" r:id="rId1812"/>
+    <x:hyperlink ref="D837" r:id="rId1813"/>
+    <x:hyperlink ref="D838" r:id="rId1814"/>
+    <x:hyperlink ref="D839" r:id="rId1815"/>
+    <x:hyperlink ref="D840" r:id="rId1816"/>
+    <x:hyperlink ref="D841" r:id="rId1817"/>
+    <x:hyperlink ref="D842" r:id="rId1818"/>
+    <x:hyperlink ref="D843" r:id="rId1819"/>
+    <x:hyperlink ref="D844" r:id="rId1820"/>
+    <x:hyperlink ref="D845" r:id="rId1821"/>
+    <x:hyperlink ref="D846" r:id="rId1822"/>
+    <x:hyperlink ref="D847" r:id="rId1823"/>
+    <x:hyperlink ref="D848" r:id="rId1824"/>
+    <x:hyperlink ref="D849" r:id="rId1825"/>
+    <x:hyperlink ref="D850" r:id="rId1826"/>
+    <x:hyperlink ref="D851" r:id="rId1827"/>
+    <x:hyperlink ref="D852" r:id="rId1828"/>
+    <x:hyperlink ref="D853" r:id="rId1829"/>
+    <x:hyperlink ref="D854" r:id="rId1830"/>
+    <x:hyperlink ref="D855" r:id="rId1831"/>
+    <x:hyperlink ref="D856" r:id="rId1832"/>
+    <x:hyperlink ref="D857" r:id="rId1833"/>
+    <x:hyperlink ref="D858" r:id="rId1834"/>
+    <x:hyperlink ref="D859" r:id="rId1835"/>
+    <x:hyperlink ref="D860" r:id="rId1836"/>
+    <x:hyperlink ref="D861" r:id="rId1837"/>
+    <x:hyperlink ref="D862" r:id="rId1838"/>
+    <x:hyperlink ref="D863" r:id="rId1839"/>
+    <x:hyperlink ref="D864" r:id="rId1840"/>
+    <x:hyperlink ref="D865" r:id="rId1841"/>
+    <x:hyperlink ref="D866" r:id="rId1842"/>
+    <x:hyperlink ref="D867" r:id="rId1843"/>
+    <x:hyperlink ref="D868" r:id="rId1844"/>
+    <x:hyperlink ref="D869" r:id="rId1845"/>
+    <x:hyperlink ref="D870" r:id="rId1846"/>
+    <x:hyperlink ref="D871" r:id="rId1847"/>
+    <x:hyperlink ref="D872" r:id="rId1848"/>
+    <x:hyperlink ref="D873" r:id="rId1849"/>
+    <x:hyperlink ref="D874" r:id="rId1850"/>
+    <x:hyperlink ref="D875" r:id="rId1851"/>
+    <x:hyperlink ref="D876" r:id="rId1852"/>
+    <x:hyperlink ref="D877" r:id="rId1853"/>
+    <x:hyperlink ref="D878" r:id="rId1854"/>
+    <x:hyperlink ref="D879" r:id="rId1855"/>
+    <x:hyperlink ref="D880" r:id="rId1856"/>
+    <x:hyperlink ref="D881" r:id="rId1857"/>
+    <x:hyperlink ref="D882" r:id="rId1858"/>
+    <x:hyperlink ref="D883" r:id="rId1859"/>
+    <x:hyperlink ref="D884" r:id="rId1860"/>
+    <x:hyperlink ref="D885" r:id="rId1861"/>
+    <x:hyperlink ref="D886" r:id="rId1862"/>
+    <x:hyperlink ref="D887" r:id="rId1863"/>
+    <x:hyperlink ref="D888" r:id="rId1864"/>
+    <x:hyperlink ref="D889" r:id="rId1865"/>
+    <x:hyperlink ref="D890" r:id="rId1866"/>
+    <x:hyperlink ref="D891" r:id="rId1867"/>
+    <x:hyperlink ref="D892" r:id="rId1868"/>
+    <x:hyperlink ref="D893" r:id="rId1869"/>
+    <x:hyperlink ref="D894" r:id="rId1870"/>
+    <x:hyperlink ref="D895" r:id="rId1871"/>
+    <x:hyperlink ref="D896" r:id="rId1872"/>
+    <x:hyperlink ref="D897" r:id="rId1873"/>
+    <x:hyperlink ref="D898" r:id="rId1874"/>
+    <x:hyperlink ref="D899" r:id="rId1875"/>
+    <x:hyperlink ref="D900" r:id="rId1876"/>
+    <x:hyperlink ref="D901" r:id="rId1877"/>
+    <x:hyperlink ref="D902" r:id="rId1878"/>
+    <x:hyperlink ref="D903" r:id="rId1879"/>
+    <x:hyperlink ref="D904" r:id="rId1880"/>
+    <x:hyperlink ref="D905" r:id="rId1881"/>
+    <x:hyperlink ref="D906" r:id="rId1882"/>
+    <x:hyperlink ref="D907" r:id="rId1883"/>
+    <x:hyperlink ref="D908" r:id="rId1884"/>
+    <x:hyperlink ref="D909" r:id="rId1885"/>
+    <x:hyperlink ref="D910" r:id="rId1886"/>
+    <x:hyperlink ref="D911" r:id="rId1887"/>
+    <x:hyperlink ref="D912" r:id="rId1888"/>
+    <x:hyperlink ref="D913" r:id="rId1889"/>
+    <x:hyperlink ref="D914" r:id="rId1890"/>
+    <x:hyperlink ref="D915" r:id="rId1891"/>
+    <x:hyperlink ref="D916" r:id="rId1892"/>
+    <x:hyperlink ref="D917" r:id="rId1893"/>
+    <x:hyperlink ref="D918" r:id="rId1894"/>
+    <x:hyperlink ref="D919" r:id="rId1895"/>
+    <x:hyperlink ref="D920" r:id="rId1896"/>
+    <x:hyperlink ref="D921" r:id="rId1897"/>
+    <x:hyperlink ref="D922" r:id="rId1898"/>
+    <x:hyperlink ref="D923" r:id="rId1899"/>
+    <x:hyperlink ref="D924" r:id="rId1900"/>
+    <x:hyperlink ref="D925" r:id="rId1901"/>
+    <x:hyperlink ref="D926" r:id="rId1902"/>
+    <x:hyperlink ref="D927" r:id="rId1903"/>
+    <x:hyperlink ref="D928" r:id="rId1904"/>
+    <x:hyperlink ref="D929" r:id="rId1905"/>
+    <x:hyperlink ref="D930" r:id="rId1906"/>
+    <x:hyperlink ref="D931" r:id="rId1907"/>
+    <x:hyperlink ref="D932" r:id="rId1908"/>
+    <x:hyperlink ref="D933" r:id="rId1909"/>
+    <x:hyperlink ref="D934" r:id="rId1910"/>
+    <x:hyperlink ref="D935" r:id="rId1911"/>
+    <x:hyperlink ref="D936" r:id="rId1912"/>
+    <x:hyperlink ref="D937" r:id="rId1913"/>
+    <x:hyperlink ref="D938" r:id="rId1914"/>
+    <x:hyperlink ref="D939" r:id="rId1915"/>
+    <x:hyperlink ref="D940" r:id="rId1916"/>
+    <x:hyperlink ref="D941" r:id="rId1917"/>
+    <x:hyperlink ref="D942" r:id="rId1918"/>
+    <x:hyperlink ref="D943" r:id="rId1919"/>
+    <x:hyperlink ref="D944" r:id="rId1920"/>
+    <x:hyperlink ref="D945" r:id="rId1921"/>
+    <x:hyperlink ref="D946" r:id="rId1922"/>
+    <x:hyperlink ref="D947" r:id="rId1923"/>
+    <x:hyperlink ref="D948" r:id="rId1924"/>
+    <x:hyperlink ref="D949" r:id="rId1925"/>
+    <x:hyperlink ref="D950" r:id="rId1926"/>
+    <x:hyperlink ref="D951" r:id="rId1927"/>
+    <x:hyperlink ref="D952" r:id="rId1928"/>
+    <x:hyperlink ref="D953" r:id="rId1929"/>
+    <x:hyperlink ref="D954" r:id="rId1930"/>
+    <x:hyperlink ref="D955" r:id="rId1931"/>
+    <x:hyperlink ref="D956" r:id="rId1932"/>
+    <x:hyperlink ref="D957" r:id="rId1933"/>
+    <x:hyperlink ref="D958" r:id="rId1934"/>
+    <x:hyperlink ref="D959" r:id="rId1935"/>
+    <x:hyperlink ref="D960" r:id="rId1936"/>
+    <x:hyperlink ref="D961" r:id="rId1937"/>
+    <x:hyperlink ref="D962" r:id="rId1938"/>
+    <x:hyperlink ref="D963" r:id="rId1939"/>
+    <x:hyperlink ref="D964" r:id="rId1940"/>
+    <x:hyperlink ref="D965" r:id="rId1941"/>
+    <x:hyperlink ref="D966" r:id="rId1942"/>
+    <x:hyperlink ref="D967" r:id="rId1943"/>
+    <x:hyperlink ref="D968" r:id="rId1944"/>
+    <x:hyperlink ref="D969" r:id="rId1945"/>
+    <x:hyperlink ref="D970" r:id="rId1946"/>
+    <x:hyperlink ref="D971" r:id="rId1947"/>
+    <x:hyperlink ref="D972" r:id="rId1948"/>
+    <x:hyperlink ref="D973" r:id="rId1949"/>
+    <x:hyperlink ref="D974" r:id="rId1950"/>
+    <x:hyperlink ref="D975" r:id="rId1951"/>
+    <x:hyperlink ref="D976" r:id="rId1952"/>
+    <x:hyperlink ref="D977" r:id="rId1953"/>
+    <x:hyperlink ref="D978" r:id="rId1954"/>
+    <x:hyperlink ref="D979" r:id="rId1955"/>
   </x:hyperlinks>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
   <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
   <x:headerFooter/>
   <x:tableParts count="1">
-    <x:tablePart r:id="rId977"/>
+    <x:tablePart r:id="rId981"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
chore: actualiza dashboard 2026-06-04T08:14Z
</commit_message>
<xml_diff>
--- a/INFORME EXCESOS DE VELOCIDAD.xlsx
+++ b/INFORME EXCESOS DE VELOCIDAD.xlsx
@@ -4096,6 +4096,114 @@
   </x:si>
   <x:si>
     <x:t>-33.699609,-70.800395</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026/06/03 22:58:54</x:t>
+  </x:si>
+  <x:si>
+    <x:t>-33.693877,-70.791349</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026/06/03 22:59:00</x:t>
+  </x:si>
+  <x:si>
+    <x:t>-33.693405,-70.791771</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026/06/03 22:59:19</x:t>
+  </x:si>
+  <x:si>
+    <x:t>-33.691905,-70.790878</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026/06/03 22:59:24</x:t>
+  </x:si>
+  <x:si>
+    <x:t>-33.691454,-70.790635</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026/06/03 22:59:49</x:t>
+  </x:si>
+  <x:si>
+    <x:t>-33.689794,-70.790306</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026/06/03 22:59:52</x:t>
+  </x:si>
+  <x:si>
+    <x:t>-33.689662,-70.789984</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026/06/03 23:01:45</x:t>
+  </x:si>
+  <x:si>
+    <x:t>-33.6819,-70.788021</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026/06/03 23:01:50</x:t>
+  </x:si>
+  <x:si>
+    <x:t>-33.681563,-70.787588</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026/06/03 23:02:29</x:t>
+  </x:si>
+  <x:si>
+    <x:t>-33.680393,-70.783983</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026/06/03 23:02:35</x:t>
+  </x:si>
+  <x:si>
+    <x:t>-33.680381,-70.783272</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026/06/03 23:09:57</x:t>
+  </x:si>
+  <x:si>
+    <x:t>-33.677152,-70.780578</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026/06/03 23:10:03</x:t>
+  </x:si>
+  <x:si>
+    <x:t>-33.677173,-70.781298</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026/06/03 23:10:32</x:t>
+  </x:si>
+  <x:si>
+    <x:t>-33.678428,-70.782857</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026/06/03 23:10:40</x:t>
+  </x:si>
+  <x:si>
+    <x:t>-33.679226,-70.782692</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026/06/03 23:22:06</x:t>
+  </x:si>
+  <x:si>
+    <x:t>-33.700046,-70.801622</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026/06/03 23:22:14</x:t>
+  </x:si>
+  <x:si>
+    <x:t>-33.700017,-70.802128</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026/06/03 23:22:23</x:t>
+  </x:si>
+  <x:si>
+    <x:t>-33.699731,-70.802406</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026/06/03 23:22:33</x:t>
+  </x:si>
+  <x:si>
+    <x:t>-33.699418,-70.801932</x:t>
   </x:si>
   <x:si>
     <x:t>Fecha</x:t>
@@ -4284,8 +4392,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="SpeedingByUnitsFleetsDetailTable_1" displayName="SpeedingByUnitsFleetsDetailTable_1" ref="A5:O337" totalsRowShown="0">
-  <x:autoFilter ref="A5:O337"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="SpeedingByUnitsFleetsDetailTable_1" displayName="SpeedingByUnitsFleetsDetailTable_1" ref="A5:O346" totalsRowShown="0">
+  <x:autoFilter ref="A5:O346"/>
   <x:tableColumns count="15">
     <x:tableColumn id="1" name="Alias"/>
     <x:tableColumn id="2" name="Conductor"/>
@@ -4308,8 +4416,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SpeedingByUnitsFleetsDataTable_1" displayName="SpeedingByUnitsFleetsDataTable_1" ref="A5:H672" totalsRowShown="0">
-  <x:autoFilter ref="A5:H672"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SpeedingByUnitsFleetsDataTable_1" displayName="SpeedingByUnitsFleetsDataTable_1" ref="A5:H690" totalsRowShown="0">
+  <x:autoFilter ref="A5:H690"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="Alias"/>
     <x:tableColumn id="2" name="Secuencial" dataDxfId="0"/>
@@ -4721,22 +4829,22 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="B7" s="4">
-        <x:v>197</x:v>
+        <x:v>206</x:v>
       </x:c>
       <x:c r="C7" s="5">
-        <x:v>0.0208564814814815</x:v>
+        <x:v>0.0215162037037037</x:v>
       </x:c>
       <x:c r="D7" s="5">
-        <x:v>0.00010587046412037</x:v>
+        <x:v>0.000104447590277778</x:v>
       </x:c>
       <x:c r="E7" s="4">
-        <x:v>14.4</x:v>
+        <x:v>15.2</x:v>
       </x:c>
       <x:c r="F7" s="4">
         <x:v>59.6</x:v>
       </x:c>
       <x:c r="G7" s="4">
-        <x:v>25.9</x:v>
+        <x:v>26.3</x:v>
       </x:c>
       <x:c r="H7" s="4">
         <x:v>0</x:v>
@@ -4766,7 +4874,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:O337"/>
+  <x:dimension ref="A1:O346"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="30.710625" style="0" customWidth="1"/>
@@ -20483,6 +20591,429 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="O337" s="4">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="338" spans="1:15">
+      <x:c r="A338" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B338" s="0" t="s">
+        <x:v>572</x:v>
+      </x:c>
+      <x:c r="C338" s="4">
+        <x:v>466</x:v>
+      </x:c>
+      <x:c r="D338" s="4" t="s">
+        <x:v>1360</x:v>
+      </x:c>
+      <x:c r="E338" s="6" t="s">
+        <x:v>1361</x:v>
+      </x:c>
+      <x:c r="F338" s="4" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="G338" s="4" t="s">
+        <x:v>1362</x:v>
+      </x:c>
+      <x:c r="H338" s="6" t="s">
+        <x:v>1363</x:v>
+      </x:c>
+      <x:c r="I338" s="4" t="s">
+        <x:v>77</x:v>
+      </x:c>
+      <x:c r="J338" s="5">
+        <x:v>6.94444444444444E-05</x:v>
+      </x:c>
+      <x:c r="K338" s="4">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="L338" s="4">
+        <x:v>43.2</x:v>
+      </x:c>
+      <x:c r="M338" s="4">
+        <x:v>39.6</x:v>
+      </x:c>
+      <x:c r="N338" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O338" s="4">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="339" spans="1:15">
+      <x:c r="A339" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B339" s="0" t="s">
+        <x:v>572</x:v>
+      </x:c>
+      <x:c r="C339" s="4">
+        <x:v>467</x:v>
+      </x:c>
+      <x:c r="D339" s="4" t="s">
+        <x:v>1364</x:v>
+      </x:c>
+      <x:c r="E339" s="6" t="s">
+        <x:v>1365</x:v>
+      </x:c>
+      <x:c r="F339" s="4" t="s">
+        <x:v>77</x:v>
+      </x:c>
+      <x:c r="G339" s="4" t="s">
+        <x:v>1366</x:v>
+      </x:c>
+      <x:c r="H339" s="6" t="s">
+        <x:v>1367</x:v>
+      </x:c>
+      <x:c r="I339" s="4" t="s">
+        <x:v>77</x:v>
+      </x:c>
+      <x:c r="J339" s="5">
+        <x:v>5.78703703703704E-05</x:v>
+      </x:c>
+      <x:c r="K339" s="4">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="L339" s="4">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="M339" s="4">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="N339" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O339" s="4">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="340" spans="1:15">
+      <x:c r="A340" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B340" s="0" t="s">
+        <x:v>572</x:v>
+      </x:c>
+      <x:c r="C340" s="4">
+        <x:v>468</x:v>
+      </x:c>
+      <x:c r="D340" s="4" t="s">
+        <x:v>1368</x:v>
+      </x:c>
+      <x:c r="E340" s="6" t="s">
+        <x:v>1369</x:v>
+      </x:c>
+      <x:c r="F340" s="4" t="s">
+        <x:v>77</x:v>
+      </x:c>
+      <x:c r="G340" s="4" t="s">
+        <x:v>1370</x:v>
+      </x:c>
+      <x:c r="H340" s="6" t="s">
+        <x:v>1371</x:v>
+      </x:c>
+      <x:c r="I340" s="4" t="s">
+        <x:v>77</x:v>
+      </x:c>
+      <x:c r="J340" s="5">
+        <x:v>3.47222222222222E-05</x:v>
+      </x:c>
+      <x:c r="K340" s="4" t="s">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="L340" s="4">
+        <x:v>40.5</x:v>
+      </x:c>
+      <x:c r="M340" s="4">
+        <x:v>39.6</x:v>
+      </x:c>
+      <x:c r="N340" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O340" s="4">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="341" spans="1:15">
+      <x:c r="A341" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B341" s="0" t="s">
+        <x:v>572</x:v>
+      </x:c>
+      <x:c r="C341" s="4">
+        <x:v>469</x:v>
+      </x:c>
+      <x:c r="D341" s="4" t="s">
+        <x:v>1372</x:v>
+      </x:c>
+      <x:c r="E341" s="6" t="s">
+        <x:v>1373</x:v>
+      </x:c>
+      <x:c r="F341" s="4" t="s">
+        <x:v>77</x:v>
+      </x:c>
+      <x:c r="G341" s="4" t="s">
+        <x:v>1374</x:v>
+      </x:c>
+      <x:c r="H341" s="6" t="s">
+        <x:v>1375</x:v>
+      </x:c>
+      <x:c r="I341" s="4" t="s">
+        <x:v>77</x:v>
+      </x:c>
+      <x:c r="J341" s="5">
+        <x:v>5.78703703703704E-05</x:v>
+      </x:c>
+      <x:c r="K341" s="4">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="L341" s="4">
+        <x:v>40.2</x:v>
+      </x:c>
+      <x:c r="M341" s="4">
+        <x:v>39.2</x:v>
+      </x:c>
+      <x:c r="N341" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O341" s="4">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="342" spans="1:15">
+      <x:c r="A342" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B342" s="0" t="s">
+        <x:v>572</x:v>
+      </x:c>
+      <x:c r="C342" s="4">
+        <x:v>470</x:v>
+      </x:c>
+      <x:c r="D342" s="4" t="s">
+        <x:v>1376</x:v>
+      </x:c>
+      <x:c r="E342" s="6" t="s">
+        <x:v>1377</x:v>
+      </x:c>
+      <x:c r="F342" s="4" t="s">
+        <x:v>77</x:v>
+      </x:c>
+      <x:c r="G342" s="4" t="s">
+        <x:v>1378</x:v>
+      </x:c>
+      <x:c r="H342" s="6" t="s">
+        <x:v>1379</x:v>
+      </x:c>
+      <x:c r="I342" s="4" t="s">
+        <x:v>77</x:v>
+      </x:c>
+      <x:c r="J342" s="5">
+        <x:v>6.94444444444444E-05</x:v>
+      </x:c>
+      <x:c r="K342" s="4">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="L342" s="4">
+        <x:v>41.7</x:v>
+      </x:c>
+      <x:c r="M342" s="4">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="N342" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O342" s="4">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="343" spans="1:15">
+      <x:c r="A343" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B343" s="0" t="s">
+        <x:v>572</x:v>
+      </x:c>
+      <x:c r="C343" s="4">
+        <x:v>471</x:v>
+      </x:c>
+      <x:c r="D343" s="4" t="s">
+        <x:v>1380</x:v>
+      </x:c>
+      <x:c r="E343" s="6" t="s">
+        <x:v>1381</x:v>
+      </x:c>
+      <x:c r="F343" s="4" t="s">
+        <x:v>77</x:v>
+      </x:c>
+      <x:c r="G343" s="4" t="s">
+        <x:v>1382</x:v>
+      </x:c>
+      <x:c r="H343" s="6" t="s">
+        <x:v>1383</x:v>
+      </x:c>
+      <x:c r="I343" s="4" t="s">
+        <x:v>563</x:v>
+      </x:c>
+      <x:c r="J343" s="5">
+        <x:v>6.94444444444444E-05</x:v>
+      </x:c>
+      <x:c r="K343" s="4">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="L343" s="4">
+        <x:v>40.7</x:v>
+      </x:c>
+      <x:c r="M343" s="4">
+        <x:v>39.6</x:v>
+      </x:c>
+      <x:c r="N343" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O343" s="4">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="344" spans="1:15">
+      <x:c r="A344" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B344" s="0" t="s">
+        <x:v>572</x:v>
+      </x:c>
+      <x:c r="C344" s="4">
+        <x:v>472</x:v>
+      </x:c>
+      <x:c r="D344" s="4" t="s">
+        <x:v>1384</x:v>
+      </x:c>
+      <x:c r="E344" s="6" t="s">
+        <x:v>1385</x:v>
+      </x:c>
+      <x:c r="F344" s="4" t="s">
+        <x:v>563</x:v>
+      </x:c>
+      <x:c r="G344" s="4" t="s">
+        <x:v>1386</x:v>
+      </x:c>
+      <x:c r="H344" s="6" t="s">
+        <x:v>1387</x:v>
+      </x:c>
+      <x:c r="I344" s="4" t="s">
+        <x:v>77</x:v>
+      </x:c>
+      <x:c r="J344" s="5">
+        <x:v>9.25925925925926E-05</x:v>
+      </x:c>
+      <x:c r="K344" s="4">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="L344" s="4">
+        <x:v>41.4</x:v>
+      </x:c>
+      <x:c r="M344" s="4">
+        <x:v>39.7</x:v>
+      </x:c>
+      <x:c r="N344" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O344" s="4">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="345" spans="1:15">
+      <x:c r="A345" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B345" s="0" t="s">
+        <x:v>572</x:v>
+      </x:c>
+      <x:c r="C345" s="4">
+        <x:v>474</x:v>
+      </x:c>
+      <x:c r="D345" s="4" t="s">
+        <x:v>1388</x:v>
+      </x:c>
+      <x:c r="E345" s="6" t="s">
+        <x:v>1389</x:v>
+      </x:c>
+      <x:c r="F345" s="4" t="s">
+        <x:v>77</x:v>
+      </x:c>
+      <x:c r="G345" s="4" t="s">
+        <x:v>1390</x:v>
+      </x:c>
+      <x:c r="H345" s="6" t="s">
+        <x:v>1391</x:v>
+      </x:c>
+      <x:c r="I345" s="4" t="s">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="J345" s="5">
+        <x:v>9.25925925925926E-05</x:v>
+      </x:c>
+      <x:c r="K345" s="4">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="L345" s="4">
+        <x:v>23.1</x:v>
+      </x:c>
+      <x:c r="M345" s="4">
+        <x:v>19.7</x:v>
+      </x:c>
+      <x:c r="N345" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O345" s="4">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="346" spans="1:15">
+      <x:c r="A346" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B346" s="0" t="s">
+        <x:v>572</x:v>
+      </x:c>
+      <x:c r="C346" s="4">
+        <x:v>475</x:v>
+      </x:c>
+      <x:c r="D346" s="4" t="s">
+        <x:v>1392</x:v>
+      </x:c>
+      <x:c r="E346" s="6" t="s">
+        <x:v>1393</x:v>
+      </x:c>
+      <x:c r="F346" s="4" t="s">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="G346" s="4" t="s">
+        <x:v>1394</x:v>
+      </x:c>
+      <x:c r="H346" s="6" t="s">
+        <x:v>1395</x:v>
+      </x:c>
+      <x:c r="I346" s="4" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="J346" s="5">
+        <x:v>0.000115740740740741</x:v>
+      </x:c>
+      <x:c r="K346" s="4">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="L346" s="4">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="M346" s="4">
+        <x:v>19.3</x:v>
+      </x:c>
+      <x:c r="N346" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O346" s="4">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -21157,6 +21688,24 @@
     <x:hyperlink ref="H336" r:id="rId670"/>
     <x:hyperlink ref="E337" r:id="rId671"/>
     <x:hyperlink ref="H337" r:id="rId672"/>
+    <x:hyperlink ref="E338" r:id="rId673"/>
+    <x:hyperlink ref="H338" r:id="rId674"/>
+    <x:hyperlink ref="E339" r:id="rId675"/>
+    <x:hyperlink ref="H339" r:id="rId676"/>
+    <x:hyperlink ref="E340" r:id="rId677"/>
+    <x:hyperlink ref="H340" r:id="rId678"/>
+    <x:hyperlink ref="E341" r:id="rId679"/>
+    <x:hyperlink ref="H341" r:id="rId680"/>
+    <x:hyperlink ref="E342" r:id="rId681"/>
+    <x:hyperlink ref="H342" r:id="rId682"/>
+    <x:hyperlink ref="E343" r:id="rId683"/>
+    <x:hyperlink ref="H343" r:id="rId684"/>
+    <x:hyperlink ref="E344" r:id="rId685"/>
+    <x:hyperlink ref="H344" r:id="rId686"/>
+    <x:hyperlink ref="E345" r:id="rId687"/>
+    <x:hyperlink ref="H345" r:id="rId688"/>
+    <x:hyperlink ref="E346" r:id="rId689"/>
+    <x:hyperlink ref="H346" r:id="rId690"/>
   </x:hyperlinks>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
@@ -21173,7 +21722,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:H672"/>
+  <x:dimension ref="A1:H690"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="30.710625" style="0" customWidth="1"/>
@@ -21226,22 +21775,22 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="C5" s="3" t="s">
-        <x:v>1360</x:v>
+        <x:v>1396</x:v>
       </x:c>
       <x:c r="D5" s="3" t="s">
-        <x:v>1361</x:v>
+        <x:v>1397</x:v>
       </x:c>
       <x:c r="E5" s="3" t="s">
-        <x:v>1362</x:v>
+        <x:v>1398</x:v>
       </x:c>
       <x:c r="F5" s="3" t="s">
-        <x:v>1363</x:v>
+        <x:v>1399</x:v>
       </x:c>
       <x:c r="G5" s="3" t="s">
-        <x:v>1364</x:v>
+        <x:v>1400</x:v>
       </x:c>
       <x:c r="H5" s="3" t="s">
-        <x:v>1365</x:v>
+        <x:v>1401</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:8">
@@ -25204,10 +25753,10 @@
         <x:v>123</x:v>
       </x:c>
       <x:c r="C158" s="4" t="s">
-        <x:v>1366</x:v>
+        <x:v>1402</x:v>
       </x:c>
       <x:c r="D158" s="6" t="s">
-        <x:v>1367</x:v>
+        <x:v>1403</x:v>
       </x:c>
       <x:c r="E158" s="4" t="s">
         <x:v>27</x:v>
@@ -28662,10 +29211,10 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="C291" s="4" t="s">
-        <x:v>1368</x:v>
+        <x:v>1404</x:v>
       </x:c>
       <x:c r="D291" s="6" t="s">
-        <x:v>1369</x:v>
+        <x:v>1405</x:v>
       </x:c>
       <x:c r="E291" s="4" t="s">
         <x:v>35</x:v>
@@ -38584,6 +39133,474 @@
       </x:c>
       <x:c r="H672" s="4">
         <x:v>566.4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="673" spans="1:8">
+      <x:c r="A673" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B673" s="4">
+        <x:v>466</x:v>
+      </x:c>
+      <x:c r="C673" s="4" t="s">
+        <x:v>1360</x:v>
+      </x:c>
+      <x:c r="D673" s="6" t="s">
+        <x:v>1361</x:v>
+      </x:c>
+      <x:c r="E673" s="4" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="F673" s="4">
+        <x:v>43.2</x:v>
+      </x:c>
+      <x:c r="G673" s="4">
+        <x:v>5338.2</x:v>
+      </x:c>
+      <x:c r="H673" s="4">
+        <x:v>673.3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="674" spans="1:8">
+      <x:c r="A674" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B674" s="4">
+        <x:v>466</x:v>
+      </x:c>
+      <x:c r="C674" s="4" t="s">
+        <x:v>1362</x:v>
+      </x:c>
+      <x:c r="D674" s="6" t="s">
+        <x:v>1363</x:v>
+      </x:c>
+      <x:c r="E674" s="4" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="F674" s="4">
+        <x:v>35.9</x:v>
+      </x:c>
+      <x:c r="G674" s="4">
+        <x:v>5338.3</x:v>
+      </x:c>
+      <x:c r="H674" s="4">
+        <x:v>667.4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="675" spans="1:8">
+      <x:c r="A675" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B675" s="4">
+        <x:v>467</x:v>
+      </x:c>
+      <x:c r="C675" s="4" t="s">
+        <x:v>1364</x:v>
+      </x:c>
+      <x:c r="D675" s="6" t="s">
+        <x:v>1365</x:v>
+      </x:c>
+      <x:c r="E675" s="4" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="F675" s="4">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="G675" s="4">
+        <x:v>5338.4</x:v>
+      </x:c>
+      <x:c r="H675" s="4">
+        <x:v>650.4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="676" spans="1:8">
+      <x:c r="A676" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B676" s="4">
+        <x:v>467</x:v>
+      </x:c>
+      <x:c r="C676" s="4" t="s">
+        <x:v>1366</x:v>
+      </x:c>
+      <x:c r="D676" s="6" t="s">
+        <x:v>1367</x:v>
+      </x:c>
+      <x:c r="E676" s="4" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="F676" s="4">
+        <x:v>36.9</x:v>
+      </x:c>
+      <x:c r="G676" s="4">
+        <x:v>5338.5</x:v>
+      </x:c>
+      <x:c r="H676" s="4">
+        <x:v>645</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="677" spans="1:8">
+      <x:c r="A677" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B677" s="4">
+        <x:v>468</x:v>
+      </x:c>
+      <x:c r="C677" s="4" t="s">
+        <x:v>1368</x:v>
+      </x:c>
+      <x:c r="D677" s="6" t="s">
+        <x:v>1369</x:v>
+      </x:c>
+      <x:c r="E677" s="4" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="F677" s="4">
+        <x:v>40.5</x:v>
+      </x:c>
+      <x:c r="G677" s="4">
+        <x:v>5338.8</x:v>
+      </x:c>
+      <x:c r="H677" s="4">
+        <x:v>629.7</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="678" spans="1:8">
+      <x:c r="A678" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B678" s="4">
+        <x:v>468</x:v>
+      </x:c>
+      <x:c r="C678" s="4" t="s">
+        <x:v>1370</x:v>
+      </x:c>
+      <x:c r="D678" s="6" t="s">
+        <x:v>1371</x:v>
+      </x:c>
+      <x:c r="E678" s="4" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="F678" s="4">
+        <x:v>38.6</x:v>
+      </x:c>
+      <x:c r="G678" s="4">
+        <x:v>5338.8</x:v>
+      </x:c>
+      <x:c r="H678" s="4">
+        <x:v>629.2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="679" spans="1:8">
+      <x:c r="A679" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B679" s="4">
+        <x:v>469</x:v>
+      </x:c>
+      <x:c r="C679" s="4" t="s">
+        <x:v>1372</x:v>
+      </x:c>
+      <x:c r="D679" s="6" t="s">
+        <x:v>1373</x:v>
+      </x:c>
+      <x:c r="E679" s="4" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="F679" s="4">
+        <x:v>40.2</x:v>
+      </x:c>
+      <x:c r="G679" s="4">
+        <x:v>5339.9</x:v>
+      </x:c>
+      <x:c r="H679" s="4">
+        <x:v>541.6</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="680" spans="1:8">
+      <x:c r="A680" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B680" s="4">
+        <x:v>469</x:v>
+      </x:c>
+      <x:c r="C680" s="4" t="s">
+        <x:v>1374</x:v>
+      </x:c>
+      <x:c r="D680" s="6" t="s">
+        <x:v>1375</x:v>
+      </x:c>
+      <x:c r="E680" s="4" t="s">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="F680" s="4">
+        <x:v>38.1</x:v>
+      </x:c>
+      <x:c r="G680" s="4">
+        <x:v>5340</x:v>
+      </x:c>
+      <x:c r="H680" s="4">
+        <x:v>535.4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="681" spans="1:8">
+      <x:c r="A681" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B681" s="4">
+        <x:v>470</x:v>
+      </x:c>
+      <x:c r="C681" s="4" t="s">
+        <x:v>1376</x:v>
+      </x:c>
+      <x:c r="D681" s="6" t="s">
+        <x:v>1377</x:v>
+      </x:c>
+      <x:c r="E681" s="4" t="s">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="F681" s="4">
+        <x:v>41.7</x:v>
+      </x:c>
+      <x:c r="G681" s="4">
+        <x:v>5340.3</x:v>
+      </x:c>
+      <x:c r="H681" s="4">
+        <x:v>507.7</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="682" spans="1:8">
+      <x:c r="A682" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B682" s="4">
+        <x:v>470</x:v>
+      </x:c>
+      <x:c r="C682" s="4" t="s">
+        <x:v>1378</x:v>
+      </x:c>
+      <x:c r="D682" s="6" t="s">
+        <x:v>1379</x:v>
+      </x:c>
+      <x:c r="E682" s="4" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="F682" s="4">
+        <x:v>36.2</x:v>
+      </x:c>
+      <x:c r="G682" s="4">
+        <x:v>5340.4</x:v>
+      </x:c>
+      <x:c r="H682" s="4">
+        <x:v>500.9</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="683" spans="1:8">
+      <x:c r="A683" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B683" s="4">
+        <x:v>471</x:v>
+      </x:c>
+      <x:c r="C683" s="4" t="s">
+        <x:v>1380</x:v>
+      </x:c>
+      <x:c r="D683" s="6" t="s">
+        <x:v>1381</x:v>
+      </x:c>
+      <x:c r="E683" s="4" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="F683" s="4">
+        <x:v>40.7</x:v>
+      </x:c>
+      <x:c r="G683" s="4">
+        <x:v>5343.7</x:v>
+      </x:c>
+      <x:c r="H683" s="4">
+        <x:v>482.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="684" spans="1:8">
+      <x:c r="A684" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B684" s="4">
+        <x:v>471</x:v>
+      </x:c>
+      <x:c r="C684" s="4" t="s">
+        <x:v>1382</x:v>
+      </x:c>
+      <x:c r="D684" s="6" t="s">
+        <x:v>1383</x:v>
+      </x:c>
+      <x:c r="E684" s="4" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="F684" s="4">
+        <x:v>38.5</x:v>
+      </x:c>
+      <x:c r="G684" s="4">
+        <x:v>5343.8</x:v>
+      </x:c>
+      <x:c r="H684" s="4">
+        <x:v>482.4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="685" spans="1:8">
+      <x:c r="A685" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B685" s="4">
+        <x:v>472</x:v>
+      </x:c>
+      <x:c r="C685" s="4" t="s">
+        <x:v>1384</x:v>
+      </x:c>
+      <x:c r="D685" s="6" t="s">
+        <x:v>1385</x:v>
+      </x:c>
+      <x:c r="E685" s="4" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="F685" s="4">
+        <x:v>41.4</x:v>
+      </x:c>
+      <x:c r="G685" s="4">
+        <x:v>5344.1</x:v>
+      </x:c>
+      <x:c r="H685" s="4">
+        <x:v>487.1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="686" spans="1:8">
+      <x:c r="A686" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B686" s="4">
+        <x:v>472</x:v>
+      </x:c>
+      <x:c r="C686" s="4" t="s">
+        <x:v>1386</x:v>
+      </x:c>
+      <x:c r="D686" s="6" t="s">
+        <x:v>1387</x:v>
+      </x:c>
+      <x:c r="E686" s="4" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="F686" s="4">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="G686" s="4">
+        <x:v>5344.2</x:v>
+      </x:c>
+      <x:c r="H686" s="4">
+        <x:v>492.3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="687" spans="1:8">
+      <x:c r="A687" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B687" s="4">
+        <x:v>474</x:v>
+      </x:c>
+      <x:c r="C687" s="4" t="s">
+        <x:v>1388</x:v>
+      </x:c>
+      <x:c r="D687" s="6" t="s">
+        <x:v>1389</x:v>
+      </x:c>
+      <x:c r="E687" s="4" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="F687" s="4">
+        <x:v>23.1</x:v>
+      </x:c>
+      <x:c r="G687" s="4">
+        <x:v>5349.1</x:v>
+      </x:c>
+      <x:c r="H687" s="4">
+        <x:v>550.7</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="688" spans="1:8">
+      <x:c r="A688" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B688" s="4">
+        <x:v>474</x:v>
+      </x:c>
+      <x:c r="C688" s="4" t="s">
+        <x:v>1390</x:v>
+      </x:c>
+      <x:c r="D688" s="6" t="s">
+        <x:v>1391</x:v>
+      </x:c>
+      <x:c r="E688" s="4" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="F688" s="4">
+        <x:v>16.3</x:v>
+      </x:c>
+      <x:c r="G688" s="4">
+        <x:v>5349.2</x:v>
+      </x:c>
+      <x:c r="H688" s="4">
+        <x:v>546.3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="689" spans="1:8">
+      <x:c r="A689" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B689" s="4">
+        <x:v>475</x:v>
+      </x:c>
+      <x:c r="C689" s="4" t="s">
+        <x:v>1392</x:v>
+      </x:c>
+      <x:c r="D689" s="6" t="s">
+        <x:v>1393</x:v>
+      </x:c>
+      <x:c r="E689" s="4" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="F689" s="4">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="G689" s="4">
+        <x:v>5349.2</x:v>
+      </x:c>
+      <x:c r="H689" s="4">
+        <x:v>542.6</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="690" spans="1:8">
+      <x:c r="A690" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B690" s="4">
+        <x:v>475</x:v>
+      </x:c>
+      <x:c r="C690" s="4" t="s">
+        <x:v>1394</x:v>
+      </x:c>
+      <x:c r="D690" s="6" t="s">
+        <x:v>1395</x:v>
+      </x:c>
+      <x:c r="E690" s="4" t="s">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="F690" s="4">
+        <x:v>17.5</x:v>
+      </x:c>
+      <x:c r="G690" s="4">
+        <x:v>5349.3</x:v>
+      </x:c>
+      <x:c r="H690" s="4">
+        <x:v>539.6</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -38593,680 +39610,698 @@
     <x:mergeCell ref="A3:H3"/>
   </x:mergeCells>
   <x:hyperlinks>
-    <x:hyperlink ref="D6" r:id="rId674"/>
-    <x:hyperlink ref="D7" r:id="rId675"/>
-    <x:hyperlink ref="D8" r:id="rId676"/>
-    <x:hyperlink ref="D9" r:id="rId677"/>
-    <x:hyperlink ref="D10" r:id="rId678"/>
-    <x:hyperlink ref="D11" r:id="rId679"/>
-    <x:hyperlink ref="D12" r:id="rId680"/>
-    <x:hyperlink ref="D13" r:id="rId681"/>
-    <x:hyperlink ref="D14" r:id="rId682"/>
-    <x:hyperlink ref="D15" r:id="rId683"/>
-    <x:hyperlink ref="D16" r:id="rId684"/>
-    <x:hyperlink ref="D17" r:id="rId685"/>
-    <x:hyperlink ref="D18" r:id="rId686"/>
-    <x:hyperlink ref="D19" r:id="rId687"/>
-    <x:hyperlink ref="D20" r:id="rId688"/>
-    <x:hyperlink ref="D21" r:id="rId689"/>
-    <x:hyperlink ref="D22" r:id="rId690"/>
-    <x:hyperlink ref="D23" r:id="rId691"/>
-    <x:hyperlink ref="D24" r:id="rId692"/>
-    <x:hyperlink ref="D25" r:id="rId693"/>
-    <x:hyperlink ref="D26" r:id="rId694"/>
-    <x:hyperlink ref="D27" r:id="rId695"/>
-    <x:hyperlink ref="D28" r:id="rId696"/>
-    <x:hyperlink ref="D29" r:id="rId697"/>
-    <x:hyperlink ref="D30" r:id="rId698"/>
-    <x:hyperlink ref="D31" r:id="rId699"/>
-    <x:hyperlink ref="D32" r:id="rId700"/>
-    <x:hyperlink ref="D33" r:id="rId701"/>
-    <x:hyperlink ref="D34" r:id="rId702"/>
-    <x:hyperlink ref="D35" r:id="rId703"/>
-    <x:hyperlink ref="D36" r:id="rId704"/>
-    <x:hyperlink ref="D37" r:id="rId705"/>
-    <x:hyperlink ref="D38" r:id="rId706"/>
-    <x:hyperlink ref="D39" r:id="rId707"/>
-    <x:hyperlink ref="D40" r:id="rId708"/>
-    <x:hyperlink ref="D41" r:id="rId709"/>
-    <x:hyperlink ref="D42" r:id="rId710"/>
-    <x:hyperlink ref="D43" r:id="rId711"/>
-    <x:hyperlink ref="D44" r:id="rId712"/>
-    <x:hyperlink ref="D45" r:id="rId713"/>
-    <x:hyperlink ref="D46" r:id="rId714"/>
-    <x:hyperlink ref="D47" r:id="rId715"/>
-    <x:hyperlink ref="D48" r:id="rId716"/>
-    <x:hyperlink ref="D49" r:id="rId717"/>
-    <x:hyperlink ref="D50" r:id="rId718"/>
-    <x:hyperlink ref="D51" r:id="rId719"/>
-    <x:hyperlink ref="D52" r:id="rId720"/>
-    <x:hyperlink ref="D53" r:id="rId721"/>
-    <x:hyperlink ref="D54" r:id="rId722"/>
-    <x:hyperlink ref="D55" r:id="rId723"/>
-    <x:hyperlink ref="D56" r:id="rId724"/>
-    <x:hyperlink ref="D57" r:id="rId725"/>
-    <x:hyperlink ref="D58" r:id="rId726"/>
-    <x:hyperlink ref="D59" r:id="rId727"/>
-    <x:hyperlink ref="D60" r:id="rId728"/>
-    <x:hyperlink ref="D61" r:id="rId729"/>
-    <x:hyperlink ref="D62" r:id="rId730"/>
-    <x:hyperlink ref="D63" r:id="rId731"/>
-    <x:hyperlink ref="D64" r:id="rId732"/>
-    <x:hyperlink ref="D65" r:id="rId733"/>
-    <x:hyperlink ref="D66" r:id="rId734"/>
-    <x:hyperlink ref="D67" r:id="rId735"/>
-    <x:hyperlink ref="D68" r:id="rId736"/>
-    <x:hyperlink ref="D69" r:id="rId737"/>
-    <x:hyperlink ref="D70" r:id="rId738"/>
-    <x:hyperlink ref="D71" r:id="rId739"/>
-    <x:hyperlink ref="D72" r:id="rId740"/>
-    <x:hyperlink ref="D73" r:id="rId741"/>
-    <x:hyperlink ref="D74" r:id="rId742"/>
-    <x:hyperlink ref="D75" r:id="rId743"/>
-    <x:hyperlink ref="D76" r:id="rId744"/>
-    <x:hyperlink ref="D77" r:id="rId745"/>
-    <x:hyperlink ref="D78" r:id="rId746"/>
-    <x:hyperlink ref="D79" r:id="rId747"/>
-    <x:hyperlink ref="D80" r:id="rId748"/>
-    <x:hyperlink ref="D81" r:id="rId749"/>
-    <x:hyperlink ref="D82" r:id="rId750"/>
-    <x:hyperlink ref="D83" r:id="rId751"/>
-    <x:hyperlink ref="D84" r:id="rId752"/>
-    <x:hyperlink ref="D85" r:id="rId753"/>
-    <x:hyperlink ref="D86" r:id="rId754"/>
-    <x:hyperlink ref="D87" r:id="rId755"/>
-    <x:hyperlink ref="D88" r:id="rId756"/>
-    <x:hyperlink ref="D89" r:id="rId757"/>
-    <x:hyperlink ref="D90" r:id="rId758"/>
-    <x:hyperlink ref="D91" r:id="rId759"/>
-    <x:hyperlink ref="D92" r:id="rId760"/>
-    <x:hyperlink ref="D93" r:id="rId761"/>
-    <x:hyperlink ref="D94" r:id="rId762"/>
-    <x:hyperlink ref="D95" r:id="rId763"/>
-    <x:hyperlink ref="D96" r:id="rId764"/>
-    <x:hyperlink ref="D97" r:id="rId765"/>
-    <x:hyperlink ref="D98" r:id="rId766"/>
-    <x:hyperlink ref="D99" r:id="rId767"/>
-    <x:hyperlink ref="D100" r:id="rId768"/>
-    <x:hyperlink ref="D101" r:id="rId769"/>
-    <x:hyperlink ref="D102" r:id="rId770"/>
-    <x:hyperlink ref="D103" r:id="rId771"/>
-    <x:hyperlink ref="D104" r:id="rId772"/>
-    <x:hyperlink ref="D105" r:id="rId773"/>
-    <x:hyperlink ref="D106" r:id="rId774"/>
-    <x:hyperlink ref="D107" r:id="rId775"/>
-    <x:hyperlink ref="D108" r:id="rId776"/>
-    <x:hyperlink ref="D109" r:id="rId777"/>
-    <x:hyperlink ref="D110" r:id="rId778"/>
-    <x:hyperlink ref="D111" r:id="rId779"/>
-    <x:hyperlink ref="D112" r:id="rId780"/>
-    <x:hyperlink ref="D113" r:id="rId781"/>
-    <x:hyperlink ref="D114" r:id="rId782"/>
-    <x:hyperlink ref="D115" r:id="rId783"/>
-    <x:hyperlink ref="D116" r:id="rId784"/>
-    <x:hyperlink ref="D117" r:id="rId785"/>
-    <x:hyperlink ref="D118" r:id="rId786"/>
-    <x:hyperlink ref="D119" r:id="rId787"/>
-    <x:hyperlink ref="D120" r:id="rId788"/>
-    <x:hyperlink ref="D121" r:id="rId789"/>
-    <x:hyperlink ref="D122" r:id="rId790"/>
-    <x:hyperlink ref="D123" r:id="rId791"/>
-    <x:hyperlink ref="D124" r:id="rId792"/>
-    <x:hyperlink ref="D125" r:id="rId793"/>
-    <x:hyperlink ref="D126" r:id="rId794"/>
-    <x:hyperlink ref="D127" r:id="rId795"/>
-    <x:hyperlink ref="D128" r:id="rId796"/>
-    <x:hyperlink ref="D129" r:id="rId797"/>
-    <x:hyperlink ref="D130" r:id="rId798"/>
-    <x:hyperlink ref="D131" r:id="rId799"/>
-    <x:hyperlink ref="D132" r:id="rId800"/>
-    <x:hyperlink ref="D133" r:id="rId801"/>
-    <x:hyperlink ref="D134" r:id="rId802"/>
-    <x:hyperlink ref="D135" r:id="rId803"/>
-    <x:hyperlink ref="D136" r:id="rId804"/>
-    <x:hyperlink ref="D137" r:id="rId805"/>
-    <x:hyperlink ref="D138" r:id="rId806"/>
-    <x:hyperlink ref="D139" r:id="rId807"/>
-    <x:hyperlink ref="D140" r:id="rId808"/>
-    <x:hyperlink ref="D141" r:id="rId809"/>
-    <x:hyperlink ref="D142" r:id="rId810"/>
-    <x:hyperlink ref="D143" r:id="rId811"/>
-    <x:hyperlink ref="D144" r:id="rId812"/>
-    <x:hyperlink ref="D145" r:id="rId813"/>
-    <x:hyperlink ref="D146" r:id="rId814"/>
-    <x:hyperlink ref="D147" r:id="rId815"/>
-    <x:hyperlink ref="D148" r:id="rId816"/>
-    <x:hyperlink ref="D149" r:id="rId817"/>
-    <x:hyperlink ref="D150" r:id="rId818"/>
-    <x:hyperlink ref="D151" r:id="rId819"/>
-    <x:hyperlink ref="D152" r:id="rId820"/>
-    <x:hyperlink ref="D153" r:id="rId821"/>
-    <x:hyperlink ref="D154" r:id="rId822"/>
-    <x:hyperlink ref="D155" r:id="rId823"/>
-    <x:hyperlink ref="D156" r:id="rId824"/>
-    <x:hyperlink ref="D157" r:id="rId825"/>
-    <x:hyperlink ref="D158" r:id="rId826"/>
-    <x:hyperlink ref="D159" r:id="rId827"/>
-    <x:hyperlink ref="D160" r:id="rId828"/>
-    <x:hyperlink ref="D161" r:id="rId829"/>
-    <x:hyperlink ref="D162" r:id="rId830"/>
-    <x:hyperlink ref="D163" r:id="rId831"/>
-    <x:hyperlink ref="D164" r:id="rId832"/>
-    <x:hyperlink ref="D165" r:id="rId833"/>
-    <x:hyperlink ref="D166" r:id="rId834"/>
-    <x:hyperlink ref="D167" r:id="rId835"/>
-    <x:hyperlink ref="D168" r:id="rId836"/>
-    <x:hyperlink ref="D169" r:id="rId837"/>
-    <x:hyperlink ref="D170" r:id="rId838"/>
-    <x:hyperlink ref="D171" r:id="rId839"/>
-    <x:hyperlink ref="D172" r:id="rId840"/>
-    <x:hyperlink ref="D173" r:id="rId841"/>
-    <x:hyperlink ref="D174" r:id="rId842"/>
-    <x:hyperlink ref="D175" r:id="rId843"/>
-    <x:hyperlink ref="D176" r:id="rId844"/>
-    <x:hyperlink ref="D177" r:id="rId845"/>
-    <x:hyperlink ref="D178" r:id="rId846"/>
-    <x:hyperlink ref="D179" r:id="rId847"/>
-    <x:hyperlink ref="D180" r:id="rId848"/>
-    <x:hyperlink ref="D181" r:id="rId849"/>
-    <x:hyperlink ref="D182" r:id="rId850"/>
-    <x:hyperlink ref="D183" r:id="rId851"/>
-    <x:hyperlink ref="D184" r:id="rId852"/>
-    <x:hyperlink ref="D185" r:id="rId853"/>
-    <x:hyperlink ref="D186" r:id="rId854"/>
-    <x:hyperlink ref="D187" r:id="rId855"/>
-    <x:hyperlink ref="D188" r:id="rId856"/>
-    <x:hyperlink ref="D189" r:id="rId857"/>
-    <x:hyperlink ref="D190" r:id="rId858"/>
-    <x:hyperlink ref="D191" r:id="rId859"/>
-    <x:hyperlink ref="D192" r:id="rId860"/>
-    <x:hyperlink ref="D193" r:id="rId861"/>
-    <x:hyperlink ref="D194" r:id="rId862"/>
-    <x:hyperlink ref="D195" r:id="rId863"/>
-    <x:hyperlink ref="D196" r:id="rId864"/>
-    <x:hyperlink ref="D197" r:id="rId865"/>
-    <x:hyperlink ref="D198" r:id="rId866"/>
-    <x:hyperlink ref="D199" r:id="rId867"/>
-    <x:hyperlink ref="D200" r:id="rId868"/>
-    <x:hyperlink ref="D201" r:id="rId869"/>
-    <x:hyperlink ref="D202" r:id="rId870"/>
-    <x:hyperlink ref="D203" r:id="rId871"/>
-    <x:hyperlink ref="D204" r:id="rId872"/>
-    <x:hyperlink ref="D205" r:id="rId873"/>
-    <x:hyperlink ref="D206" r:id="rId874"/>
-    <x:hyperlink ref="D207" r:id="rId875"/>
-    <x:hyperlink ref="D208" r:id="rId876"/>
-    <x:hyperlink ref="D209" r:id="rId877"/>
-    <x:hyperlink ref="D210" r:id="rId878"/>
-    <x:hyperlink ref="D211" r:id="rId879"/>
-    <x:hyperlink ref="D212" r:id="rId880"/>
-    <x:hyperlink ref="D213" r:id="rId881"/>
-    <x:hyperlink ref="D214" r:id="rId882"/>
-    <x:hyperlink ref="D215" r:id="rId883"/>
-    <x:hyperlink ref="D216" r:id="rId884"/>
-    <x:hyperlink ref="D217" r:id="rId885"/>
-    <x:hyperlink ref="D218" r:id="rId886"/>
-    <x:hyperlink ref="D219" r:id="rId887"/>
-    <x:hyperlink ref="D220" r:id="rId888"/>
-    <x:hyperlink ref="D221" r:id="rId889"/>
-    <x:hyperlink ref="D222" r:id="rId890"/>
-    <x:hyperlink ref="D223" r:id="rId891"/>
-    <x:hyperlink ref="D224" r:id="rId892"/>
-    <x:hyperlink ref="D225" r:id="rId893"/>
-    <x:hyperlink ref="D226" r:id="rId894"/>
-    <x:hyperlink ref="D227" r:id="rId895"/>
-    <x:hyperlink ref="D228" r:id="rId896"/>
-    <x:hyperlink ref="D229" r:id="rId897"/>
-    <x:hyperlink ref="D230" r:id="rId898"/>
-    <x:hyperlink ref="D231" r:id="rId899"/>
-    <x:hyperlink ref="D232" r:id="rId900"/>
-    <x:hyperlink ref="D233" r:id="rId901"/>
-    <x:hyperlink ref="D234" r:id="rId902"/>
-    <x:hyperlink ref="D235" r:id="rId903"/>
-    <x:hyperlink ref="D236" r:id="rId904"/>
-    <x:hyperlink ref="D237" r:id="rId905"/>
-    <x:hyperlink ref="D238" r:id="rId906"/>
-    <x:hyperlink ref="D239" r:id="rId907"/>
-    <x:hyperlink ref="D240" r:id="rId908"/>
-    <x:hyperlink ref="D241" r:id="rId909"/>
-    <x:hyperlink ref="D242" r:id="rId910"/>
-    <x:hyperlink ref="D243" r:id="rId911"/>
-    <x:hyperlink ref="D244" r:id="rId912"/>
-    <x:hyperlink ref="D245" r:id="rId913"/>
-    <x:hyperlink ref="D246" r:id="rId914"/>
-    <x:hyperlink ref="D247" r:id="rId915"/>
-    <x:hyperlink ref="D248" r:id="rId916"/>
-    <x:hyperlink ref="D249" r:id="rId917"/>
-    <x:hyperlink ref="D250" r:id="rId918"/>
-    <x:hyperlink ref="D251" r:id="rId919"/>
-    <x:hyperlink ref="D252" r:id="rId920"/>
-    <x:hyperlink ref="D253" r:id="rId921"/>
-    <x:hyperlink ref="D254" r:id="rId922"/>
-    <x:hyperlink ref="D255" r:id="rId923"/>
-    <x:hyperlink ref="D256" r:id="rId924"/>
-    <x:hyperlink ref="D257" r:id="rId925"/>
-    <x:hyperlink ref="D258" r:id="rId926"/>
-    <x:hyperlink ref="D259" r:id="rId927"/>
-    <x:hyperlink ref="D260" r:id="rId928"/>
-    <x:hyperlink ref="D261" r:id="rId929"/>
-    <x:hyperlink ref="D262" r:id="rId930"/>
-    <x:hyperlink ref="D263" r:id="rId931"/>
-    <x:hyperlink ref="D264" r:id="rId932"/>
-    <x:hyperlink ref="D265" r:id="rId933"/>
-    <x:hyperlink ref="D266" r:id="rId934"/>
-    <x:hyperlink ref="D267" r:id="rId935"/>
-    <x:hyperlink ref="D268" r:id="rId936"/>
-    <x:hyperlink ref="D269" r:id="rId937"/>
-    <x:hyperlink ref="D270" r:id="rId938"/>
-    <x:hyperlink ref="D271" r:id="rId939"/>
-    <x:hyperlink ref="D272" r:id="rId940"/>
-    <x:hyperlink ref="D273" r:id="rId941"/>
-    <x:hyperlink ref="D274" r:id="rId942"/>
-    <x:hyperlink ref="D275" r:id="rId943"/>
-    <x:hyperlink ref="D276" r:id="rId944"/>
-    <x:hyperlink ref="D277" r:id="rId945"/>
-    <x:hyperlink ref="D278" r:id="rId946"/>
-    <x:hyperlink ref="D279" r:id="rId947"/>
-    <x:hyperlink ref="D280" r:id="rId948"/>
-    <x:hyperlink ref="D281" r:id="rId949"/>
-    <x:hyperlink ref="D282" r:id="rId950"/>
-    <x:hyperlink ref="D283" r:id="rId951"/>
-    <x:hyperlink ref="D284" r:id="rId952"/>
-    <x:hyperlink ref="D285" r:id="rId953"/>
-    <x:hyperlink ref="D286" r:id="rId954"/>
-    <x:hyperlink ref="D287" r:id="rId955"/>
-    <x:hyperlink ref="D288" r:id="rId956"/>
-    <x:hyperlink ref="D289" r:id="rId957"/>
-    <x:hyperlink ref="D290" r:id="rId958"/>
-    <x:hyperlink ref="D291" r:id="rId959"/>
-    <x:hyperlink ref="D292" r:id="rId960"/>
-    <x:hyperlink ref="D293" r:id="rId961"/>
-    <x:hyperlink ref="D294" r:id="rId962"/>
-    <x:hyperlink ref="D295" r:id="rId963"/>
-    <x:hyperlink ref="D296" r:id="rId964"/>
-    <x:hyperlink ref="D297" r:id="rId965"/>
-    <x:hyperlink ref="D298" r:id="rId966"/>
-    <x:hyperlink ref="D299" r:id="rId967"/>
-    <x:hyperlink ref="D300" r:id="rId968"/>
-    <x:hyperlink ref="D301" r:id="rId969"/>
-    <x:hyperlink ref="D302" r:id="rId970"/>
-    <x:hyperlink ref="D303" r:id="rId971"/>
-    <x:hyperlink ref="D304" r:id="rId972"/>
-    <x:hyperlink ref="D305" r:id="rId973"/>
-    <x:hyperlink ref="D306" r:id="rId974"/>
-    <x:hyperlink ref="D307" r:id="rId975"/>
-    <x:hyperlink ref="D308" r:id="rId976"/>
-    <x:hyperlink ref="D309" r:id="rId977"/>
-    <x:hyperlink ref="D310" r:id="rId978"/>
-    <x:hyperlink ref="D311" r:id="rId979"/>
-    <x:hyperlink ref="D312" r:id="rId980"/>
-    <x:hyperlink ref="D313" r:id="rId981"/>
-    <x:hyperlink ref="D314" r:id="rId982"/>
-    <x:hyperlink ref="D315" r:id="rId983"/>
-    <x:hyperlink ref="D316" r:id="rId984"/>
-    <x:hyperlink ref="D317" r:id="rId985"/>
-    <x:hyperlink ref="D318" r:id="rId986"/>
-    <x:hyperlink ref="D319" r:id="rId987"/>
-    <x:hyperlink ref="D320" r:id="rId988"/>
-    <x:hyperlink ref="D321" r:id="rId989"/>
-    <x:hyperlink ref="D322" r:id="rId990"/>
-    <x:hyperlink ref="D323" r:id="rId991"/>
-    <x:hyperlink ref="D324" r:id="rId992"/>
-    <x:hyperlink ref="D325" r:id="rId993"/>
-    <x:hyperlink ref="D326" r:id="rId994"/>
-    <x:hyperlink ref="D327" r:id="rId995"/>
-    <x:hyperlink ref="D328" r:id="rId996"/>
-    <x:hyperlink ref="D329" r:id="rId997"/>
-    <x:hyperlink ref="D330" r:id="rId998"/>
-    <x:hyperlink ref="D331" r:id="rId999"/>
-    <x:hyperlink ref="D332" r:id="rId1000"/>
-    <x:hyperlink ref="D333" r:id="rId1001"/>
-    <x:hyperlink ref="D334" r:id="rId1002"/>
-    <x:hyperlink ref="D335" r:id="rId1003"/>
-    <x:hyperlink ref="D336" r:id="rId1004"/>
-    <x:hyperlink ref="D337" r:id="rId1005"/>
-    <x:hyperlink ref="D338" r:id="rId1006"/>
-    <x:hyperlink ref="D339" r:id="rId1007"/>
-    <x:hyperlink ref="D340" r:id="rId1008"/>
-    <x:hyperlink ref="D341" r:id="rId1009"/>
-    <x:hyperlink ref="D342" r:id="rId1010"/>
-    <x:hyperlink ref="D343" r:id="rId1011"/>
-    <x:hyperlink ref="D344" r:id="rId1012"/>
-    <x:hyperlink ref="D345" r:id="rId1013"/>
-    <x:hyperlink ref="D346" r:id="rId1014"/>
-    <x:hyperlink ref="D347" r:id="rId1015"/>
-    <x:hyperlink ref="D348" r:id="rId1016"/>
-    <x:hyperlink ref="D349" r:id="rId1017"/>
-    <x:hyperlink ref="D350" r:id="rId1018"/>
-    <x:hyperlink ref="D351" r:id="rId1019"/>
-    <x:hyperlink ref="D352" r:id="rId1020"/>
-    <x:hyperlink ref="D353" r:id="rId1021"/>
-    <x:hyperlink ref="D354" r:id="rId1022"/>
-    <x:hyperlink ref="D355" r:id="rId1023"/>
-    <x:hyperlink ref="D356" r:id="rId1024"/>
-    <x:hyperlink ref="D357" r:id="rId1025"/>
-    <x:hyperlink ref="D358" r:id="rId1026"/>
-    <x:hyperlink ref="D359" r:id="rId1027"/>
-    <x:hyperlink ref="D360" r:id="rId1028"/>
-    <x:hyperlink ref="D361" r:id="rId1029"/>
-    <x:hyperlink ref="D362" r:id="rId1030"/>
-    <x:hyperlink ref="D363" r:id="rId1031"/>
-    <x:hyperlink ref="D364" r:id="rId1032"/>
-    <x:hyperlink ref="D365" r:id="rId1033"/>
-    <x:hyperlink ref="D366" r:id="rId1034"/>
-    <x:hyperlink ref="D367" r:id="rId1035"/>
-    <x:hyperlink ref="D368" r:id="rId1036"/>
-    <x:hyperlink ref="D369" r:id="rId1037"/>
-    <x:hyperlink ref="D370" r:id="rId1038"/>
-    <x:hyperlink ref="D371" r:id="rId1039"/>
-    <x:hyperlink ref="D372" r:id="rId1040"/>
-    <x:hyperlink ref="D373" r:id="rId1041"/>
-    <x:hyperlink ref="D374" r:id="rId1042"/>
-    <x:hyperlink ref="D375" r:id="rId1043"/>
-    <x:hyperlink ref="D376" r:id="rId1044"/>
-    <x:hyperlink ref="D377" r:id="rId1045"/>
-    <x:hyperlink ref="D378" r:id="rId1046"/>
-    <x:hyperlink ref="D379" r:id="rId1047"/>
-    <x:hyperlink ref="D380" r:id="rId1048"/>
-    <x:hyperlink ref="D381" r:id="rId1049"/>
-    <x:hyperlink ref="D382" r:id="rId1050"/>
-    <x:hyperlink ref="D383" r:id="rId1051"/>
-    <x:hyperlink ref="D384" r:id="rId1052"/>
-    <x:hyperlink ref="D385" r:id="rId1053"/>
-    <x:hyperlink ref="D386" r:id="rId1054"/>
-    <x:hyperlink ref="D387" r:id="rId1055"/>
-    <x:hyperlink ref="D388" r:id="rId1056"/>
-    <x:hyperlink ref="D389" r:id="rId1057"/>
-    <x:hyperlink ref="D390" r:id="rId1058"/>
-    <x:hyperlink ref="D391" r:id="rId1059"/>
-    <x:hyperlink ref="D392" r:id="rId1060"/>
-    <x:hyperlink ref="D393" r:id="rId1061"/>
-    <x:hyperlink ref="D394" r:id="rId1062"/>
-    <x:hyperlink ref="D395" r:id="rId1063"/>
-    <x:hyperlink ref="D396" r:id="rId1064"/>
-    <x:hyperlink ref="D397" r:id="rId1065"/>
-    <x:hyperlink ref="D398" r:id="rId1066"/>
-    <x:hyperlink ref="D399" r:id="rId1067"/>
-    <x:hyperlink ref="D400" r:id="rId1068"/>
-    <x:hyperlink ref="D401" r:id="rId1069"/>
-    <x:hyperlink ref="D402" r:id="rId1070"/>
-    <x:hyperlink ref="D403" r:id="rId1071"/>
-    <x:hyperlink ref="D404" r:id="rId1072"/>
-    <x:hyperlink ref="D405" r:id="rId1073"/>
-    <x:hyperlink ref="D406" r:id="rId1074"/>
-    <x:hyperlink ref="D407" r:id="rId1075"/>
-    <x:hyperlink ref="D408" r:id="rId1076"/>
-    <x:hyperlink ref="D409" r:id="rId1077"/>
-    <x:hyperlink ref="D410" r:id="rId1078"/>
-    <x:hyperlink ref="D411" r:id="rId1079"/>
-    <x:hyperlink ref="D412" r:id="rId1080"/>
-    <x:hyperlink ref="D413" r:id="rId1081"/>
-    <x:hyperlink ref="D414" r:id="rId1082"/>
-    <x:hyperlink ref="D415" r:id="rId1083"/>
-    <x:hyperlink ref="D416" r:id="rId1084"/>
-    <x:hyperlink ref="D417" r:id="rId1085"/>
-    <x:hyperlink ref="D418" r:id="rId1086"/>
-    <x:hyperlink ref="D419" r:id="rId1087"/>
-    <x:hyperlink ref="D420" r:id="rId1088"/>
-    <x:hyperlink ref="D421" r:id="rId1089"/>
-    <x:hyperlink ref="D422" r:id="rId1090"/>
-    <x:hyperlink ref="D423" r:id="rId1091"/>
-    <x:hyperlink ref="D424" r:id="rId1092"/>
-    <x:hyperlink ref="D425" r:id="rId1093"/>
-    <x:hyperlink ref="D426" r:id="rId1094"/>
-    <x:hyperlink ref="D427" r:id="rId1095"/>
-    <x:hyperlink ref="D428" r:id="rId1096"/>
-    <x:hyperlink ref="D429" r:id="rId1097"/>
-    <x:hyperlink ref="D430" r:id="rId1098"/>
-    <x:hyperlink ref="D431" r:id="rId1099"/>
-    <x:hyperlink ref="D432" r:id="rId1100"/>
-    <x:hyperlink ref="D433" r:id="rId1101"/>
-    <x:hyperlink ref="D434" r:id="rId1102"/>
-    <x:hyperlink ref="D435" r:id="rId1103"/>
-    <x:hyperlink ref="D436" r:id="rId1104"/>
-    <x:hyperlink ref="D437" r:id="rId1105"/>
-    <x:hyperlink ref="D438" r:id="rId1106"/>
-    <x:hyperlink ref="D439" r:id="rId1107"/>
-    <x:hyperlink ref="D440" r:id="rId1108"/>
-    <x:hyperlink ref="D441" r:id="rId1109"/>
-    <x:hyperlink ref="D442" r:id="rId1110"/>
-    <x:hyperlink ref="D443" r:id="rId1111"/>
-    <x:hyperlink ref="D444" r:id="rId1112"/>
-    <x:hyperlink ref="D445" r:id="rId1113"/>
-    <x:hyperlink ref="D446" r:id="rId1114"/>
-    <x:hyperlink ref="D447" r:id="rId1115"/>
-    <x:hyperlink ref="D448" r:id="rId1116"/>
-    <x:hyperlink ref="D449" r:id="rId1117"/>
-    <x:hyperlink ref="D450" r:id="rId1118"/>
-    <x:hyperlink ref="D451" r:id="rId1119"/>
-    <x:hyperlink ref="D452" r:id="rId1120"/>
-    <x:hyperlink ref="D453" r:id="rId1121"/>
-    <x:hyperlink ref="D454" r:id="rId1122"/>
-    <x:hyperlink ref="D455" r:id="rId1123"/>
-    <x:hyperlink ref="D456" r:id="rId1124"/>
-    <x:hyperlink ref="D457" r:id="rId1125"/>
-    <x:hyperlink ref="D458" r:id="rId1126"/>
-    <x:hyperlink ref="D459" r:id="rId1127"/>
-    <x:hyperlink ref="D460" r:id="rId1128"/>
-    <x:hyperlink ref="D461" r:id="rId1129"/>
-    <x:hyperlink ref="D462" r:id="rId1130"/>
-    <x:hyperlink ref="D463" r:id="rId1131"/>
-    <x:hyperlink ref="D464" r:id="rId1132"/>
-    <x:hyperlink ref="D465" r:id="rId1133"/>
-    <x:hyperlink ref="D466" r:id="rId1134"/>
-    <x:hyperlink ref="D467" r:id="rId1135"/>
-    <x:hyperlink ref="D468" r:id="rId1136"/>
-    <x:hyperlink ref="D469" r:id="rId1137"/>
-    <x:hyperlink ref="D470" r:id="rId1138"/>
-    <x:hyperlink ref="D471" r:id="rId1139"/>
-    <x:hyperlink ref="D472" r:id="rId1140"/>
-    <x:hyperlink ref="D473" r:id="rId1141"/>
-    <x:hyperlink ref="D474" r:id="rId1142"/>
-    <x:hyperlink ref="D475" r:id="rId1143"/>
-    <x:hyperlink ref="D476" r:id="rId1144"/>
-    <x:hyperlink ref="D477" r:id="rId1145"/>
-    <x:hyperlink ref="D478" r:id="rId1146"/>
-    <x:hyperlink ref="D479" r:id="rId1147"/>
-    <x:hyperlink ref="D480" r:id="rId1148"/>
-    <x:hyperlink ref="D481" r:id="rId1149"/>
-    <x:hyperlink ref="D482" r:id="rId1150"/>
-    <x:hyperlink ref="D483" r:id="rId1151"/>
-    <x:hyperlink ref="D484" r:id="rId1152"/>
-    <x:hyperlink ref="D485" r:id="rId1153"/>
-    <x:hyperlink ref="D486" r:id="rId1154"/>
-    <x:hyperlink ref="D487" r:id="rId1155"/>
-    <x:hyperlink ref="D488" r:id="rId1156"/>
-    <x:hyperlink ref="D489" r:id="rId1157"/>
-    <x:hyperlink ref="D490" r:id="rId1158"/>
-    <x:hyperlink ref="D491" r:id="rId1159"/>
-    <x:hyperlink ref="D492" r:id="rId1160"/>
-    <x:hyperlink ref="D493" r:id="rId1161"/>
-    <x:hyperlink ref="D494" r:id="rId1162"/>
-    <x:hyperlink ref="D495" r:id="rId1163"/>
-    <x:hyperlink ref="D496" r:id="rId1164"/>
-    <x:hyperlink ref="D497" r:id="rId1165"/>
-    <x:hyperlink ref="D498" r:id="rId1166"/>
-    <x:hyperlink ref="D499" r:id="rId1167"/>
-    <x:hyperlink ref="D500" r:id="rId1168"/>
-    <x:hyperlink ref="D501" r:id="rId1169"/>
-    <x:hyperlink ref="D502" r:id="rId1170"/>
-    <x:hyperlink ref="D503" r:id="rId1171"/>
-    <x:hyperlink ref="D504" r:id="rId1172"/>
-    <x:hyperlink ref="D505" r:id="rId1173"/>
-    <x:hyperlink ref="D506" r:id="rId1174"/>
-    <x:hyperlink ref="D507" r:id="rId1175"/>
-    <x:hyperlink ref="D508" r:id="rId1176"/>
-    <x:hyperlink ref="D509" r:id="rId1177"/>
-    <x:hyperlink ref="D510" r:id="rId1178"/>
-    <x:hyperlink ref="D511" r:id="rId1179"/>
-    <x:hyperlink ref="D512" r:id="rId1180"/>
-    <x:hyperlink ref="D513" r:id="rId1181"/>
-    <x:hyperlink ref="D514" r:id="rId1182"/>
-    <x:hyperlink ref="D515" r:id="rId1183"/>
-    <x:hyperlink ref="D516" r:id="rId1184"/>
-    <x:hyperlink ref="D517" r:id="rId1185"/>
-    <x:hyperlink ref="D518" r:id="rId1186"/>
-    <x:hyperlink ref="D519" r:id="rId1187"/>
-    <x:hyperlink ref="D520" r:id="rId1188"/>
-    <x:hyperlink ref="D521" r:id="rId1189"/>
-    <x:hyperlink ref="D522" r:id="rId1190"/>
-    <x:hyperlink ref="D523" r:id="rId1191"/>
-    <x:hyperlink ref="D524" r:id="rId1192"/>
-    <x:hyperlink ref="D525" r:id="rId1193"/>
-    <x:hyperlink ref="D526" r:id="rId1194"/>
-    <x:hyperlink ref="D527" r:id="rId1195"/>
-    <x:hyperlink ref="D528" r:id="rId1196"/>
-    <x:hyperlink ref="D529" r:id="rId1197"/>
-    <x:hyperlink ref="D530" r:id="rId1198"/>
-    <x:hyperlink ref="D531" r:id="rId1199"/>
-    <x:hyperlink ref="D532" r:id="rId1200"/>
-    <x:hyperlink ref="D533" r:id="rId1201"/>
-    <x:hyperlink ref="D534" r:id="rId1202"/>
-    <x:hyperlink ref="D535" r:id="rId1203"/>
-    <x:hyperlink ref="D536" r:id="rId1204"/>
-    <x:hyperlink ref="D537" r:id="rId1205"/>
-    <x:hyperlink ref="D538" r:id="rId1206"/>
-    <x:hyperlink ref="D539" r:id="rId1207"/>
-    <x:hyperlink ref="D540" r:id="rId1208"/>
-    <x:hyperlink ref="D541" r:id="rId1209"/>
-    <x:hyperlink ref="D542" r:id="rId1210"/>
-    <x:hyperlink ref="D543" r:id="rId1211"/>
-    <x:hyperlink ref="D544" r:id="rId1212"/>
-    <x:hyperlink ref="D545" r:id="rId1213"/>
-    <x:hyperlink ref="D546" r:id="rId1214"/>
-    <x:hyperlink ref="D547" r:id="rId1215"/>
-    <x:hyperlink ref="D548" r:id="rId1216"/>
-    <x:hyperlink ref="D549" r:id="rId1217"/>
-    <x:hyperlink ref="D550" r:id="rId1218"/>
-    <x:hyperlink ref="D551" r:id="rId1219"/>
-    <x:hyperlink ref="D552" r:id="rId1220"/>
-    <x:hyperlink ref="D553" r:id="rId1221"/>
-    <x:hyperlink ref="D554" r:id="rId1222"/>
-    <x:hyperlink ref="D555" r:id="rId1223"/>
-    <x:hyperlink ref="D556" r:id="rId1224"/>
-    <x:hyperlink ref="D557" r:id="rId1225"/>
-    <x:hyperlink ref="D558" r:id="rId1226"/>
-    <x:hyperlink ref="D559" r:id="rId1227"/>
-    <x:hyperlink ref="D560" r:id="rId1228"/>
-    <x:hyperlink ref="D561" r:id="rId1229"/>
-    <x:hyperlink ref="D562" r:id="rId1230"/>
-    <x:hyperlink ref="D563" r:id="rId1231"/>
-    <x:hyperlink ref="D564" r:id="rId1232"/>
-    <x:hyperlink ref="D565" r:id="rId1233"/>
-    <x:hyperlink ref="D566" r:id="rId1234"/>
-    <x:hyperlink ref="D567" r:id="rId1235"/>
-    <x:hyperlink ref="D568" r:id="rId1236"/>
-    <x:hyperlink ref="D569" r:id="rId1237"/>
-    <x:hyperlink ref="D570" r:id="rId1238"/>
-    <x:hyperlink ref="D571" r:id="rId1239"/>
-    <x:hyperlink ref="D572" r:id="rId1240"/>
-    <x:hyperlink ref="D573" r:id="rId1241"/>
-    <x:hyperlink ref="D574" r:id="rId1242"/>
-    <x:hyperlink ref="D575" r:id="rId1243"/>
-    <x:hyperlink ref="D576" r:id="rId1244"/>
-    <x:hyperlink ref="D577" r:id="rId1245"/>
-    <x:hyperlink ref="D578" r:id="rId1246"/>
-    <x:hyperlink ref="D579" r:id="rId1247"/>
-    <x:hyperlink ref="D580" r:id="rId1248"/>
-    <x:hyperlink ref="D581" r:id="rId1249"/>
-    <x:hyperlink ref="D582" r:id="rId1250"/>
-    <x:hyperlink ref="D583" r:id="rId1251"/>
-    <x:hyperlink ref="D584" r:id="rId1252"/>
-    <x:hyperlink ref="D585" r:id="rId1253"/>
-    <x:hyperlink ref="D586" r:id="rId1254"/>
-    <x:hyperlink ref="D587" r:id="rId1255"/>
-    <x:hyperlink ref="D588" r:id="rId1256"/>
-    <x:hyperlink ref="D589" r:id="rId1257"/>
-    <x:hyperlink ref="D590" r:id="rId1258"/>
-    <x:hyperlink ref="D591" r:id="rId1259"/>
-    <x:hyperlink ref="D592" r:id="rId1260"/>
-    <x:hyperlink ref="D593" r:id="rId1261"/>
-    <x:hyperlink ref="D594" r:id="rId1262"/>
-    <x:hyperlink ref="D595" r:id="rId1263"/>
-    <x:hyperlink ref="D596" r:id="rId1264"/>
-    <x:hyperlink ref="D597" r:id="rId1265"/>
-    <x:hyperlink ref="D598" r:id="rId1266"/>
-    <x:hyperlink ref="D599" r:id="rId1267"/>
-    <x:hyperlink ref="D600" r:id="rId1268"/>
-    <x:hyperlink ref="D601" r:id="rId1269"/>
-    <x:hyperlink ref="D602" r:id="rId1270"/>
-    <x:hyperlink ref="D603" r:id="rId1271"/>
-    <x:hyperlink ref="D604" r:id="rId1272"/>
-    <x:hyperlink ref="D605" r:id="rId1273"/>
-    <x:hyperlink ref="D606" r:id="rId1274"/>
-    <x:hyperlink ref="D607" r:id="rId1275"/>
-    <x:hyperlink ref="D608" r:id="rId1276"/>
-    <x:hyperlink ref="D609" r:id="rId1277"/>
-    <x:hyperlink ref="D610" r:id="rId1278"/>
-    <x:hyperlink ref="D611" r:id="rId1279"/>
-    <x:hyperlink ref="D612" r:id="rId1280"/>
-    <x:hyperlink ref="D613" r:id="rId1281"/>
-    <x:hyperlink ref="D614" r:id="rId1282"/>
-    <x:hyperlink ref="D615" r:id="rId1283"/>
-    <x:hyperlink ref="D616" r:id="rId1284"/>
-    <x:hyperlink ref="D617" r:id="rId1285"/>
-    <x:hyperlink ref="D618" r:id="rId1286"/>
-    <x:hyperlink ref="D619" r:id="rId1287"/>
-    <x:hyperlink ref="D620" r:id="rId1288"/>
-    <x:hyperlink ref="D621" r:id="rId1289"/>
-    <x:hyperlink ref="D622" r:id="rId1290"/>
-    <x:hyperlink ref="D623" r:id="rId1291"/>
-    <x:hyperlink ref="D624" r:id="rId1292"/>
-    <x:hyperlink ref="D625" r:id="rId1293"/>
-    <x:hyperlink ref="D626" r:id="rId1294"/>
-    <x:hyperlink ref="D627" r:id="rId1295"/>
-    <x:hyperlink ref="D628" r:id="rId1296"/>
-    <x:hyperlink ref="D629" r:id="rId1297"/>
-    <x:hyperlink ref="D630" r:id="rId1298"/>
-    <x:hyperlink ref="D631" r:id="rId1299"/>
-    <x:hyperlink ref="D632" r:id="rId1300"/>
-    <x:hyperlink ref="D633" r:id="rId1301"/>
-    <x:hyperlink ref="D634" r:id="rId1302"/>
-    <x:hyperlink ref="D635" r:id="rId1303"/>
-    <x:hyperlink ref="D636" r:id="rId1304"/>
-    <x:hyperlink ref="D637" r:id="rId1305"/>
-    <x:hyperlink ref="D638" r:id="rId1306"/>
-    <x:hyperlink ref="D639" r:id="rId1307"/>
-    <x:hyperlink ref="D640" r:id="rId1308"/>
-    <x:hyperlink ref="D641" r:id="rId1309"/>
-    <x:hyperlink ref="D642" r:id="rId1310"/>
-    <x:hyperlink ref="D643" r:id="rId1311"/>
-    <x:hyperlink ref="D644" r:id="rId1312"/>
-    <x:hyperlink ref="D645" r:id="rId1313"/>
-    <x:hyperlink ref="D646" r:id="rId1314"/>
-    <x:hyperlink ref="D647" r:id="rId1315"/>
-    <x:hyperlink ref="D648" r:id="rId1316"/>
-    <x:hyperlink ref="D649" r:id="rId1317"/>
-    <x:hyperlink ref="D650" r:id="rId1318"/>
-    <x:hyperlink ref="D651" r:id="rId1319"/>
-    <x:hyperlink ref="D652" r:id="rId1320"/>
-    <x:hyperlink ref="D653" r:id="rId1321"/>
-    <x:hyperlink ref="D654" r:id="rId1322"/>
-    <x:hyperlink ref="D655" r:id="rId1323"/>
-    <x:hyperlink ref="D656" r:id="rId1324"/>
-    <x:hyperlink ref="D657" r:id="rId1325"/>
-    <x:hyperlink ref="D658" r:id="rId1326"/>
-    <x:hyperlink ref="D659" r:id="rId1327"/>
-    <x:hyperlink ref="D660" r:id="rId1328"/>
-    <x:hyperlink ref="D661" r:id="rId1329"/>
-    <x:hyperlink ref="D662" r:id="rId1330"/>
-    <x:hyperlink ref="D663" r:id="rId1331"/>
-    <x:hyperlink ref="D664" r:id="rId1332"/>
-    <x:hyperlink ref="D665" r:id="rId1333"/>
-    <x:hyperlink ref="D666" r:id="rId1334"/>
-    <x:hyperlink ref="D667" r:id="rId1335"/>
-    <x:hyperlink ref="D668" r:id="rId1336"/>
-    <x:hyperlink ref="D669" r:id="rId1337"/>
-    <x:hyperlink ref="D670" r:id="rId1338"/>
-    <x:hyperlink ref="D671" r:id="rId1339"/>
-    <x:hyperlink ref="D672" r:id="rId1340"/>
+    <x:hyperlink ref="D6" r:id="rId692"/>
+    <x:hyperlink ref="D7" r:id="rId693"/>
+    <x:hyperlink ref="D8" r:id="rId694"/>
+    <x:hyperlink ref="D9" r:id="rId695"/>
+    <x:hyperlink ref="D10" r:id="rId696"/>
+    <x:hyperlink ref="D11" r:id="rId697"/>
+    <x:hyperlink ref="D12" r:id="rId698"/>
+    <x:hyperlink ref="D13" r:id="rId699"/>
+    <x:hyperlink ref="D14" r:id="rId700"/>
+    <x:hyperlink ref="D15" r:id="rId701"/>
+    <x:hyperlink ref="D16" r:id="rId702"/>
+    <x:hyperlink ref="D17" r:id="rId703"/>
+    <x:hyperlink ref="D18" r:id="rId704"/>
+    <x:hyperlink ref="D19" r:id="rId705"/>
+    <x:hyperlink ref="D20" r:id="rId706"/>
+    <x:hyperlink ref="D21" r:id="rId707"/>
+    <x:hyperlink ref="D22" r:id="rId708"/>
+    <x:hyperlink ref="D23" r:id="rId709"/>
+    <x:hyperlink ref="D24" r:id="rId710"/>
+    <x:hyperlink ref="D25" r:id="rId711"/>
+    <x:hyperlink ref="D26" r:id="rId712"/>
+    <x:hyperlink ref="D27" r:id="rId713"/>
+    <x:hyperlink ref="D28" r:id="rId714"/>
+    <x:hyperlink ref="D29" r:id="rId715"/>
+    <x:hyperlink ref="D30" r:id="rId716"/>
+    <x:hyperlink ref="D31" r:id="rId717"/>
+    <x:hyperlink ref="D32" r:id="rId718"/>
+    <x:hyperlink ref="D33" r:id="rId719"/>
+    <x:hyperlink ref="D34" r:id="rId720"/>
+    <x:hyperlink ref="D35" r:id="rId721"/>
+    <x:hyperlink ref="D36" r:id="rId722"/>
+    <x:hyperlink ref="D37" r:id="rId723"/>
+    <x:hyperlink ref="D38" r:id="rId724"/>
+    <x:hyperlink ref="D39" r:id="rId725"/>
+    <x:hyperlink ref="D40" r:id="rId726"/>
+    <x:hyperlink ref="D41" r:id="rId727"/>
+    <x:hyperlink ref="D42" r:id="rId728"/>
+    <x:hyperlink ref="D43" r:id="rId729"/>
+    <x:hyperlink ref="D44" r:id="rId730"/>
+    <x:hyperlink ref="D45" r:id="rId731"/>
+    <x:hyperlink ref="D46" r:id="rId732"/>
+    <x:hyperlink ref="D47" r:id="rId733"/>
+    <x:hyperlink ref="D48" r:id="rId734"/>
+    <x:hyperlink ref="D49" r:id="rId735"/>
+    <x:hyperlink ref="D50" r:id="rId736"/>
+    <x:hyperlink ref="D51" r:id="rId737"/>
+    <x:hyperlink ref="D52" r:id="rId738"/>
+    <x:hyperlink ref="D53" r:id="rId739"/>
+    <x:hyperlink ref="D54" r:id="rId740"/>
+    <x:hyperlink ref="D55" r:id="rId741"/>
+    <x:hyperlink ref="D56" r:id="rId742"/>
+    <x:hyperlink ref="D57" r:id="rId743"/>
+    <x:hyperlink ref="D58" r:id="rId744"/>
+    <x:hyperlink ref="D59" r:id="rId745"/>
+    <x:hyperlink ref="D60" r:id="rId746"/>
+    <x:hyperlink ref="D61" r:id="rId747"/>
+    <x:hyperlink ref="D62" r:id="rId748"/>
+    <x:hyperlink ref="D63" r:id="rId749"/>
+    <x:hyperlink ref="D64" r:id="rId750"/>
+    <x:hyperlink ref="D65" r:id="rId751"/>
+    <x:hyperlink ref="D66" r:id="rId752"/>
+    <x:hyperlink ref="D67" r:id="rId753"/>
+    <x:hyperlink ref="D68" r:id="rId754"/>
+    <x:hyperlink ref="D69" r:id="rId755"/>
+    <x:hyperlink ref="D70" r:id="rId756"/>
+    <x:hyperlink ref="D71" r:id="rId757"/>
+    <x:hyperlink ref="D72" r:id="rId758"/>
+    <x:hyperlink ref="D73" r:id="rId759"/>
+    <x:hyperlink ref="D74" r:id="rId760"/>
+    <x:hyperlink ref="D75" r:id="rId761"/>
+    <x:hyperlink ref="D76" r:id="rId762"/>
+    <x:hyperlink ref="D77" r:id="rId763"/>
+    <x:hyperlink ref="D78" r:id="rId764"/>
+    <x:hyperlink ref="D79" r:id="rId765"/>
+    <x:hyperlink ref="D80" r:id="rId766"/>
+    <x:hyperlink ref="D81" r:id="rId767"/>
+    <x:hyperlink ref="D82" r:id="rId768"/>
+    <x:hyperlink ref="D83" r:id="rId769"/>
+    <x:hyperlink ref="D84" r:id="rId770"/>
+    <x:hyperlink ref="D85" r:id="rId771"/>
+    <x:hyperlink ref="D86" r:id="rId772"/>
+    <x:hyperlink ref="D87" r:id="rId773"/>
+    <x:hyperlink ref="D88" r:id="rId774"/>
+    <x:hyperlink ref="D89" r:id="rId775"/>
+    <x:hyperlink ref="D90" r:id="rId776"/>
+    <x:hyperlink ref="D91" r:id="rId777"/>
+    <x:hyperlink ref="D92" r:id="rId778"/>
+    <x:hyperlink ref="D93" r:id="rId779"/>
+    <x:hyperlink ref="D94" r:id="rId780"/>
+    <x:hyperlink ref="D95" r:id="rId781"/>
+    <x:hyperlink ref="D96" r:id="rId782"/>
+    <x:hyperlink ref="D97" r:id="rId783"/>
+    <x:hyperlink ref="D98" r:id="rId784"/>
+    <x:hyperlink ref="D99" r:id="rId785"/>
+    <x:hyperlink ref="D100" r:id="rId786"/>
+    <x:hyperlink ref="D101" r:id="rId787"/>
+    <x:hyperlink ref="D102" r:id="rId788"/>
+    <x:hyperlink ref="D103" r:id="rId789"/>
+    <x:hyperlink ref="D104" r:id="rId790"/>
+    <x:hyperlink ref="D105" r:id="rId791"/>
+    <x:hyperlink ref="D106" r:id="rId792"/>
+    <x:hyperlink ref="D107" r:id="rId793"/>
+    <x:hyperlink ref="D108" r:id="rId794"/>
+    <x:hyperlink ref="D109" r:id="rId795"/>
+    <x:hyperlink ref="D110" r:id="rId796"/>
+    <x:hyperlink ref="D111" r:id="rId797"/>
+    <x:hyperlink ref="D112" r:id="rId798"/>
+    <x:hyperlink ref="D113" r:id="rId799"/>
+    <x:hyperlink ref="D114" r:id="rId800"/>
+    <x:hyperlink ref="D115" r:id="rId801"/>
+    <x:hyperlink ref="D116" r:id="rId802"/>
+    <x:hyperlink ref="D117" r:id="rId803"/>
+    <x:hyperlink ref="D118" r:id="rId804"/>
+    <x:hyperlink ref="D119" r:id="rId805"/>
+    <x:hyperlink ref="D120" r:id="rId806"/>
+    <x:hyperlink ref="D121" r:id="rId807"/>
+    <x:hyperlink ref="D122" r:id="rId808"/>
+    <x:hyperlink ref="D123" r:id="rId809"/>
+    <x:hyperlink ref="D124" r:id="rId810"/>
+    <x:hyperlink ref="D125" r:id="rId811"/>
+    <x:hyperlink ref="D126" r:id="rId812"/>
+    <x:hyperlink ref="D127" r:id="rId813"/>
+    <x:hyperlink ref="D128" r:id="rId814"/>
+    <x:hyperlink ref="D129" r:id="rId815"/>
+    <x:hyperlink ref="D130" r:id="rId816"/>
+    <x:hyperlink ref="D131" r:id="rId817"/>
+    <x:hyperlink ref="D132" r:id="rId818"/>
+    <x:hyperlink ref="D133" r:id="rId819"/>
+    <x:hyperlink ref="D134" r:id="rId820"/>
+    <x:hyperlink ref="D135" r:id="rId821"/>
+    <x:hyperlink ref="D136" r:id="rId822"/>
+    <x:hyperlink ref="D137" r:id="rId823"/>
+    <x:hyperlink ref="D138" r:id="rId824"/>
+    <x:hyperlink ref="D139" r:id="rId825"/>
+    <x:hyperlink ref="D140" r:id="rId826"/>
+    <x:hyperlink ref="D141" r:id="rId827"/>
+    <x:hyperlink ref="D142" r:id="rId828"/>
+    <x:hyperlink ref="D143" r:id="rId829"/>
+    <x:hyperlink ref="D144" r:id="rId830"/>
+    <x:hyperlink ref="D145" r:id="rId831"/>
+    <x:hyperlink ref="D146" r:id="rId832"/>
+    <x:hyperlink ref="D147" r:id="rId833"/>
+    <x:hyperlink ref="D148" r:id="rId834"/>
+    <x:hyperlink ref="D149" r:id="rId835"/>
+    <x:hyperlink ref="D150" r:id="rId836"/>
+    <x:hyperlink ref="D151" r:id="rId837"/>
+    <x:hyperlink ref="D152" r:id="rId838"/>
+    <x:hyperlink ref="D153" r:id="rId839"/>
+    <x:hyperlink ref="D154" r:id="rId840"/>
+    <x:hyperlink ref="D155" r:id="rId841"/>
+    <x:hyperlink ref="D156" r:id="rId842"/>
+    <x:hyperlink ref="D157" r:id="rId843"/>
+    <x:hyperlink ref="D158" r:id="rId844"/>
+    <x:hyperlink ref="D159" r:id="rId845"/>
+    <x:hyperlink ref="D160" r:id="rId846"/>
+    <x:hyperlink ref="D161" r:id="rId847"/>
+    <x:hyperlink ref="D162" r:id="rId848"/>
+    <x:hyperlink ref="D163" r:id="rId849"/>
+    <x:hyperlink ref="D164" r:id="rId850"/>
+    <x:hyperlink ref="D165" r:id="rId851"/>
+    <x:hyperlink ref="D166" r:id="rId852"/>
+    <x:hyperlink ref="D167" r:id="rId853"/>
+    <x:hyperlink ref="D168" r:id="rId854"/>
+    <x:hyperlink ref="D169" r:id="rId855"/>
+    <x:hyperlink ref="D170" r:id="rId856"/>
+    <x:hyperlink ref="D171" r:id="rId857"/>
+    <x:hyperlink ref="D172" r:id="rId858"/>
+    <x:hyperlink ref="D173" r:id="rId859"/>
+    <x:hyperlink ref="D174" r:id="rId860"/>
+    <x:hyperlink ref="D175" r:id="rId861"/>
+    <x:hyperlink ref="D176" r:id="rId862"/>
+    <x:hyperlink ref="D177" r:id="rId863"/>
+    <x:hyperlink ref="D178" r:id="rId864"/>
+    <x:hyperlink ref="D179" r:id="rId865"/>
+    <x:hyperlink ref="D180" r:id="rId866"/>
+    <x:hyperlink ref="D181" r:id="rId867"/>
+    <x:hyperlink ref="D182" r:id="rId868"/>
+    <x:hyperlink ref="D183" r:id="rId869"/>
+    <x:hyperlink ref="D184" r:id="rId870"/>
+    <x:hyperlink ref="D185" r:id="rId871"/>
+    <x:hyperlink ref="D186" r:id="rId872"/>
+    <x:hyperlink ref="D187" r:id="rId873"/>
+    <x:hyperlink ref="D188" r:id="rId874"/>
+    <x:hyperlink ref="D189" r:id="rId875"/>
+    <x:hyperlink ref="D190" r:id="rId876"/>
+    <x:hyperlink ref="D191" r:id="rId877"/>
+    <x:hyperlink ref="D192" r:id="rId878"/>
+    <x:hyperlink ref="D193" r:id="rId879"/>
+    <x:hyperlink ref="D194" r:id="rId880"/>
+    <x:hyperlink ref="D195" r:id="rId881"/>
+    <x:hyperlink ref="D196" r:id="rId882"/>
+    <x:hyperlink ref="D197" r:id="rId883"/>
+    <x:hyperlink ref="D198" r:id="rId884"/>
+    <x:hyperlink ref="D199" r:id="rId885"/>
+    <x:hyperlink ref="D200" r:id="rId886"/>
+    <x:hyperlink ref="D201" r:id="rId887"/>
+    <x:hyperlink ref="D202" r:id="rId888"/>
+    <x:hyperlink ref="D203" r:id="rId889"/>
+    <x:hyperlink ref="D204" r:id="rId890"/>
+    <x:hyperlink ref="D205" r:id="rId891"/>
+    <x:hyperlink ref="D206" r:id="rId892"/>
+    <x:hyperlink ref="D207" r:id="rId893"/>
+    <x:hyperlink ref="D208" r:id="rId894"/>
+    <x:hyperlink ref="D209" r:id="rId895"/>
+    <x:hyperlink ref="D210" r:id="rId896"/>
+    <x:hyperlink ref="D211" r:id="rId897"/>
+    <x:hyperlink ref="D212" r:id="rId898"/>
+    <x:hyperlink ref="D213" r:id="rId899"/>
+    <x:hyperlink ref="D214" r:id="rId900"/>
+    <x:hyperlink ref="D215" r:id="rId901"/>
+    <x:hyperlink ref="D216" r:id="rId902"/>
+    <x:hyperlink ref="D217" r:id="rId903"/>
+    <x:hyperlink ref="D218" r:id="rId904"/>
+    <x:hyperlink ref="D219" r:id="rId905"/>
+    <x:hyperlink ref="D220" r:id="rId906"/>
+    <x:hyperlink ref="D221" r:id="rId907"/>
+    <x:hyperlink ref="D222" r:id="rId908"/>
+    <x:hyperlink ref="D223" r:id="rId909"/>
+    <x:hyperlink ref="D224" r:id="rId910"/>
+    <x:hyperlink ref="D225" r:id="rId911"/>
+    <x:hyperlink ref="D226" r:id="rId912"/>
+    <x:hyperlink ref="D227" r:id="rId913"/>
+    <x:hyperlink ref="D228" r:id="rId914"/>
+    <x:hyperlink ref="D229" r:id="rId915"/>
+    <x:hyperlink ref="D230" r:id="rId916"/>
+    <x:hyperlink ref="D231" r:id="rId917"/>
+    <x:hyperlink ref="D232" r:id="rId918"/>
+    <x:hyperlink ref="D233" r:id="rId919"/>
+    <x:hyperlink ref="D234" r:id="rId920"/>
+    <x:hyperlink ref="D235" r:id="rId921"/>
+    <x:hyperlink ref="D236" r:id="rId922"/>
+    <x:hyperlink ref="D237" r:id="rId923"/>
+    <x:hyperlink ref="D238" r:id="rId924"/>
+    <x:hyperlink ref="D239" r:id="rId925"/>
+    <x:hyperlink ref="D240" r:id="rId926"/>
+    <x:hyperlink ref="D241" r:id="rId927"/>
+    <x:hyperlink ref="D242" r:id="rId928"/>
+    <x:hyperlink ref="D243" r:id="rId929"/>
+    <x:hyperlink ref="D244" r:id="rId930"/>
+    <x:hyperlink ref="D245" r:id="rId931"/>
+    <x:hyperlink ref="D246" r:id="rId932"/>
+    <x:hyperlink ref="D247" r:id="rId933"/>
+    <x:hyperlink ref="D248" r:id="rId934"/>
+    <x:hyperlink ref="D249" r:id="rId935"/>
+    <x:hyperlink ref="D250" r:id="rId936"/>
+    <x:hyperlink ref="D251" r:id="rId937"/>
+    <x:hyperlink ref="D252" r:id="rId938"/>
+    <x:hyperlink ref="D253" r:id="rId939"/>
+    <x:hyperlink ref="D254" r:id="rId940"/>
+    <x:hyperlink ref="D255" r:id="rId941"/>
+    <x:hyperlink ref="D256" r:id="rId942"/>
+    <x:hyperlink ref="D257" r:id="rId943"/>
+    <x:hyperlink ref="D258" r:id="rId944"/>
+    <x:hyperlink ref="D259" r:id="rId945"/>
+    <x:hyperlink ref="D260" r:id="rId946"/>
+    <x:hyperlink ref="D261" r:id="rId947"/>
+    <x:hyperlink ref="D262" r:id="rId948"/>
+    <x:hyperlink ref="D263" r:id="rId949"/>
+    <x:hyperlink ref="D264" r:id="rId950"/>
+    <x:hyperlink ref="D265" r:id="rId951"/>
+    <x:hyperlink ref="D266" r:id="rId952"/>
+    <x:hyperlink ref="D267" r:id="rId953"/>
+    <x:hyperlink ref="D268" r:id="rId954"/>
+    <x:hyperlink ref="D269" r:id="rId955"/>
+    <x:hyperlink ref="D270" r:id="rId956"/>
+    <x:hyperlink ref="D271" r:id="rId957"/>
+    <x:hyperlink ref="D272" r:id="rId958"/>
+    <x:hyperlink ref="D273" r:id="rId959"/>
+    <x:hyperlink ref="D274" r:id="rId960"/>
+    <x:hyperlink ref="D275" r:id="rId961"/>
+    <x:hyperlink ref="D276" r:id="rId962"/>
+    <x:hyperlink ref="D277" r:id="rId963"/>
+    <x:hyperlink ref="D278" r:id="rId964"/>
+    <x:hyperlink ref="D279" r:id="rId965"/>
+    <x:hyperlink ref="D280" r:id="rId966"/>
+    <x:hyperlink ref="D281" r:id="rId967"/>
+    <x:hyperlink ref="D282" r:id="rId968"/>
+    <x:hyperlink ref="D283" r:id="rId969"/>
+    <x:hyperlink ref="D284" r:id="rId970"/>
+    <x:hyperlink ref="D285" r:id="rId971"/>
+    <x:hyperlink ref="D286" r:id="rId972"/>
+    <x:hyperlink ref="D287" r:id="rId973"/>
+    <x:hyperlink ref="D288" r:id="rId974"/>
+    <x:hyperlink ref="D289" r:id="rId975"/>
+    <x:hyperlink ref="D290" r:id="rId976"/>
+    <x:hyperlink ref="D291" r:id="rId977"/>
+    <x:hyperlink ref="D292" r:id="rId978"/>
+    <x:hyperlink ref="D293" r:id="rId979"/>
+    <x:hyperlink ref="D294" r:id="rId980"/>
+    <x:hyperlink ref="D295" r:id="rId981"/>
+    <x:hyperlink ref="D296" r:id="rId982"/>
+    <x:hyperlink ref="D297" r:id="rId983"/>
+    <x:hyperlink ref="D298" r:id="rId984"/>
+    <x:hyperlink ref="D299" r:id="rId985"/>
+    <x:hyperlink ref="D300" r:id="rId986"/>
+    <x:hyperlink ref="D301" r:id="rId987"/>
+    <x:hyperlink ref="D302" r:id="rId988"/>
+    <x:hyperlink ref="D303" r:id="rId989"/>
+    <x:hyperlink ref="D304" r:id="rId990"/>
+    <x:hyperlink ref="D305" r:id="rId991"/>
+    <x:hyperlink ref="D306" r:id="rId992"/>
+    <x:hyperlink ref="D307" r:id="rId993"/>
+    <x:hyperlink ref="D308" r:id="rId994"/>
+    <x:hyperlink ref="D309" r:id="rId995"/>
+    <x:hyperlink ref="D310" r:id="rId996"/>
+    <x:hyperlink ref="D311" r:id="rId997"/>
+    <x:hyperlink ref="D312" r:id="rId998"/>
+    <x:hyperlink ref="D313" r:id="rId999"/>
+    <x:hyperlink ref="D314" r:id="rId1000"/>
+    <x:hyperlink ref="D315" r:id="rId1001"/>
+    <x:hyperlink ref="D316" r:id="rId1002"/>
+    <x:hyperlink ref="D317" r:id="rId1003"/>
+    <x:hyperlink ref="D318" r:id="rId1004"/>
+    <x:hyperlink ref="D319" r:id="rId1005"/>
+    <x:hyperlink ref="D320" r:id="rId1006"/>
+    <x:hyperlink ref="D321" r:id="rId1007"/>
+    <x:hyperlink ref="D322" r:id="rId1008"/>
+    <x:hyperlink ref="D323" r:id="rId1009"/>
+    <x:hyperlink ref="D324" r:id="rId1010"/>
+    <x:hyperlink ref="D325" r:id="rId1011"/>
+    <x:hyperlink ref="D326" r:id="rId1012"/>
+    <x:hyperlink ref="D327" r:id="rId1013"/>
+    <x:hyperlink ref="D328" r:id="rId1014"/>
+    <x:hyperlink ref="D329" r:id="rId1015"/>
+    <x:hyperlink ref="D330" r:id="rId1016"/>
+    <x:hyperlink ref="D331" r:id="rId1017"/>
+    <x:hyperlink ref="D332" r:id="rId1018"/>
+    <x:hyperlink ref="D333" r:id="rId1019"/>
+    <x:hyperlink ref="D334" r:id="rId1020"/>
+    <x:hyperlink ref="D335" r:id="rId1021"/>
+    <x:hyperlink ref="D336" r:id="rId1022"/>
+    <x:hyperlink ref="D337" r:id="rId1023"/>
+    <x:hyperlink ref="D338" r:id="rId1024"/>
+    <x:hyperlink ref="D339" r:id="rId1025"/>
+    <x:hyperlink ref="D340" r:id="rId1026"/>
+    <x:hyperlink ref="D341" r:id="rId1027"/>
+    <x:hyperlink ref="D342" r:id="rId1028"/>
+    <x:hyperlink ref="D343" r:id="rId1029"/>
+    <x:hyperlink ref="D344" r:id="rId1030"/>
+    <x:hyperlink ref="D345" r:id="rId1031"/>
+    <x:hyperlink ref="D346" r:id="rId1032"/>
+    <x:hyperlink ref="D347" r:id="rId1033"/>
+    <x:hyperlink ref="D348" r:id="rId1034"/>
+    <x:hyperlink ref="D349" r:id="rId1035"/>
+    <x:hyperlink ref="D350" r:id="rId1036"/>
+    <x:hyperlink ref="D351" r:id="rId1037"/>
+    <x:hyperlink ref="D352" r:id="rId1038"/>
+    <x:hyperlink ref="D353" r:id="rId1039"/>
+    <x:hyperlink ref="D354" r:id="rId1040"/>
+    <x:hyperlink ref="D355" r:id="rId1041"/>
+    <x:hyperlink ref="D356" r:id="rId1042"/>
+    <x:hyperlink ref="D357" r:id="rId1043"/>
+    <x:hyperlink ref="D358" r:id="rId1044"/>
+    <x:hyperlink ref="D359" r:id="rId1045"/>
+    <x:hyperlink ref="D360" r:id="rId1046"/>
+    <x:hyperlink ref="D361" r:id="rId1047"/>
+    <x:hyperlink ref="D362" r:id="rId1048"/>
+    <x:hyperlink ref="D363" r:id="rId1049"/>
+    <x:hyperlink ref="D364" r:id="rId1050"/>
+    <x:hyperlink ref="D365" r:id="rId1051"/>
+    <x:hyperlink ref="D366" r:id="rId1052"/>
+    <x:hyperlink ref="D367" r:id="rId1053"/>
+    <x:hyperlink ref="D368" r:id="rId1054"/>
+    <x:hyperlink ref="D369" r:id="rId1055"/>
+    <x:hyperlink ref="D370" r:id="rId1056"/>
+    <x:hyperlink ref="D371" r:id="rId1057"/>
+    <x:hyperlink ref="D372" r:id="rId1058"/>
+    <x:hyperlink ref="D373" r:id="rId1059"/>
+    <x:hyperlink ref="D374" r:id="rId1060"/>
+    <x:hyperlink ref="D375" r:id="rId1061"/>
+    <x:hyperlink ref="D376" r:id="rId1062"/>
+    <x:hyperlink ref="D377" r:id="rId1063"/>
+    <x:hyperlink ref="D378" r:id="rId1064"/>
+    <x:hyperlink ref="D379" r:id="rId1065"/>
+    <x:hyperlink ref="D380" r:id="rId1066"/>
+    <x:hyperlink ref="D381" r:id="rId1067"/>
+    <x:hyperlink ref="D382" r:id="rId1068"/>
+    <x:hyperlink ref="D383" r:id="rId1069"/>
+    <x:hyperlink ref="D384" r:id="rId1070"/>
+    <x:hyperlink ref="D385" r:id="rId1071"/>
+    <x:hyperlink ref="D386" r:id="rId1072"/>
+    <x:hyperlink ref="D387" r:id="rId1073"/>
+    <x:hyperlink ref="D388" r:id="rId1074"/>
+    <x:hyperlink ref="D389" r:id="rId1075"/>
+    <x:hyperlink ref="D390" r:id="rId1076"/>
+    <x:hyperlink ref="D391" r:id="rId1077"/>
+    <x:hyperlink ref="D392" r:id="rId1078"/>
+    <x:hyperlink ref="D393" r:id="rId1079"/>
+    <x:hyperlink ref="D394" r:id="rId1080"/>
+    <x:hyperlink ref="D395" r:id="rId1081"/>
+    <x:hyperlink ref="D396" r:id="rId1082"/>
+    <x:hyperlink ref="D397" r:id="rId1083"/>
+    <x:hyperlink ref="D398" r:id="rId1084"/>
+    <x:hyperlink ref="D399" r:id="rId1085"/>
+    <x:hyperlink ref="D400" r:id="rId1086"/>
+    <x:hyperlink ref="D401" r:id="rId1087"/>
+    <x:hyperlink ref="D402" r:id="rId1088"/>
+    <x:hyperlink ref="D403" r:id="rId1089"/>
+    <x:hyperlink ref="D404" r:id="rId1090"/>
+    <x:hyperlink ref="D405" r:id="rId1091"/>
+    <x:hyperlink ref="D406" r:id="rId1092"/>
+    <x:hyperlink ref="D407" r:id="rId1093"/>
+    <x:hyperlink ref="D408" r:id="rId1094"/>
+    <x:hyperlink ref="D409" r:id="rId1095"/>
+    <x:hyperlink ref="D410" r:id="rId1096"/>
+    <x:hyperlink ref="D411" r:id="rId1097"/>
+    <x:hyperlink ref="D412" r:id="rId1098"/>
+    <x:hyperlink ref="D413" r:id="rId1099"/>
+    <x:hyperlink ref="D414" r:id="rId1100"/>
+    <x:hyperlink ref="D415" r:id="rId1101"/>
+    <x:hyperlink ref="D416" r:id="rId1102"/>
+    <x:hyperlink ref="D417" r:id="rId1103"/>
+    <x:hyperlink ref="D418" r:id="rId1104"/>
+    <x:hyperlink ref="D419" r:id="rId1105"/>
+    <x:hyperlink ref="D420" r:id="rId1106"/>
+    <x:hyperlink ref="D421" r:id="rId1107"/>
+    <x:hyperlink ref="D422" r:id="rId1108"/>
+    <x:hyperlink ref="D423" r:id="rId1109"/>
+    <x:hyperlink ref="D424" r:id="rId1110"/>
+    <x:hyperlink ref="D425" r:id="rId1111"/>
+    <x:hyperlink ref="D426" r:id="rId1112"/>
+    <x:hyperlink ref="D427" r:id="rId1113"/>
+    <x:hyperlink ref="D428" r:id="rId1114"/>
+    <x:hyperlink ref="D429" r:id="rId1115"/>
+    <x:hyperlink ref="D430" r:id="rId1116"/>
+    <x:hyperlink ref="D431" r:id="rId1117"/>
+    <x:hyperlink ref="D432" r:id="rId1118"/>
+    <x:hyperlink ref="D433" r:id="rId1119"/>
+    <x:hyperlink ref="D434" r:id="rId1120"/>
+    <x:hyperlink ref="D435" r:id="rId1121"/>
+    <x:hyperlink ref="D436" r:id="rId1122"/>
+    <x:hyperlink ref="D437" r:id="rId1123"/>
+    <x:hyperlink ref="D438" r:id="rId1124"/>
+    <x:hyperlink ref="D439" r:id="rId1125"/>
+    <x:hyperlink ref="D440" r:id="rId1126"/>
+    <x:hyperlink ref="D441" r:id="rId1127"/>
+    <x:hyperlink ref="D442" r:id="rId1128"/>
+    <x:hyperlink ref="D443" r:id="rId1129"/>
+    <x:hyperlink ref="D444" r:id="rId1130"/>
+    <x:hyperlink ref="D445" r:id="rId1131"/>
+    <x:hyperlink ref="D446" r:id="rId1132"/>
+    <x:hyperlink ref="D447" r:id="rId1133"/>
+    <x:hyperlink ref="D448" r:id="rId1134"/>
+    <x:hyperlink ref="D449" r:id="rId1135"/>
+    <x:hyperlink ref="D450" r:id="rId1136"/>
+    <x:hyperlink ref="D451" r:id="rId1137"/>
+    <x:hyperlink ref="D452" r:id="rId1138"/>
+    <x:hyperlink ref="D453" r:id="rId1139"/>
+    <x:hyperlink ref="D454" r:id="rId1140"/>
+    <x:hyperlink ref="D455" r:id="rId1141"/>
+    <x:hyperlink ref="D456" r:id="rId1142"/>
+    <x:hyperlink ref="D457" r:id="rId1143"/>
+    <x:hyperlink ref="D458" r:id="rId1144"/>
+    <x:hyperlink ref="D459" r:id="rId1145"/>
+    <x:hyperlink ref="D460" r:id="rId1146"/>
+    <x:hyperlink ref="D461" r:id="rId1147"/>
+    <x:hyperlink ref="D462" r:id="rId1148"/>
+    <x:hyperlink ref="D463" r:id="rId1149"/>
+    <x:hyperlink ref="D464" r:id="rId1150"/>
+    <x:hyperlink ref="D465" r:id="rId1151"/>
+    <x:hyperlink ref="D466" r:id="rId1152"/>
+    <x:hyperlink ref="D467" r:id="rId1153"/>
+    <x:hyperlink ref="D468" r:id="rId1154"/>
+    <x:hyperlink ref="D469" r:id="rId1155"/>
+    <x:hyperlink ref="D470" r:id="rId1156"/>
+    <x:hyperlink ref="D471" r:id="rId1157"/>
+    <x:hyperlink ref="D472" r:id="rId1158"/>
+    <x:hyperlink ref="D473" r:id="rId1159"/>
+    <x:hyperlink ref="D474" r:id="rId1160"/>
+    <x:hyperlink ref="D475" r:id="rId1161"/>
+    <x:hyperlink ref="D476" r:id="rId1162"/>
+    <x:hyperlink ref="D477" r:id="rId1163"/>
+    <x:hyperlink ref="D478" r:id="rId1164"/>
+    <x:hyperlink ref="D479" r:id="rId1165"/>
+    <x:hyperlink ref="D480" r:id="rId1166"/>
+    <x:hyperlink ref="D481" r:id="rId1167"/>
+    <x:hyperlink ref="D482" r:id="rId1168"/>
+    <x:hyperlink ref="D483" r:id="rId1169"/>
+    <x:hyperlink ref="D484" r:id="rId1170"/>
+    <x:hyperlink ref="D485" r:id="rId1171"/>
+    <x:hyperlink ref="D486" r:id="rId1172"/>
+    <x:hyperlink ref="D487" r:id="rId1173"/>
+    <x:hyperlink ref="D488" r:id="rId1174"/>
+    <x:hyperlink ref="D489" r:id="rId1175"/>
+    <x:hyperlink ref="D490" r:id="rId1176"/>
+    <x:hyperlink ref="D491" r:id="rId1177"/>
+    <x:hyperlink ref="D492" r:id="rId1178"/>
+    <x:hyperlink ref="D493" r:id="rId1179"/>
+    <x:hyperlink ref="D494" r:id="rId1180"/>
+    <x:hyperlink ref="D495" r:id="rId1181"/>
+    <x:hyperlink ref="D496" r:id="rId1182"/>
+    <x:hyperlink ref="D497" r:id="rId1183"/>
+    <x:hyperlink ref="D498" r:id="rId1184"/>
+    <x:hyperlink ref="D499" r:id="rId1185"/>
+    <x:hyperlink ref="D500" r:id="rId1186"/>
+    <x:hyperlink ref="D501" r:id="rId1187"/>
+    <x:hyperlink ref="D502" r:id="rId1188"/>
+    <x:hyperlink ref="D503" r:id="rId1189"/>
+    <x:hyperlink ref="D504" r:id="rId1190"/>
+    <x:hyperlink ref="D505" r:id="rId1191"/>
+    <x:hyperlink ref="D506" r:id="rId1192"/>
+    <x:hyperlink ref="D507" r:id="rId1193"/>
+    <x:hyperlink ref="D508" r:id="rId1194"/>
+    <x:hyperlink ref="D509" r:id="rId1195"/>
+    <x:hyperlink ref="D510" r:id="rId1196"/>
+    <x:hyperlink ref="D511" r:id="rId1197"/>
+    <x:hyperlink ref="D512" r:id="rId1198"/>
+    <x:hyperlink ref="D513" r:id="rId1199"/>
+    <x:hyperlink ref="D514" r:id="rId1200"/>
+    <x:hyperlink ref="D515" r:id="rId1201"/>
+    <x:hyperlink ref="D516" r:id="rId1202"/>
+    <x:hyperlink ref="D517" r:id="rId1203"/>
+    <x:hyperlink ref="D518" r:id="rId1204"/>
+    <x:hyperlink ref="D519" r:id="rId1205"/>
+    <x:hyperlink ref="D520" r:id="rId1206"/>
+    <x:hyperlink ref="D521" r:id="rId1207"/>
+    <x:hyperlink ref="D522" r:id="rId1208"/>
+    <x:hyperlink ref="D523" r:id="rId1209"/>
+    <x:hyperlink ref="D524" r:id="rId1210"/>
+    <x:hyperlink ref="D525" r:id="rId1211"/>
+    <x:hyperlink ref="D526" r:id="rId1212"/>
+    <x:hyperlink ref="D527" r:id="rId1213"/>
+    <x:hyperlink ref="D528" r:id="rId1214"/>
+    <x:hyperlink ref="D529" r:id="rId1215"/>
+    <x:hyperlink ref="D530" r:id="rId1216"/>
+    <x:hyperlink ref="D531" r:id="rId1217"/>
+    <x:hyperlink ref="D532" r:id="rId1218"/>
+    <x:hyperlink ref="D533" r:id="rId1219"/>
+    <x:hyperlink ref="D534" r:id="rId1220"/>
+    <x:hyperlink ref="D535" r:id="rId1221"/>
+    <x:hyperlink ref="D536" r:id="rId1222"/>
+    <x:hyperlink ref="D537" r:id="rId1223"/>
+    <x:hyperlink ref="D538" r:id="rId1224"/>
+    <x:hyperlink ref="D539" r:id="rId1225"/>
+    <x:hyperlink ref="D540" r:id="rId1226"/>
+    <x:hyperlink ref="D541" r:id="rId1227"/>
+    <x:hyperlink ref="D542" r:id="rId1228"/>
+    <x:hyperlink ref="D543" r:id="rId1229"/>
+    <x:hyperlink ref="D544" r:id="rId1230"/>
+    <x:hyperlink ref="D545" r:id="rId1231"/>
+    <x:hyperlink ref="D546" r:id="rId1232"/>
+    <x:hyperlink ref="D547" r:id="rId1233"/>
+    <x:hyperlink ref="D548" r:id="rId1234"/>
+    <x:hyperlink ref="D549" r:id="rId1235"/>
+    <x:hyperlink ref="D550" r:id="rId1236"/>
+    <x:hyperlink ref="D551" r:id="rId1237"/>
+    <x:hyperlink ref="D552" r:id="rId1238"/>
+    <x:hyperlink ref="D553" r:id="rId1239"/>
+    <x:hyperlink ref="D554" r:id="rId1240"/>
+    <x:hyperlink ref="D555" r:id="rId1241"/>
+    <x:hyperlink ref="D556" r:id="rId1242"/>
+    <x:hyperlink ref="D557" r:id="rId1243"/>
+    <x:hyperlink ref="D558" r:id="rId1244"/>
+    <x:hyperlink ref="D559" r:id="rId1245"/>
+    <x:hyperlink ref="D560" r:id="rId1246"/>
+    <x:hyperlink ref="D561" r:id="rId1247"/>
+    <x:hyperlink ref="D562" r:id="rId1248"/>
+    <x:hyperlink ref="D563" r:id="rId1249"/>
+    <x:hyperlink ref="D564" r:id="rId1250"/>
+    <x:hyperlink ref="D565" r:id="rId1251"/>
+    <x:hyperlink ref="D566" r:id="rId1252"/>
+    <x:hyperlink ref="D567" r:id="rId1253"/>
+    <x:hyperlink ref="D568" r:id="rId1254"/>
+    <x:hyperlink ref="D569" r:id="rId1255"/>
+    <x:hyperlink ref="D570" r:id="rId1256"/>
+    <x:hyperlink ref="D571" r:id="rId1257"/>
+    <x:hyperlink ref="D572" r:id="rId1258"/>
+    <x:hyperlink ref="D573" r:id="rId1259"/>
+    <x:hyperlink ref="D574" r:id="rId1260"/>
+    <x:hyperlink ref="D575" r:id="rId1261"/>
+    <x:hyperlink ref="D576" r:id="rId1262"/>
+    <x:hyperlink ref="D577" r:id="rId1263"/>
+    <x:hyperlink ref="D578" r:id="rId1264"/>
+    <x:hyperlink ref="D579" r:id="rId1265"/>
+    <x:hyperlink ref="D580" r:id="rId1266"/>
+    <x:hyperlink ref="D581" r:id="rId1267"/>
+    <x:hyperlink ref="D582" r:id="rId1268"/>
+    <x:hyperlink ref="D583" r:id="rId1269"/>
+    <x:hyperlink ref="D584" r:id="rId1270"/>
+    <x:hyperlink ref="D585" r:id="rId1271"/>
+    <x:hyperlink ref="D586" r:id="rId1272"/>
+    <x:hyperlink ref="D587" r:id="rId1273"/>
+    <x:hyperlink ref="D588" r:id="rId1274"/>
+    <x:hyperlink ref="D589" r:id="rId1275"/>
+    <x:hyperlink ref="D590" r:id="rId1276"/>
+    <x:hyperlink ref="D591" r:id="rId1277"/>
+    <x:hyperlink ref="D592" r:id="rId1278"/>
+    <x:hyperlink ref="D593" r:id="rId1279"/>
+    <x:hyperlink ref="D594" r:id="rId1280"/>
+    <x:hyperlink ref="D595" r:id="rId1281"/>
+    <x:hyperlink ref="D596" r:id="rId1282"/>
+    <x:hyperlink ref="D597" r:id="rId1283"/>
+    <x:hyperlink ref="D598" r:id="rId1284"/>
+    <x:hyperlink ref="D599" r:id="rId1285"/>
+    <x:hyperlink ref="D600" r:id="rId1286"/>
+    <x:hyperlink ref="D601" r:id="rId1287"/>
+    <x:hyperlink ref="D602" r:id="rId1288"/>
+    <x:hyperlink ref="D603" r:id="rId1289"/>
+    <x:hyperlink ref="D604" r:id="rId1290"/>
+    <x:hyperlink ref="D605" r:id="rId1291"/>
+    <x:hyperlink ref="D606" r:id="rId1292"/>
+    <x:hyperlink ref="D607" r:id="rId1293"/>
+    <x:hyperlink ref="D608" r:id="rId1294"/>
+    <x:hyperlink ref="D609" r:id="rId1295"/>
+    <x:hyperlink ref="D610" r:id="rId1296"/>
+    <x:hyperlink ref="D611" r:id="rId1297"/>
+    <x:hyperlink ref="D612" r:id="rId1298"/>
+    <x:hyperlink ref="D613" r:id="rId1299"/>
+    <x:hyperlink ref="D614" r:id="rId1300"/>
+    <x:hyperlink ref="D615" r:id="rId1301"/>
+    <x:hyperlink ref="D616" r:id="rId1302"/>
+    <x:hyperlink ref="D617" r:id="rId1303"/>
+    <x:hyperlink ref="D618" r:id="rId1304"/>
+    <x:hyperlink ref="D619" r:id="rId1305"/>
+    <x:hyperlink ref="D620" r:id="rId1306"/>
+    <x:hyperlink ref="D621" r:id="rId1307"/>
+    <x:hyperlink ref="D622" r:id="rId1308"/>
+    <x:hyperlink ref="D623" r:id="rId1309"/>
+    <x:hyperlink ref="D624" r:id="rId1310"/>
+    <x:hyperlink ref="D625" r:id="rId1311"/>
+    <x:hyperlink ref="D626" r:id="rId1312"/>
+    <x:hyperlink ref="D627" r:id="rId1313"/>
+    <x:hyperlink ref="D628" r:id="rId1314"/>
+    <x:hyperlink ref="D629" r:id="rId1315"/>
+    <x:hyperlink ref="D630" r:id="rId1316"/>
+    <x:hyperlink ref="D631" r:id="rId1317"/>
+    <x:hyperlink ref="D632" r:id="rId1318"/>
+    <x:hyperlink ref="D633" r:id="rId1319"/>
+    <x:hyperlink ref="D634" r:id="rId1320"/>
+    <x:hyperlink ref="D635" r:id="rId1321"/>
+    <x:hyperlink ref="D636" r:id="rId1322"/>
+    <x:hyperlink ref="D637" r:id="rId1323"/>
+    <x:hyperlink ref="D638" r:id="rId1324"/>
+    <x:hyperlink ref="D639" r:id="rId1325"/>
+    <x:hyperlink ref="D640" r:id="rId1326"/>
+    <x:hyperlink ref="D641" r:id="rId1327"/>
+    <x:hyperlink ref="D642" r:id="rId1328"/>
+    <x:hyperlink ref="D643" r:id="rId1329"/>
+    <x:hyperlink ref="D644" r:id="rId1330"/>
+    <x:hyperlink ref="D645" r:id="rId1331"/>
+    <x:hyperlink ref="D646" r:id="rId1332"/>
+    <x:hyperlink ref="D647" r:id="rId1333"/>
+    <x:hyperlink ref="D648" r:id="rId1334"/>
+    <x:hyperlink ref="D649" r:id="rId1335"/>
+    <x:hyperlink ref="D650" r:id="rId1336"/>
+    <x:hyperlink ref="D651" r:id="rId1337"/>
+    <x:hyperlink ref="D652" r:id="rId1338"/>
+    <x:hyperlink ref="D653" r:id="rId1339"/>
+    <x:hyperlink ref="D654" r:id="rId1340"/>
+    <x:hyperlink ref="D655" r:id="rId1341"/>
+    <x:hyperlink ref="D656" r:id="rId1342"/>
+    <x:hyperlink ref="D657" r:id="rId1343"/>
+    <x:hyperlink ref="D658" r:id="rId1344"/>
+    <x:hyperlink ref="D659" r:id="rId1345"/>
+    <x:hyperlink ref="D660" r:id="rId1346"/>
+    <x:hyperlink ref="D661" r:id="rId1347"/>
+    <x:hyperlink ref="D662" r:id="rId1348"/>
+    <x:hyperlink ref="D663" r:id="rId1349"/>
+    <x:hyperlink ref="D664" r:id="rId1350"/>
+    <x:hyperlink ref="D665" r:id="rId1351"/>
+    <x:hyperlink ref="D666" r:id="rId1352"/>
+    <x:hyperlink ref="D667" r:id="rId1353"/>
+    <x:hyperlink ref="D668" r:id="rId1354"/>
+    <x:hyperlink ref="D669" r:id="rId1355"/>
+    <x:hyperlink ref="D670" r:id="rId1356"/>
+    <x:hyperlink ref="D671" r:id="rId1357"/>
+    <x:hyperlink ref="D672" r:id="rId1358"/>
+    <x:hyperlink ref="D673" r:id="rId1359"/>
+    <x:hyperlink ref="D674" r:id="rId1360"/>
+    <x:hyperlink ref="D675" r:id="rId1361"/>
+    <x:hyperlink ref="D676" r:id="rId1362"/>
+    <x:hyperlink ref="D677" r:id="rId1363"/>
+    <x:hyperlink ref="D678" r:id="rId1364"/>
+    <x:hyperlink ref="D679" r:id="rId1365"/>
+    <x:hyperlink ref="D680" r:id="rId1366"/>
+    <x:hyperlink ref="D681" r:id="rId1367"/>
+    <x:hyperlink ref="D682" r:id="rId1368"/>
+    <x:hyperlink ref="D683" r:id="rId1369"/>
+    <x:hyperlink ref="D684" r:id="rId1370"/>
+    <x:hyperlink ref="D685" r:id="rId1371"/>
+    <x:hyperlink ref="D686" r:id="rId1372"/>
+    <x:hyperlink ref="D687" r:id="rId1373"/>
+    <x:hyperlink ref="D688" r:id="rId1374"/>
+    <x:hyperlink ref="D689" r:id="rId1375"/>
+    <x:hyperlink ref="D690" r:id="rId1376"/>
   </x:hyperlinks>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
   <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
   <x:headerFooter/>
   <x:tableParts count="1">
-    <x:tablePart r:id="rId673"/>
+    <x:tablePart r:id="rId691"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
chore: actualiza dashboard 2026-06-09T07:41Z
</commit_message>
<xml_diff>
--- a/INFORME EXCESOS DE VELOCIDAD.xlsx
+++ b/INFORME EXCESOS DE VELOCIDAD.xlsx
@@ -240,8 +240,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="SpeedingByUnitsFleetsDetailTable_1" displayName="SpeedingByUnitsFleetsDetailTable_1" ref="A5:O322" headerRowCount="1" totalsRowShown="0">
-  <autoFilter ref="A5:O322"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="SpeedingByUnitsFleetsDetailTable_1" displayName="SpeedingByUnitsFleetsDetailTable_1" ref="A5:O324" headerRowCount="1" totalsRowShown="0">
+  <autoFilter ref="A5:O324"/>
   <tableColumns count="15">
     <tableColumn id="1" name="Alias"/>
     <tableColumn id="2" name="Conductor"/>
@@ -264,8 +264,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SpeedingByUnitsFleetsDataTable_1" displayName="SpeedingByUnitsFleetsDataTable_1" ref="A5:H640" headerRowCount="1" totalsRowShown="0">
-  <autoFilter ref="A5:H640"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SpeedingByUnitsFleetsDataTable_1" displayName="SpeedingByUnitsFleetsDataTable_1" ref="A5:H644" headerRowCount="1" totalsRowShown="0">
+  <autoFilter ref="A5:H644"/>
   <tableColumns count="8">
     <tableColumn id="1" name="Alias"/>
     <tableColumn id="2" name="Secuencial" dataDxfId="0"/>
@@ -682,16 +682,16 @@
         </is>
       </c>
       <c r="B7" s="12" t="n">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="C7" s="13" t="n">
-        <v>0.01596064814814815</v>
+        <v>0.01616898148148148</v>
       </c>
       <c r="D7" s="13" t="n">
-        <v>8.916666666666666e-05</v>
+        <v>8.93287037037037e-05</v>
       </c>
       <c r="E7" s="12" t="n">
-        <v>10.8</v>
+        <v>10.9</v>
       </c>
       <c r="F7" s="12" t="n">
         <v>45.6</v>
@@ -727,7 +727,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O322"/>
+  <dimension ref="A1:O324"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30.710625" customWidth="1" style="7" min="1" max="1"/>
@@ -21060,6 +21060,134 @@
         <v>0</v>
       </c>
       <c r="O322" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>TOYOTA HILUX VTGL-56</t>
+        </is>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>NICOLAS VARGAS</t>
+        </is>
+      </c>
+      <c r="C323" t="n">
+        <v>493</v>
+      </c>
+      <c r="D323" t="inlineStr">
+        <is>
+          <t>2026/06/08 22:33:18</t>
+        </is>
+      </c>
+      <c r="E323" t="inlineStr">
+        <is>
+          <t>-33.676148,-70.750395</t>
+        </is>
+      </c>
+      <c r="F323" t="inlineStr">
+        <is>
+          <t>El Rodeo, San Bernardo, Maipo, Región Metropolitana de Santiago. VMaxLiv:50, VMaxPes:50</t>
+        </is>
+      </c>
+      <c r="G323" t="inlineStr">
+        <is>
+          <t>2026/06/08 22:33:24</t>
+        </is>
+      </c>
+      <c r="H323" t="inlineStr">
+        <is>
+          <t>-33.676167,-70.751016</t>
+        </is>
+      </c>
+      <c r="I323" t="inlineStr">
+        <is>
+          <t>El Rodeo, San Bernardo, Maipo, Región Metropolitana de Santiago. VMaxLiv:50, VMaxPes:50</t>
+        </is>
+      </c>
+      <c r="J323" s="14" t="n">
+        <v>6.944444444444444e-05</v>
+      </c>
+      <c r="K323" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L323" t="n">
+        <v>36.6</v>
+      </c>
+      <c r="M323" t="n">
+        <v>34.5</v>
+      </c>
+      <c r="N323" t="n">
+        <v>0</v>
+      </c>
+      <c r="O323" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>TOYOTA HILUX VTGL-56</t>
+        </is>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>NICOLAS VARGAS</t>
+        </is>
+      </c>
+      <c r="C324" t="n">
+        <v>499</v>
+      </c>
+      <c r="D324" t="inlineStr">
+        <is>
+          <t>2026/06/08 23:04:22</t>
+        </is>
+      </c>
+      <c r="E324" t="inlineStr">
+        <is>
+          <t>-33.699518,-70.802199</t>
+        </is>
+      </c>
+      <c r="F324" t="inlineStr">
+        <is>
+          <t>El Rodeo, San Bernardo, Maipo, Región Metropolitana de Santiago. VMaxLiv:50, VMaxPes:50</t>
+        </is>
+      </c>
+      <c r="G324" t="inlineStr">
+        <is>
+          <t>2026/06/08 23:04:34</t>
+        </is>
+      </c>
+      <c r="H324" t="inlineStr">
+        <is>
+          <t>-33.700008,-70.80229</t>
+        </is>
+      </c>
+      <c r="I324" t="inlineStr">
+        <is>
+          <t>Los Nogales, Talagante, Talagante, Región Metropolitana de Santiago. VMaxLiv:50, VMaxPes:50</t>
+        </is>
+      </c>
+      <c r="J324" s="14" t="n">
+        <v>0.0001388888888888889</v>
+      </c>
+      <c r="K324" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="L324" t="n">
+        <v>22.1</v>
+      </c>
+      <c r="M324" t="n">
+        <v>20.3</v>
+      </c>
+      <c r="N324" t="n">
+        <v>0</v>
+      </c>
+      <c r="O324" t="n">
         <v>0</v>
       </c>
     </row>
@@ -21084,7 +21212,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H640"/>
+  <dimension ref="A1:H644"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30.710625" customWidth="1" style="7" min="1" max="1"/>
@@ -42744,6 +42872,142 @@
       </c>
       <c r="H640" s="12" t="n">
         <v>504.9</v>
+      </c>
+    </row>
+    <row r="641">
+      <c r="A641" s="7" t="inlineStr">
+        <is>
+          <t>TOYOTA HILUX VTGL-56</t>
+        </is>
+      </c>
+      <c r="B641" s="12" t="n">
+        <v>493</v>
+      </c>
+      <c r="C641" s="12" t="inlineStr">
+        <is>
+          <t>2026/06/08 22:33:18</t>
+        </is>
+      </c>
+      <c r="D641" s="15" t="inlineStr">
+        <is>
+          <t>-33.676148,-70.750395</t>
+        </is>
+      </c>
+      <c r="E641" s="12" t="inlineStr">
+        <is>
+          <t>s/n, Talagante, Talagante, Región Metropolitana de Santiago. VMaxLiv:50, VMaxPes:50</t>
+        </is>
+      </c>
+      <c r="F641" s="12" t="n">
+        <v>32.3</v>
+      </c>
+      <c r="G641" s="12" t="n">
+        <v>5610.5</v>
+      </c>
+      <c r="H641" s="12" t="n">
+        <v>505.3</v>
+      </c>
+    </row>
+    <row r="642">
+      <c r="A642" s="7" t="inlineStr">
+        <is>
+          <t>TOYOTA HILUX VTGL-56</t>
+        </is>
+      </c>
+      <c r="B642" s="12" t="n">
+        <v>493</v>
+      </c>
+      <c r="C642" s="12" t="inlineStr">
+        <is>
+          <t>2026/06/08 22:33:24</t>
+        </is>
+      </c>
+      <c r="D642" s="15" t="inlineStr">
+        <is>
+          <t>-33.676167,-70.751016</t>
+        </is>
+      </c>
+      <c r="E642" s="12" t="inlineStr">
+        <is>
+          <t>s/n, Talagante, Talagante, Región Metropolitana de Santiago. VMaxLiv:50, VMaxPes:50</t>
+        </is>
+      </c>
+      <c r="F642" s="12" t="n">
+        <v>36.6</v>
+      </c>
+      <c r="G642" s="12" t="n">
+        <v>5610.5</v>
+      </c>
+      <c r="H642" s="12" t="n">
+        <v>504.7</v>
+      </c>
+    </row>
+    <row r="643">
+      <c r="A643" s="7" t="inlineStr">
+        <is>
+          <t>TOYOTA HILUX VTGL-56</t>
+        </is>
+      </c>
+      <c r="B643" s="12" t="n">
+        <v>499</v>
+      </c>
+      <c r="C643" s="12" t="inlineStr">
+        <is>
+          <t>2026/06/08 23:04:22</t>
+        </is>
+      </c>
+      <c r="D643" s="15" t="inlineStr">
+        <is>
+          <t>-33.699518,-70.802199</t>
+        </is>
+      </c>
+      <c r="E643" s="12" t="inlineStr">
+        <is>
+          <t>s/n, Talagante, Talagante, Región Metropolitana de Santiago. VMaxLiv:50, VMaxPes:50</t>
+        </is>
+      </c>
+      <c r="F643" s="12" t="n">
+        <v>22.1</v>
+      </c>
+      <c r="G643" s="12" t="n">
+        <v>5619.9</v>
+      </c>
+      <c r="H643" s="12" t="n">
+        <v>543.4</v>
+      </c>
+    </row>
+    <row r="644">
+      <c r="A644" s="7" t="inlineStr">
+        <is>
+          <t>TOYOTA HILUX VTGL-56</t>
+        </is>
+      </c>
+      <c r="B644" s="12" t="n">
+        <v>499</v>
+      </c>
+      <c r="C644" s="12" t="inlineStr">
+        <is>
+          <t>2026/06/08 23:04:34</t>
+        </is>
+      </c>
+      <c r="D644" s="15" t="inlineStr">
+        <is>
+          <t>-33.700008,-70.80229</t>
+        </is>
+      </c>
+      <c r="E644" s="12" t="inlineStr">
+        <is>
+          <t>s/n, Talagante, Talagante, Región Metropolitana de Santiago. VMaxLiv:50, VMaxPes:50</t>
+        </is>
+      </c>
+      <c r="F644" s="12" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="G644" s="12" t="n">
+        <v>5620</v>
+      </c>
+      <c r="H644" s="12" t="n">
+        <v>548.3</v>
       </c>
     </row>
   </sheetData>
@@ -43388,12 +43652,16 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D638" r:id="rId633"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D639" r:id="rId634"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D640" r:id="rId635"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D641" r:id="rId636"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D642" r:id="rId637"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D643" r:id="rId638"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D644" r:id="rId639"/>
   </hyperlinks>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
   <pageSetup orientation="default" paperSize="1" scale="100" pageOrder="downThenOver" blackAndWhite="0" draft="0" errors="displayed"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId636"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId640"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore: actualiza dashboard 2026-06-15T09:54Z
</commit_message>
<xml_diff>
--- a/INFORME EXCESOS DE VELOCIDAD.xlsx
+++ b/INFORME EXCESOS DE VELOCIDAD.xlsx
@@ -585,8 +585,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="SpeedingDetailTable_1" displayName="SpeedingDetailTable_1" ref="A5:O383" headerRowCount="1">
-  <autoFilter ref="A5:O383"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="SpeedingDetailTable_1" displayName="SpeedingDetailTable_1" ref="A5:O384" headerRowCount="1">
+  <autoFilter ref="A5:O384"/>
   <tableColumns count="15">
     <tableColumn id="1" name="Alias"/>
     <tableColumn id="2" name="Conductor"/>
@@ -609,8 +609,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SpeedingDataTable_1" displayName="SpeedingDataTable_1" ref="A5:H761" headerRowCount="1">
-  <autoFilter ref="A5:H761"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SpeedingDataTable_1" displayName="SpeedingDataTable_1" ref="A5:H763" headerRowCount="1">
+  <autoFilter ref="A5:H763"/>
   <tableColumns count="8">
     <tableColumn id="1" name="Alias"/>
     <tableColumn id="2" name="Secuencial"/>
@@ -1059,13 +1059,13 @@
         </is>
       </c>
       <c r="C7" s="3" t="n">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="D7" s="5" t="n">
-        <v>0.01892361111111111</v>
+        <v>0.01899305555555555</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>9.231481481481482e-05</v>
+        <v>9.219907407407408e-05</v>
       </c>
       <c r="F7" s="3" t="n">
         <v>12.4</v>
@@ -1106,7 +1106,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O383"/>
+  <dimension ref="A1:O384"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -25413,6 +25413,71 @@
         <v>0</v>
       </c>
     </row>
+    <row r="384">
+      <c r="A384" t="inlineStr">
+        <is>
+          <t>TOYOTA HILUX VTGL-56</t>
+        </is>
+      </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>NICOLAS VARGAS</t>
+        </is>
+      </c>
+      <c r="C384" t="n">
+        <v>437</v>
+      </c>
+      <c r="D384" t="inlineStr">
+        <is>
+          <t>2026/06/14 23:30:09</t>
+        </is>
+      </c>
+      <c r="E384" t="inlineStr">
+        <is>
+          <t>-33.69946,-70.80213</t>
+        </is>
+      </c>
+      <c r="F384" t="inlineStr">
+        <is>
+          <t>s/n, Talagante, Talagante, Región Metropolitana de Santiago. VMaxLiv:50, VMaxPes:50</t>
+        </is>
+      </c>
+      <c r="G384" t="inlineStr">
+        <is>
+          <t>2026/06/14 23:30:15</t>
+        </is>
+      </c>
+      <c r="H384" t="inlineStr">
+        <is>
+          <t>-33.699353,-70.801834</t>
+        </is>
+      </c>
+      <c r="I384" t="inlineStr">
+        <is>
+          <t>s/n, Talagante, Talagante, Región Metropolitana de Santiago. VMaxLiv:50, VMaxPes:50</t>
+        </is>
+      </c>
+      <c r="J384" s="7" t="n">
+        <v>6.944444444444444e-05</v>
+      </c>
+      <c r="K384" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L384" t="n">
+        <v>25.1</v>
+      </c>
+      <c r="M384" t="n">
+        <v>18.6</v>
+      </c>
+      <c r="N384" t="n">
+        <v>0</v>
+      </c>
+      <c r="O384" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:O1"/>
@@ -25431,7 +25496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H761"/>
+  <dimension ref="A1:H763"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -51212,6 +51277,74 @@
       </c>
       <c r="H761" s="3" t="n">
         <v>544.6</v>
+      </c>
+    </row>
+    <row r="762">
+      <c r="A762" t="inlineStr">
+        <is>
+          <t>TOYOTA HILUX VTGL-56</t>
+        </is>
+      </c>
+      <c r="B762" s="3" t="n">
+        <v>437</v>
+      </c>
+      <c r="C762" s="3" t="inlineStr">
+        <is>
+          <t>2026/06/14 23:30:09</t>
+        </is>
+      </c>
+      <c r="D762" s="6" t="inlineStr">
+        <is>
+          <t>-33.69946,-70.80213</t>
+        </is>
+      </c>
+      <c r="E762" s="3" t="inlineStr">
+        <is>
+          <t>El Rodeo, San Bernardo, Maipo, Región Metropolitana de Santiago. VMaxLiv:50, VMaxPes:50</t>
+        </is>
+      </c>
+      <c r="F762" s="3" t="n">
+        <v>25.1</v>
+      </c>
+      <c r="G762" s="3" t="n">
+        <v>5881.4</v>
+      </c>
+      <c r="H762" s="3" t="n">
+        <v>547.9</v>
+      </c>
+    </row>
+    <row r="763">
+      <c r="A763" t="inlineStr">
+        <is>
+          <t>TOYOTA HILUX VTGL-56</t>
+        </is>
+      </c>
+      <c r="B763" s="3" t="n">
+        <v>437</v>
+      </c>
+      <c r="C763" s="3" t="inlineStr">
+        <is>
+          <t>2026/06/14 23:30:15</t>
+        </is>
+      </c>
+      <c r="D763" s="6" t="inlineStr">
+        <is>
+          <t>-33.699353,-70.801834</t>
+        </is>
+      </c>
+      <c r="E763" s="3" t="inlineStr">
+        <is>
+          <t>s/n, San Bernardo, Maipo, Región Metropolitana de Santiago. VMaxLiv:50, VMaxPes:50</t>
+        </is>
+      </c>
+      <c r="F763" s="3" t="n">
+        <v>12.1</v>
+      </c>
+      <c r="G763" s="3" t="n">
+        <v>5881.4</v>
+      </c>
+      <c r="H763" s="3" t="n">
+        <v>545.8</v>
       </c>
     </row>
   </sheetData>
@@ -51976,10 +52109,12 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D759" r:id="rId754"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D760" r:id="rId755"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D761" r:id="rId756"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D762" r:id="rId757"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D763" r:id="rId758"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId757"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId759"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>